<commit_message>
Updated CSCRF CIS crosswalk
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F70FB2F-1556-BA42-AC0E-0A7384CABBD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10FB854-A913-F844-AA9F-7299E079AE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Crosswalk" sheetId="2" r:id="rId1"/>
@@ -446,7 +446,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -512,28 +512,23 @@
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -868,7 +863,7 @@
       <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="27" t="s">
         <v>63</v>
       </c>
       <c r="B2" s="25"/>
@@ -882,20 +877,20 @@
       <c r="J2" s="25"/>
       <c r="K2" s="25"/>
     </row>
-    <row r="3" spans="1:11" s="26" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="33" t="s">
+    <row r="3" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="31"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
     </row>
     <row r="4" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
@@ -933,19 +928,19 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="25"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
     </row>
     <row r="6" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -1143,9 +1138,9 @@
     <col min="9" max="9" width="0.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="28" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="29" t="s">
         <v>61</v>
       </c>
       <c r="B2" s="25"/>
@@ -1157,8 +1152,8 @@
       <c r="H2" s="25"/>
       <c r="I2" s="25"/>
     </row>
-    <row r="3" spans="1:9" s="30" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+    <row r="3" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="28" t="s">
         <v>62</v>
       </c>
       <c r="B3" s="25"/>
@@ -1170,29 +1165,29 @@
       <c r="H3" s="25"/>
       <c r="I3" s="25"/>
     </row>
-    <row r="4" spans="1:9" s="26" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="G4" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="23" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Detect Function /w Validation
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771B348D-498A-1343-A869-5EAFC0D694CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D535239F-C71B-484F-A9F0-621624D99139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="119">
   <si>
     <t>CSCRF
 Function</t>
@@ -374,12 +374,71 @@
   <si>
     <t>IDENTIFY  FUNCTION</t>
   </si>
+  <si>
+    <t>DETECT</t>
+  </si>
+  <si>
+    <t>DE.CM</t>
+  </si>
+  <si>
+    <t>Continuous Monitoring &amp; Log Management</t>
+  </si>
+  <si>
+    <t>CIS 8 + CIS 13</t>
+  </si>
+  <si>
+    <t>Audit Log Management + Network Monitoring &amp; Defense</t>
+  </si>
+  <si>
+    <t>8.1 Establish Audit Log Mgmt
+8.2 Collect Audit Logs
+8.11 Centralize Log Aggregation
+13.1 Centralise Security Event Alerting</t>
+  </si>
+  <si>
+    <t>• Log management policy with retention schedule
+• SIEM/log aggregator configuration evidence
+• Log integrity verification records
+• Sample log review reports</t>
+  </si>
+  <si>
+    <t>CSCRF mandates log retention: 180 days online, 7 years offline/archive. Document log archival policy and periodic restoration test evidence aligned with CIS 8.3 (retention policy).</t>
+  </si>
+  <si>
+    <t>DE.AE</t>
+  </si>
+  <si>
+    <t>Adverse Event Analysis — SIEM &amp; UEBA</t>
+  </si>
+  <si>
+    <t>CIS 13 + CIS 10</t>
+  </si>
+  <si>
+    <t>Network Monitoring &amp; Defense + Malware Defenses</t>
+  </si>
+  <si>
+    <t>13.3 Deploy Network Intrusion Detection
+13.6 Collect Network Traffic Flow Logs
+10.1 Deploy Anti-Malware Software</t>
+  </si>
+  <si>
+    <t>• SIEM use case catalogue (mapped to MITRE ATT&amp;CK)
+• UEBA alert configuration and baseline documentation
+• Monthly threat detection summary reports
+• Incident triage records</t>
+  </si>
+  <si>
+    <t>CSCRF mandates SIEM for Qualified REs and MIIs. Build SIEM use cases around SEBI-relevant threats: insider trading, market manipulation, algo trading abuse. Document threat detection coverage matrix.</t>
+  </si>
+  <si>
+    <t>DETECT  FUNCTION</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="35" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -588,8 +647,22 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF3D1C5C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF3D1C5C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -641,6 +714,11 @@
         <fgColor rgb="FFFDE8E8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDE6F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -669,7 +747,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -812,6 +890,12 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1555,23 +1639,105 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="17" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="18" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="20" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="21" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="50" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
+    </row>
+    <row r="17" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="F17" s="35" t="s">
+        <v>108</v>
+      </c>
+      <c r="G17" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="I17" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="J17" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="K17" s="36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" s="40" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="E18" s="41" t="s">
+        <v>114</v>
+      </c>
+      <c r="F18" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="G18" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="I18" s="45" t="s">
+        <v>116</v>
+      </c>
+      <c r="J18" s="46" t="s">
+        <v>117</v>
+      </c>
+      <c r="K18" s="36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="26" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="34" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="35" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1581,11 +1747,12 @@
     <row r="39" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="40" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A16:K16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Detect Function: SOC & Threat Intelligence requirements (DE.SOC & DE.TI)
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D535239F-C71B-484F-A9F0-621624D99139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208D7A1A-A09F-EE47-BC25-0EEEA1BEABE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="129">
   <si>
     <t>CSCRF
 Function</t>
@@ -432,6 +432,38 @@
   </si>
   <si>
     <t>DETECT  FUNCTION</t>
+  </si>
+  <si>
+    <t>DE.SOC</t>
+  </si>
+  <si>
+    <t>Security Operations Centre (SOC) Operations</t>
+  </si>
+  <si>
+    <t>CIS 13 + CIS 17</t>
+  </si>
+  <si>
+    <t>Network Monitoring + Incident Response</t>
+  </si>
+  <si>
+    <t>13.1 Security Event Alerting
+17.4 Establish Communication &amp; Info Sharing</t>
+  </si>
+  <si>
+    <t>DE.TI</t>
+  </si>
+  <si>
+    <t>Threat Intelligence — SEBI CTIS Integration</t>
+  </si>
+  <si>
+    <t>CIS 13</t>
+  </si>
+  <si>
+    <t>Network Monitoring &amp; Defense</t>
+  </si>
+  <si>
+    <t>13.1 Centralise Security Event Alerting
+13.5 Manage Access Control for Remote Assets</t>
   </si>
 </sst>
 </file>
@@ -1724,8 +1756,52 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="34" t="s">
+        <v>121</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="F19" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="G19" s="47" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" s="42" t="s">
+        <v>126</v>
+      </c>
+      <c r="E20" s="41" t="s">
+        <v>127</v>
+      </c>
+      <c r="F20" s="43" t="s">
+        <v>128</v>
+      </c>
+      <c r="G20" s="47" t="s">
+        <v>86</v>
+      </c>
+    </row>
     <row r="21" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="23" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Added Assurance/Validation for Detect Function: SOC & Threat Intelligence requirements (DE.SOC & DE.TI)
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208D7A1A-A09F-EE47-BC25-0EEEA1BEABE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D31BBF3-D91E-7741-8F5A-12F702E33789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="133">
   <si>
     <t>CSCRF
 Function</t>
@@ -464,6 +464,24 @@
   <si>
     <t>13.1 Centralise Security Event Alerting
 13.5 Manage Access Control for Remote Assets</t>
+  </si>
+  <si>
+    <t>• SOC service agreement / SLA (if outsourced)
+• SOC staffing model documentation
+• Escalation matrix and playbooks
+• Monthly SOC operations report</t>
+  </si>
+  <si>
+    <t>SEBI mandates SOC operations for ALL REs: In-house (MIIs/Qualified), Hybrid (Mid-size), or SEBI-approved SOCaaS (Small REs). No equivalent CIS prescriptive requirement — CIS supports but doesn't mandate SOC model.</t>
+  </si>
+  <si>
+    <t>• SEBI CTIS platform registration confirmation
+• CTIS feed integration configuration in SIEM
+• Threat intelligence consumption process documentation
+• IOC/TTP tracking log</t>
+  </si>
+  <si>
+    <t>CSCRF requires integration with SEBI's Cyber Threat Intelligence Sharing (CTIS) platform. Register on CTIS platform and configure SIEM to ingest CTIS IOC feeds. No direct CIS equivalent — this is India-specific operationally.</t>
   </si>
 </sst>
 </file>
@@ -1778,6 +1796,18 @@
       <c r="G19" s="47" t="s">
         <v>86</v>
       </c>
+      <c r="H19" s="48" t="s">
+        <v>87</v>
+      </c>
+      <c r="I19" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="J19" s="39" t="s">
+        <v>130</v>
+      </c>
+      <c r="K19" s="47" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="51" t="s">
@@ -1800,6 +1830,18 @@
       </c>
       <c r="G20" s="47" t="s">
         <v>86</v>
+      </c>
+      <c r="H20" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="I20" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="J20" s="46" t="s">
+        <v>132</v>
+      </c>
+      <c r="K20" s="36" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Added 2 more functions, Added Implementation Roadmap, Gap analysis & Legend
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -8,20 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D31BBF3-D91E-7741-8F5A-12F702E33789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33965CD0-53FF-7941-9B2F-435832F3C15D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Crosswalk" sheetId="2" r:id="rId1"/>
-    <sheet name="Implementation Roadmap" sheetId="4" r:id="rId2"/>
+    <sheet name="Cover" sheetId="8" r:id="rId1"/>
+    <sheet name="Crosswalk" sheetId="2" r:id="rId2"/>
+    <sheet name="Implementation Roadmap" sheetId="4" r:id="rId3"/>
+    <sheet name="Gap Analysis" sheetId="7" r:id="rId4"/>
+    <sheet name="Legend" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="427">
   <si>
     <t>CSCRF
 Function</t>
@@ -109,10 +112,6 @@
   </si>
   <si>
     <t>Continuous Vulnerability Management</t>
-  </si>
-  <si>
-    <t>7.1 Establish Vulnerability Mgmt Process
-7.7 Remediate Detected Vulnerabilities</t>
   </si>
   <si>
     <t>IG2</t>
@@ -234,15 +233,6 @@
     <t>Immediate (already regulated)</t>
   </si>
   <si>
-    <t>Implementation Roadmap — RE Tier : CIS IG Alignment &amp; 12-Month Phasing</t>
-  </si>
-  <si>
-    <t>SECTION A — SEBI RE Tier : CIS Implementation Group Alignment</t>
-  </si>
-  <si>
-    <t>SEBI CSCRF : CIS Controls v8.1 — Full Crosswalk Mapping</t>
-  </si>
-  <si>
     <t xml:space="preserve">Category-level mapping | SEBI CSCRF Circular Aug 2024 | CIS Controls v8.1 (2024)  </t>
   </si>
   <si>
@@ -329,9 +319,6 @@
 • Remediation closure evidence</t>
   </si>
   <si>
-    <t>SEBI mandates VAPT by CERT-In empanelled firms only — commercial pen test firms without CERT-In empanelment do NOT satisfy this requirement. Maintain separate VAPT register.</t>
-  </si>
-  <si>
     <t>CRITICAL</t>
   </si>
   <si>
@@ -339,9 +326,6 @@
   </si>
   <si>
     <t>Supply Chain &amp; Third-Party Risk Assessment</t>
-  </si>
-  <si>
-    <t>15.1–15.7 Full Control Set</t>
   </si>
   <si>
     <t>• Third-party risk assessment reports
@@ -349,16 +333,10 @@
 • Annual vendor security review log</t>
   </si>
   <si>
-    <t>Review data localization requirements — SEBI CSCRF implies critical trading and investor data must remain within India. Affects cloud provider selection.</t>
-  </si>
-  <si>
     <t>MEDIUM</t>
   </si>
   <si>
     <t>ID.IM</t>
-  </si>
-  <si>
-    <t>Improvement — Lessons Learned &amp; Posture Review</t>
   </si>
   <si>
     <t>17.7 Conduct Post-Incident Reviews</t>
@@ -375,6 +353,214 @@
     <t>IDENTIFY  FUNCTION</t>
   </si>
   <si>
+    <t>PROTECT</t>
+  </si>
+  <si>
+    <t>PR.AA</t>
+  </si>
+  <si>
+    <t>Identity Management &amp; Privileged Access Control</t>
+  </si>
+  <si>
+    <t>CIS 5 + CIS 6</t>
+  </si>
+  <si>
+    <t>Account Management + Access Control Management</t>
+  </si>
+  <si>
+    <t>5.1 User Account Inventory
+5.3 Disable Dormant Accounts
+6.3 Require MFA for Admin
+6.4 Require MFA for Remote</t>
+  </si>
+  <si>
+    <t>• Active Directory / IAM user inventory export
+• MFA enforcement policy and logs
+• Privileged access review (quarterly)
+• Access certification records</t>
+  </si>
+  <si>
+    <t>CSCRF explicitly mandates MFA for all privileged accounts and remote access. CIS 6.3/6.4 directly satisfies this. Document admin account segregation.</t>
+  </si>
+  <si>
+    <t>PR.AT</t>
+  </si>
+  <si>
+    <t>Security Awareness &amp; Phishing Simulation</t>
+  </si>
+  <si>
+    <t>Security Awareness and Skills Training</t>
+  </si>
+  <si>
+    <t>14.1 Establish Awareness Programme
+14.2 Train Workforce on Attack Vectors
+14.4 Train Workforce on Causes of Unintended Data Exposure</t>
+  </si>
+  <si>
+    <t>• Annual security awareness training completion records
+• Phishing simulation campaign reports
+• Role-based training completion logs for IT/security staff</t>
+  </si>
+  <si>
+    <t>CSCRF mandates phishing simulation for Qualified REs and above. Document as evidence under CIS 14.2. Track click rates over time for posture improvement evidence.</t>
+  </si>
+  <si>
+    <t>PR.DS</t>
+  </si>
+  <si>
+    <t>Data Security &amp; Data Loss Prevention</t>
+  </si>
+  <si>
+    <t>CIS 3</t>
+  </si>
+  <si>
+    <t>Data Protection</t>
+  </si>
+  <si>
+    <t>3.1 Data Classification
+3.7 Encrypt Sensitive Data
+3.11 Encrypt Sensitive Data in Transit
+3.13 Deploy DLP Solutions</t>
+  </si>
+  <si>
+    <t>• Data classification policy and register
+• DLP tool deployment evidence (rules configuration + alerts log)
+• Encryption standards documentation
+• Sensitive data discovery scan results</t>
+  </si>
+  <si>
+    <t>DLP policies must cover UPSI (Unpublished Price Sensitive Information) under SEBI PIT Regulations 2015. Ensure DLP rules tag and alert on UPSI-related data patterns.</t>
+  </si>
+  <si>
+    <t>PR.PS</t>
+  </si>
+  <si>
+    <t>CIS 4 + CIS 7</t>
+  </si>
+  <si>
+    <t>Secure Configuration + Vulnerability Management</t>
+  </si>
+  <si>
+    <t>4.1 Establish Secure Config Process
+4.4 Implement Automated OS Patch Mgmt
+7.4 Manage OS Vulnerabilities</t>
+  </si>
+  <si>
+    <t>• Hardening baselines (CIS Benchmarks recommended)
+• Patch management records with SLA adherence metrics
+• Configuration compliance scan reports</t>
+  </si>
+  <si>
+    <t>CSCRF prescribes patching SLAs: Critical = 30 days, High = 45 days, Medium = 60 days. Document SLA adherence rate in monthly security metrics dashboard.</t>
+  </si>
+  <si>
+    <t>PR.IR</t>
+  </si>
+  <si>
+    <t>Infrastructure Resilience &amp; Disaster Recovery</t>
+  </si>
+  <si>
+    <t>CIS 11 + CIS 12</t>
+  </si>
+  <si>
+    <t>Data Recovery + Network Infrastructure Management</t>
+  </si>
+  <si>
+    <t>11.1 Establish Data Recovery Process
+11.3 Protect Recovery Data
+11.4 Test Data Recovery</t>
+  </si>
+  <si>
+    <t>• DR Plan with defined RTO/RPO per system tier
+• Annual DR drill report and sign-off
+• Backup integrity test results (monthly)
+• Business continuity plan</t>
+  </si>
+  <si>
+    <t>PR.NS</t>
+  </si>
+  <si>
+    <t>CIS 12 + CIS 13</t>
+  </si>
+  <si>
+    <t>Network Infrastructure + Network Monitoring &amp; Defense</t>
+  </si>
+  <si>
+    <t>12.2 Establish Network Infrastructure Mgmt
+12.8 Manage Network Infrastructure
+13.4 Perform Traffic Filtering</t>
+  </si>
+  <si>
+    <t>• Network architecture diagram (zoned)
+• Firewall policy ruleset review (quarterly)
+• Network segmentation test results
+• DMZ configuration documentation</t>
+  </si>
+  <si>
+    <t>CSCRF requires network segmentation separating trading, settlement, clearing, and internet-facing zones. Map to CIS 12.2 and validate zone isolation with penetration test findings.</t>
+  </si>
+  <si>
+    <t>PR.AS</t>
+  </si>
+  <si>
+    <t>CIS 16</t>
+  </si>
+  <si>
+    <t>Application Software Security</t>
+  </si>
+  <si>
+    <t>16.1 Establish SDLC Programme
+16.2 Establish Secure Dev Process
+16.12 Implement Code-Level Security Checks</t>
+  </si>
+  <si>
+    <t>• SAST/DAST scan reports for production applications
+• Secure SDLC policy documentation
+• SBOM export files (SPDX or CycloneDX format)
+• Open-source component vulnerability scan</t>
+  </si>
+  <si>
+    <t>CSCRF mandates Software Bill of Materials (SBOM) for trading platform applications. Use tools like Syft or SPDX to generate SBOM. Monitor SBOM for known CVEs continuously.</t>
+  </si>
+  <si>
+    <t>PR.API</t>
+  </si>
+  <si>
+    <t>Application Software Security (partial)</t>
+  </si>
+  <si>
+    <t>16.1 Establish SDLC Programme
+16.5 Use Up-to-Date and Trusted Third-Party Software</t>
+  </si>
+  <si>
+    <t>• API inventory register
+• API gateway configuration evidence
+• OWASP API Top 10 assessment report
+• API anomaly detection alert log</t>
+  </si>
+  <si>
+    <t>PR.MA</t>
+  </si>
+  <si>
+    <t>Mobile Application Security</t>
+  </si>
+  <si>
+    <t>16.1 Establish SDLC Programme
+16.8 Separate Production &amp; Non-Prod Environments</t>
+  </si>
+  <si>
+    <t>• Mobile app DAST scan reports (OWASP MASVS basis)
+• Certificate pinning implementation evidence
+• Jailbreak/root detection test results
+• App store security review documentation</t>
+  </si>
+  <si>
+    <t>CSCRF requires binary protection, certificate pinning, and jailbreak/root detection for trading mobile apps. Map against OWASP MASVS Level 2 for comprehensive coverage beyond CIS 16.</t>
+  </si>
+  <si>
+    <t>PROTECT  FUNCTION</t>
+  </si>
+  <si>
     <t>DETECT</t>
   </si>
   <si>
@@ -388,12 +574,6 @@
   </si>
   <si>
     <t>Audit Log Management + Network Monitoring &amp; Defense</t>
-  </si>
-  <si>
-    <t>8.1 Establish Audit Log Mgmt
-8.2 Collect Audit Logs
-8.11 Centralize Log Aggregation
-13.1 Centralise Security Event Alerting</t>
   </si>
   <si>
     <t>• Log management policy with retention schedule
@@ -408,9 +588,6 @@
     <t>DE.AE</t>
   </si>
   <si>
-    <t>Adverse Event Analysis — SIEM &amp; UEBA</t>
-  </si>
-  <si>
     <t>CIS 13 + CIS 10</t>
   </si>
   <si>
@@ -453,9 +630,6 @@
     <t>DE.TI</t>
   </si>
   <si>
-    <t>Threat Intelligence — SEBI CTIS Integration</t>
-  </si>
-  <si>
     <t>CIS 13</t>
   </si>
   <si>
@@ -472,23 +646,904 @@
 • Monthly SOC operations report</t>
   </si>
   <si>
-    <t>SEBI mandates SOC operations for ALL REs: In-house (MIIs/Qualified), Hybrid (Mid-size), or SEBI-approved SOCaaS (Small REs). No equivalent CIS prescriptive requirement — CIS supports but doesn't mandate SOC model.</t>
-  </si>
-  <si>
     <t>• SEBI CTIS platform registration confirmation
 • CTIS feed integration configuration in SIEM
 • Threat intelligence consumption process documentation
 • IOC/TTP tracking log</t>
   </si>
   <si>
-    <t>CSCRF requires integration with SEBI's Cyber Threat Intelligence Sharing (CTIS) platform. Register on CTIS platform and configure SIEM to ingest CTIS IOC feeds. No direct CIS equivalent — this is India-specific operationally.</t>
+    <t>RESPOND</t>
+  </si>
+  <si>
+    <t>RS.MA</t>
+  </si>
+  <si>
+    <t>Incident Management &amp; Response</t>
+  </si>
+  <si>
+    <t>17.1 Designate IR Personnel
+17.2 Establish IR Process
+17.4 Establish Communication Sharing
+17.6 Define Mechanisms for Communicating During Events</t>
+  </si>
+  <si>
+    <t>CSCRF mandates 6-hour initial report to SEBI and 2-hour notification to CERT-In for critical incidents per IT (Amendment) Act 2008. Document escalation timelines explicitly in IR Plan with regulatory notification workflows.</t>
+  </si>
+  <si>
+    <t>RS.CO</t>
+  </si>
+  <si>
+    <t>17.6 Define Communication Mechanisms</t>
+  </si>
+  <si>
+    <t>• CERT-In incident report templates (pre-filled)
+• SEBI incident notification format
+• Designated Reporting Officer appointment letter
+• Reporting drill completion records (quarterly)</t>
+  </si>
+  <si>
+    <t>CERT-In 6-hour reporting window (CERT-In Directions 2022) and SEBI incident notification format are India-only regulatory obligations. CIS 17 supports communication planning but cannot substitute mandatory regulatory reporting.</t>
+  </si>
+  <si>
+    <t>RS.AN</t>
+  </si>
+  <si>
+    <t>Incident Analysis &amp; Digital Forensics</t>
+  </si>
+  <si>
+    <t>CIS 17 + CIS 8</t>
+  </si>
+  <si>
+    <t>Incident Response + Audit Log Management</t>
+  </si>
+  <si>
+    <t>17.7 Conduct Post-Incident Reviews
+8.2 Collect Audit Logs
+8.11 Centralize Log Aggregation</t>
+  </si>
+  <si>
+    <t>• Forensic investigation reports
+• Evidence chain of custody documentation
+• Root cause analysis (RCA) reports
+• Log integrity (hash verification) evidence</t>
+  </si>
+  <si>
+    <t>RS.CCMP</t>
+  </si>
+  <si>
+    <t>Cyber Crisis Management Plan (SEBI Format)</t>
+  </si>
+  <si>
+    <t>• CCMP document (SEBI-prescribed format)
+• CCMP tabletop exercise report (annual)
+• Crisis communication templates
+• Recovery time objectives per trading system</t>
+  </si>
+  <si>
+    <t>RESPOND  FUNCTION</t>
+  </si>
+  <si>
+    <t>RECOVER</t>
+  </si>
+  <si>
+    <t>RC.RP</t>
+  </si>
+  <si>
+    <t>Incident Recovery &amp; System Restoration</t>
+  </si>
+  <si>
+    <t>CIS 11</t>
+  </si>
+  <si>
+    <t>Data Recovery</t>
+  </si>
+  <si>
+    <t>11.1 Establish Data Recovery Process
+11.2 Perform Automated Backups
+11.3 Protect Recovery Data
+11.4 Test Data Recovery</t>
+  </si>
+  <si>
+    <t>• Data recovery runbook per critical system
+• Backup completion logs (automated)
+• Recovery test results with RTO/RPO validation
+• Offsite backup confirmation records</t>
+  </si>
+  <si>
+    <t>Supplement with documented RTO/RPO targets per system criticality as required by SEBI for trading infrastructure. Include recovery SLA in DR plan.</t>
+  </si>
+  <si>
+    <t>RC.CO</t>
+  </si>
+  <si>
+    <t>• Recovery status communication templates
+• Exchange notification procedures
+• Investor communication plan for data breach scenarios</t>
+  </si>
+  <si>
+    <t>RC.IM</t>
+  </si>
+  <si>
+    <t>Post-Incident Improvement &amp; Lessons Learned</t>
+  </si>
+  <si>
+    <t>• Post-incident review (PIR) reports
+• Lessons learned register (updated after each incident)
+• Control improvement tracking log
+• Annual improvement report to Board</t>
+  </si>
+  <si>
+    <t>Feed PIR findings into both the CIS maturity model and annual CSCRF cyber audit evidence package. Lessons learned log is a key audit artifact for CERT-In empanelled auditors.</t>
+  </si>
+  <si>
+    <t>RC.AUDIT</t>
+  </si>
+  <si>
+    <t>Annual Cyber Audit by CERT-In Empanelled Firm</t>
+  </si>
+  <si>
+    <t>Penetration Testing (partial scope only)</t>
+  </si>
+  <si>
+    <t>18.2 Perform Periodic External Pen Tests</t>
+  </si>
+  <si>
+    <t>• CERT-In empanelled auditor engagement letter
+• Audit scope document and work programme
+• Final audit report (SEBI format)
+• Management response and remediation plan
+• Remediation closure evidence</t>
+  </si>
+  <si>
+    <t>RECOVER  FUNCTION</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF : CIS Controls v8.1 - Full Crosswalk Mapping</t>
+  </si>
+  <si>
+    <t>SEBI mandates VAPT by CERT-In empanelled firms only - commercial pen test firms without CERT-In empanelment do NOT satisfy this requirement. Maintain separate VAPT register.</t>
+  </si>
+  <si>
+    <t>Review data localization requirements - SEBI CSCRF implies critical trading and investor data must remain within India. Affects cloud provider selection.</t>
+  </si>
+  <si>
+    <t>Improvement - Lessons Learned &amp; Posture Review</t>
+  </si>
+  <si>
+    <t>Adverse Event Analysis - SIEM &amp; UEBA</t>
+  </si>
+  <si>
+    <t>SEBI mandates SOC operations for ALL REs: In-house (MIIs/Qualified), Hybrid (Mid-size), or SEBI-approved SOCaaS (Small REs). No equivalent CIS prescriptive requirement - CIS supports but doesn't mandate SOC model.</t>
+  </si>
+  <si>
+    <t>Threat Intelligence - SEBI CTIS Integration</t>
+  </si>
+  <si>
+    <t>CSCRF requires integration with SEBI's Cyber Threat Intelligence Sharing (CTIS) platform. Register on CTIS platform and configure SIEM to ingest CTIS IOC feeds. No direct CIS equivalent - this is India-specific operationally.</t>
+  </si>
+  <si>
+    <t>• Incident Response Plan (IRP) - current version
+• IR team roster and contact tree
+• Incident log / ticketing system extract
+• Tabletop exercise reports (annual)</t>
+  </si>
+  <si>
+    <t>Incident Reporting - CERT-In &amp; SEBI Notifications</t>
+  </si>
+  <si>
+    <t>Ensure log integrity (CIS 8.2 - hash/tamper-evidence) is maintained for evidential chain of custody during forensic investigations and regulatory inquiry.</t>
+  </si>
+  <si>
+    <t>SEBI mandates a formal CCMP covering market disruption, trading halt, investor data breach, and system recovery scenarios - in SEBI-prescribed format. CIS 17 informs structure but a SEBI-format CCMP is a mandatory standalone obligation.</t>
+  </si>
+  <si>
+    <t>Platform Security - Patch &amp; Secure Configuration</t>
+  </si>
+  <si>
+    <t>CSCRF mandates documented RTO/RPO targets for critical trading systems and annual DR drill evidence. CIS 11 covers data recovery but not DR orchestration - supplement with full DR runbook.</t>
+  </si>
+  <si>
+    <t>Network Security - Segmentation &amp; Perimeter</t>
+  </si>
+  <si>
+    <t>Application Security - SDLC &amp; SBOM</t>
+  </si>
+  <si>
+    <t>API Security - Trading &amp; Data APIs</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF has a dedicated API Security mandate covering authentication, rate limiting, and anomaly detection on trading APIs. CIS 16 covers application security broadly - supplement with standalone OWASP API Top 10 assessment.</t>
+  </si>
+  <si>
+    <t>Recovery Communication - Investors &amp; Exchanges</t>
+  </si>
+  <si>
+    <t>CSCRF requires investor communication and stock exchange notification during recovery phase. CIS 17 partially covers recovery communication - supplement with standalone investor/exchange notification protocols.</t>
+  </si>
+  <si>
+    <t>Annual Cyber Audit by a CERT-In empanelled firm is a SEBI legal requirement - not satisfied by CIS assessments alone. Maintain auditor independence. Scope must cover all systems classified as Critical Information Infrastructure (CII).</t>
+  </si>
+  <si>
+    <t>7.1 Establish Vulnerability Mgmt. Process
+7.7 Remediate Detected Vulnerabilities</t>
+  </si>
+  <si>
+    <t>8.1 Establish Audit Log Mgmt.
+8.2 Collect Audit Logs
+8.11 Centralize Log Aggregation
+13.1 Centralise Security Event Alerting</t>
+  </si>
+  <si>
+    <t>CSCRF FUNCTION COLOURS</t>
+  </si>
+  <si>
+    <t>Governance, risk strategy, policy, supply chain risk management</t>
+  </si>
+  <si>
+    <t>Asset management, risk assessment, third-party risk, improvement</t>
+  </si>
+  <si>
+    <t>Access control, data security, platform hardening, network, application, API security</t>
+  </si>
+  <si>
+    <t>Continuous monitoring, SIEM, SOC operations, threat intelligence</t>
+  </si>
+  <si>
+    <t>Incident management, CERT-In reporting, analysis, crisis management</t>
+  </si>
+  <si>
+    <t>Recovery, restoration, investor communication, post-incident improvement, cyber audit</t>
+  </si>
+  <si>
+    <t>COVERAGE TYPE COLOURS</t>
+  </si>
+  <si>
+    <t>CIS safeguard(s) fully satisfy the CSCRF control objective. Evidence directly reusable.</t>
+  </si>
+  <si>
+    <t>CIS covers the intent but CSCRF adds India-specific specificity. Supplement evidence required.</t>
+  </si>
+  <si>
+    <t>CSCRF requirement has no CIS equivalent. Requires standalone compliance process.</t>
+  </si>
+  <si>
+    <t>CIS Exceeds CSCRF</t>
+  </si>
+  <si>
+    <t>CIS control addresses risks not explicitly mandated by CSCRF. Recommended as best practice.</t>
+  </si>
+  <si>
+    <t>CIS IMPLEMENTATION GROUP (IG) COLOURS</t>
+  </si>
+  <si>
+    <t>Intermediate controls for organisations with dedicated security staff and elevated risk.</t>
+  </si>
+  <si>
+    <t>Advanced controls for organisations facing sophisticated threats (MIIs, large qualified REs).</t>
+  </si>
+  <si>
+    <t>AUDIT PRIORITY COLOURS</t>
+  </si>
+  <si>
+    <t>ABBREVIATIONS &amp; REFERENCES</t>
+  </si>
+  <si>
+    <t>SEBI</t>
+  </si>
+  <si>
+    <t>Securities and Exchange Board of India</t>
+  </si>
+  <si>
+    <t>CSCRF</t>
+  </si>
+  <si>
+    <t>Cybersecurity and Cyber Resilience Framework (SEBI, 2024)</t>
+  </si>
+  <si>
+    <t>CIS</t>
+  </si>
+  <si>
+    <t>Center for Internet Security</t>
+  </si>
+  <si>
+    <t>CERT-In</t>
+  </si>
+  <si>
+    <t>Indian Computer Emergency Response Team (Ministry of Electronics &amp; IT)</t>
+  </si>
+  <si>
+    <t>RE</t>
+  </si>
+  <si>
+    <t>Regulated Entity (under SEBI jurisdiction)</t>
+  </si>
+  <si>
+    <t>MII</t>
+  </si>
+  <si>
+    <t>Market Infrastructure Institution (NSE, BSE, CDSL, NSDL, CCIL, etc.)</t>
+  </si>
+  <si>
+    <t>VAPT</t>
+  </si>
+  <si>
+    <t>Vulnerability Assessment and Penetration Testing</t>
+  </si>
+  <si>
+    <t>SBOM</t>
+  </si>
+  <si>
+    <t>Software Bill of Materials</t>
+  </si>
+  <si>
+    <t>CCMP</t>
+  </si>
+  <si>
+    <t>Cyber Crisis Management Plan</t>
+  </si>
+  <si>
+    <t>CTIS</t>
+  </si>
+  <si>
+    <t>Cyber Threat Intelligence Sharing (SEBI platform)</t>
+  </si>
+  <si>
+    <t>UPSI</t>
+  </si>
+  <si>
+    <t>Unpublished Price Sensitive Information (SEBI PIT Regulations, 2015)</t>
+  </si>
+  <si>
+    <t>CII</t>
+  </si>
+  <si>
+    <t>Critical Information Infrastructure</t>
+  </si>
+  <si>
+    <t>IRP</t>
+  </si>
+  <si>
+    <t>Incident Response Plan</t>
+  </si>
+  <si>
+    <t>DLP</t>
+  </si>
+  <si>
+    <t>Data Loss Prevention</t>
+  </si>
+  <si>
+    <t>IG</t>
+  </si>
+  <si>
+    <t>Implementation Group (CIS Controls categorization: IG1, IG2, IG3)</t>
+  </si>
+  <si>
+    <t>NIST CSF</t>
+  </si>
+  <si>
+    <t>NIST Cybersecurity Framework 2.0 (conceptual parent of SEBI CSCRF structure)</t>
+  </si>
+  <si>
+    <t>SOCaaS</t>
+  </si>
+  <si>
+    <t>SOC-as-a-Service (SEBI-approved model for Small REs)</t>
+  </si>
+  <si>
+    <t>RTO/RPO</t>
+  </si>
+  <si>
+    <t>Recovery Time Objective / Recovery Point Objective</t>
+  </si>
+  <si>
+    <t>Legend - Colour Codes, Abbreviations &amp; Framework References</t>
+  </si>
+  <si>
+    <t>Essential cyber hygiene - applicable to all organisations. Minimum baseline.</t>
+  </si>
+  <si>
+    <t>Regulatory obligation - non-compliance may result in SEBI enforcement or legal liability.</t>
+  </si>
+  <si>
+    <t>Significant compliance requirement - must be in place for annual cyber audit.</t>
+  </si>
+  <si>
+    <t>Good practice - include in Year 2 implementation plan.</t>
+  </si>
+  <si>
+    <t>Implementation Roadmap - RE Tier : CIS IG Alignment &amp; 12-Month Phasing</t>
+  </si>
+  <si>
+    <t>SECTION A - SEBI RE Tier : CIS Implementation Group Alignment</t>
+  </si>
+  <si>
+    <t>Qualified Regulated Entities</t>
+  </si>
+  <si>
+    <t>Large brokers (&gt;10L clients), custodians, AMCs &gt;₹5,000 Cr AUM</t>
+  </si>
+  <si>
+    <t>Hybrid SOC or managed SOC
+SIEM mandatory</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>• Annual CERT-In VAPT
+• SOC (hybrid)
+• CCMP
+• SBOM (own platforms)
+• API security
+• CERT-In reporting workflow</t>
+  </si>
+  <si>
+    <t>Year 1 baseline by Jan 2025
+Year 2 by Dec 2025</t>
+  </si>
+  <si>
+    <t>Mid-Size Regulated Entities</t>
+  </si>
+  <si>
+    <t>Mid-tier brokers, Investment Advisors, Registrar &amp; Transfer Agents</t>
+  </si>
+  <si>
+    <t>Managed SOC or SOCaaS
+SIEM recommended</t>
+  </si>
+  <si>
+    <t>• Annual CERT-In VAPT
+• SOC (managed)
+• CCMP (simplified)
+• CERT-In reporting workflow</t>
+  </si>
+  <si>
+    <t>6-month implementation window</t>
+  </si>
+  <si>
+    <t>Small Regulated Entities</t>
+  </si>
+  <si>
+    <t>Sub-brokers, small Investment Advisors, small RTA</t>
+  </si>
+  <si>
+    <t>SEBI-approved SOCaaS
+(subscription model)</t>
+  </si>
+  <si>
+    <t>Biennial</t>
+  </si>
+  <si>
+    <t>• SEBI-approved SOCaaS subscription
+• Basic IR Plan with CERT-In reporting
+• Annual security awareness training</t>
+  </si>
+  <si>
+    <t>12-month phased roll-out</t>
+  </si>
+  <si>
+    <t>IG2 - IG3
+(Year 1 - Year 2)</t>
+  </si>
+  <si>
+    <t>Year 1: CIS 1-13
+Year 2: CIS 14-18</t>
+  </si>
+  <si>
+    <t>CIS 1-13 minimum
+CIS 14 &amp; 17 essential</t>
+  </si>
+  <si>
+    <t>CIS 1-6, 8, 11, 14
+Essential cyber hygiene</t>
+  </si>
+  <si>
+    <t>15.1-15.7 Full Control Set</t>
+  </si>
+  <si>
+    <t>17.1-17.7 Full IR Set</t>
+  </si>
+  <si>
+    <t>SECTION B — 12-Month Implementation Roadmap (Qualified RE Reference Model)</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Timeframe</t>
+  </si>
+  <si>
+    <t>Theme</t>
+  </si>
+  <si>
+    <t>CIS Controls Targeted</t>
+  </si>
+  <si>
+    <t>CSCRF Milestones</t>
+  </si>
+  <si>
+    <t>India-Specific Actions</t>
+  </si>
+  <si>
+    <t>Key Deliverables</t>
+  </si>
+  <si>
+    <t>Success Metrics</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Foundation &amp; Inventory</t>
+  </si>
+  <si>
+    <t>CIS 1: Asset Inventory
+CIS 2: Software Inventory
+CIS 5: Account Management
+CIS 6: Access Control (MFA)</t>
+  </si>
+  <si>
+    <t>• Complete asset inventory
+• MFA on all privileged accounts
+• Establish IR Plan skeleton</t>
+  </si>
+  <si>
+    <t>• CERT-In reporting officer designated
+• Reporting templates pre-filled</t>
+  </si>
+  <si>
+    <t>• Asset register (hardware + software)
+• MFA enforcement logs
+• IR Plan v1.0
+• CERT-In designation letter</t>
+  </si>
+  <si>
+    <t>100% privileged accounts MFA-enabled
+Asset inventory &gt;95% coverage
+IR Plan signed off by CISO</t>
+  </si>
+  <si>
+    <t>IT Security Lead</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Protection Hardening</t>
+  </si>
+  <si>
+    <t>CIS 3: Data Protection (DLP)
+CIS 4: Secure Configuration
+CIS 7: Vulnerability Management
+CIS 11: Data Recovery
+CIS 12: Network Segmentation</t>
+  </si>
+  <si>
+    <t>• DLP deployment covering UPSI data
+• Vulnerability scanning active
+• Network zones documented</t>
+  </si>
+  <si>
+    <t>• Data classification register with UPSI tier
+• DR plan with RTO/RPO targets
+• Patch management SLA tracking starts</t>
+  </si>
+  <si>
+    <t>• DLP policy + deployment evidence
+• Network architecture diagram
+• DR plan with RTO/RPO per system
+• Patch SLA dashboard</t>
+  </si>
+  <si>
+    <t>DLP alerts operational
+Critical patches &lt;30 day SLA met ≥95%
+DR test completed</t>
+  </si>
+  <si>
+    <t>IT Security + Infrastructure</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Detection &amp; Governance</t>
+  </si>
+  <si>
+    <t>CIS 8: Audit Log Management
+CIS 13: SIEM + Network Monitoring
+CIS 14: Security Awareness
+CIS 15: Vendor Risk</t>
+  </si>
+  <si>
+    <t>• SIEM operational with baseline use cases
+• Security awareness programme launched
+• Log retention policy active (180 days online)</t>
+  </si>
+  <si>
+    <t>• SOC operational (managed or in-house)
+• SEBI CTIS platform registration
+• First CERT-In empanelled VAPT scheduled</t>
+  </si>
+  <si>
+    <t>• SIEM use case catalogue
+• SOC SLA agreement
+• CTIS registration confirmation
+• Awareness training completion records</t>
+  </si>
+  <si>
+    <t>SIEM detecting &gt;15 use cases live
+80%+ staff awareness training complete
+VAPT vendor contracted</t>
+  </si>
+  <si>
+    <t>SOC Manager / CISO</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Advanced Controls &amp; First Audit</t>
+  </si>
+  <si>
+    <t>CIS 16: Application Security
+CIS 17: IR Maturity
+CIS 18: Penetration Testing</t>
+  </si>
+  <si>
+    <t>• SAST/DAST on critical applications
+• CCMP tabletop exercise completed
+• IR Plan v2.0 with regulatory timelines</t>
+  </si>
+  <si>
+    <t>• CERT-In VAPT completed
+• CCMP finalised in SEBI format
+• Board cyber posture report submitted
+• Prepare for annual CERT-In audit</t>
+  </si>
+  <si>
+    <t>• VAPT final report + remediation plan
+• CCMP document
+• Board presentation (cyber posture)
+• Audit readiness checklist</t>
+  </si>
+  <si>
+    <t>VAPT remediation plan accepted
+CCMP tabletop passed
+Board report presented
+Audit readiness ≥85%</t>
+  </si>
+  <si>
+    <t>CISO + Compliance</t>
+  </si>
+  <si>
+    <t>Months 1-3</t>
+  </si>
+  <si>
+    <t>Months 4-6</t>
+  </si>
+  <si>
+    <t>Months 7-9</t>
+  </si>
+  <si>
+    <t>Months 10-12</t>
+  </si>
+  <si>
+    <t>CSCRF Ref</t>
+  </si>
+  <si>
+    <t>Requirement</t>
+  </si>
+  <si>
+    <t>Applicable RE Tier</t>
+  </si>
+  <si>
+    <t>Regulatory Citation</t>
+  </si>
+  <si>
+    <t>Standalone Control Action</t>
+  </si>
+  <si>
+    <t>Key Evidence Artifacts</t>
+  </si>
+  <si>
+    <t>Deadline / Frequency</t>
+  </si>
+  <si>
+    <t>Risk if Missing</t>
+  </si>
+  <si>
+    <t>Annual VAPT by CERT-In Empanelled Vendor</t>
+  </si>
+  <si>
+    <t>All REs (MII: biannual, Qualified: annual, Mid-size: annual, Small: biennial)</t>
+  </si>
+  <si>
+    <t>• Maintain CERT-In empanelled vendor register
+• Define VAPT scope annually
+• Track remediation to closure</t>
+  </si>
+  <si>
+    <t>• Engagement letter
+• VAPT scope doc
+• Final VAPT report
+• Remediation tracker</t>
+  </si>
+  <si>
+    <t>Annual (MII/Qualified)
+Biennial (Small REs)</t>
+  </si>
+  <si>
+    <t>PR.AS-SBOM</t>
+  </si>
+  <si>
+    <t>Software Bill of Materials (SBOM) for Trading Platforms</t>
+  </si>
+  <si>
+    <t>MIIs &amp; Qualified REs</t>
+  </si>
+  <si>
+    <t>• Implement SBOM tooling (Syft/SPDX/CycloneDX)
+• Maintain component inventory
+• Monitor CVEs in SBOM dependencies continuously</t>
+  </si>
+  <si>
+    <t>• SBOM export files (machine-readable)
+• CVE monitoring alerts log
+• SBOM update change log</t>
+  </si>
+  <si>
+    <t>Generated at each release
+Reviewed monthly</t>
+  </si>
+  <si>
+    <t>Undetected supply chain vulnerabilities in trading platform; SEBI audit finding</t>
+  </si>
+  <si>
+    <t>Dedicated API Security Programme</t>
+  </si>
+  <si>
+    <t>All REs offering API-based trading or data services</t>
+  </si>
+  <si>
+    <t>• Create API inventory register
+• Deploy API gateway with rate limiting &amp; anomaly detection
+• Conduct OWASP API Top 10 assessment annually</t>
+  </si>
+  <si>
+    <t>• API inventory
+• Gateway config evidence
+• OWASP API Top 10 assessment
+• API monitoring logs</t>
+  </si>
+  <si>
+    <t>Programme: Ongoing
+Formal assessment: Annual</t>
+  </si>
+  <si>
+    <t>Unauthorised API access to trading systems; investor data exposure; regulatory finding</t>
+  </si>
+  <si>
+    <t>All REs (model varies by tier)</t>
+  </si>
+  <si>
+    <t>Small REs: Subscribe to SEBI-approved SOCaaS
+Qualified REs: In-house or hybrid SOC with SLA
+MIIs: Dedicated in-house SOC</t>
+  </si>
+  <si>
+    <t>• SOC SLA / service agreement
+• SOC staffing model
+• Escalation matrix
+• Monthly SOC ops report</t>
+  </si>
+  <si>
+    <t>Operational: Continuous (24x7)
+Review: Annual</t>
+  </si>
+  <si>
+    <t>Undetected incidents; delayed CERT-In reporting; SEBI enforcement</t>
+  </si>
+  <si>
+    <t>DE.TI-CTIS</t>
+  </si>
+  <si>
+    <t>SEBI Cyber Threat Intelligence Sharing (CTIS) Integration</t>
+  </si>
+  <si>
+    <t>• Register on SEBI CTIS platform
+• Configure SIEM to ingest CTIS IOC feed
+• Document TI consumption process</t>
+  </si>
+  <si>
+    <t>• CTIS registration confirmation
+• SIEM integration config
+• IOC consumption log</t>
+  </si>
+  <si>
+    <t>Registration: One-time
+Feed ingestion: Continuous</t>
+  </si>
+  <si>
+    <t>Missed India-specific threat indicators; delayed detection of sector-wide attacks</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF  4.2 + CERT-In Empanelment Scheme</t>
+  </si>
+  <si>
+    <t>Gap Analysis - India-Specific Obligations &amp; CIS Best-Practice Extensions</t>
+  </si>
+  <si>
+    <t>SECTION A - India-Specific Obligations (No Direct CIS Equivalent)</t>
+  </si>
+  <si>
+    <t>Regulatory non-compliance - audit finding, potential SEBI enforcement action</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF  5.3 - Application Security</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF  5.4 - API Security</t>
+  </si>
+  <si>
+    <t>Security Operations Centre (SOC) - Mandatory for All REs</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF  6 - SOC Operations</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF  6.3 - Threat Intelligence</t>
+  </si>
+  <si>
+    <t>WORKBOOK CONTENTS</t>
+  </si>
+  <si>
+    <t>India-Specific obligations with no CIS equivalent; CIS best-practices beyond CSCRF</t>
+  </si>
+  <si>
+    <t>Practitioner template to track compliance evidence for each mapped control pair</t>
+  </si>
+  <si>
+    <t>Colour codes, abbreviations, and framework reference guide</t>
+  </si>
+  <si>
+    <t>1 - Crosswalk</t>
+  </si>
+  <si>
+    <t>2 - Gap Analysis</t>
+  </si>
+  <si>
+    <t>3 - Implementation Roadmap</t>
+  </si>
+  <si>
+    <t>4 - Evidence Tracker</t>
+  </si>
+  <si>
+    <t>5 - Legend</t>
+  </si>
+  <si>
+    <t>Full CSCRF : CIS Controls v8.1 mapping table with coverage classification and notes</t>
+  </si>
+  <si>
+    <t>RE Tier : CIS Implementation Group alignment and 12-month phased roadmap</t>
+  </si>
+  <si>
+    <t>Prepared By: Ronit Yadav &lt;ronit.yadav@sbicapsec.com&gt;</t>
+  </si>
+  <si>
+    <t>Reviewed by: Nilisha Wandile</t>
+  </si>
+  <si>
+    <t>LinkedIn: https://www.linkedin.com/in/nilisha-wandile/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="51" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -579,13 +1634,6 @@
     <font>
       <b/>
       <sz val="9"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -700,6 +1748,20 @@
     <font>
       <b/>
       <sz val="10"/>
+      <color rgb="FF5C2A1C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF5C2A1C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color rgb="FF3D1C5C"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -711,8 +1773,112 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF5C4A1C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF5C4A1C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1C4A5C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF1C4A5C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF1A3A5C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.5"/>
+      <color rgb="FF1C5C3E"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
+      <color rgb="FF1C2B3A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.5"/>
+      <color rgb="FF7C4A00"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.5"/>
+      <color rgb="FF7C1C1C"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.5"/>
+      <color rgb="FF1C2B3A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -766,11 +1932,54 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2EAE6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFEDE6F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2EDE6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6EFF2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF122947"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5EDD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -793,11 +2002,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD4C9B0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD4C9B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD4C9B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -866,87 +2088,222 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="42" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="47" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="48" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="50" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="50" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1249,6 +2606,182 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB9251F8-4A3E-BF4A-BD2B-E73CDC9A5F26}">
+  <dimension ref="A3:L19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.1640625" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" customWidth="1"/>
+    <col min="5" max="5" width="17.1640625" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="11" max="11" width="15.1640625" customWidth="1"/>
+    <col min="12" max="12" width="13.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="62"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" s="62"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" s="62" t="s">
+        <v>424</v>
+      </c>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" s="62" t="s">
+        <v>425</v>
+      </c>
+      <c r="B11" s="62"/>
+      <c r="C11" s="62" t="s">
+        <v>426</v>
+      </c>
+      <c r="D11" s="62"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="62"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="102" t="s">
+        <v>413</v>
+      </c>
+      <c r="B14" s="81"/>
+      <c r="C14" s="81"/>
+      <c r="D14" s="81"/>
+      <c r="E14" s="81"/>
+      <c r="F14" s="81"/>
+      <c r="G14" s="81"/>
+      <c r="H14" s="81"/>
+      <c r="I14" s="81"/>
+      <c r="J14" s="81"/>
+      <c r="K14" s="81"/>
+      <c r="L14" s="81"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" s="97" t="s">
+        <v>417</v>
+      </c>
+      <c r="B15" s="98"/>
+      <c r="C15" s="98"/>
+      <c r="D15" s="101" t="s">
+        <v>422</v>
+      </c>
+      <c r="E15" s="98"/>
+      <c r="F15" s="98"/>
+      <c r="G15" s="98"/>
+      <c r="H15" s="98"/>
+      <c r="I15" s="98"/>
+      <c r="J15" s="98"/>
+      <c r="K15" s="98"/>
+      <c r="L15" s="98"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" s="99" t="s">
+        <v>418</v>
+      </c>
+      <c r="B16" s="100"/>
+      <c r="C16" s="100"/>
+      <c r="D16" s="61" t="s">
+        <v>414</v>
+      </c>
+      <c r="E16" s="100"/>
+      <c r="F16" s="100"/>
+      <c r="G16" s="100"/>
+      <c r="H16" s="100"/>
+      <c r="I16" s="100"/>
+      <c r="J16" s="100"/>
+      <c r="K16" s="100"/>
+      <c r="L16" s="100"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="97" t="s">
+        <v>419</v>
+      </c>
+      <c r="B17" s="98"/>
+      <c r="C17" s="98"/>
+      <c r="D17" s="101" t="s">
+        <v>423</v>
+      </c>
+      <c r="E17" s="98"/>
+      <c r="F17" s="98"/>
+      <c r="G17" s="98"/>
+      <c r="H17" s="98"/>
+      <c r="I17" s="98"/>
+      <c r="J17" s="98"/>
+      <c r="K17" s="98"/>
+      <c r="L17" s="98"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" s="99" t="s">
+        <v>420</v>
+      </c>
+      <c r="B18" s="100"/>
+      <c r="C18" s="100"/>
+      <c r="D18" s="61" t="s">
+        <v>415</v>
+      </c>
+      <c r="E18" s="100"/>
+      <c r="F18" s="100"/>
+      <c r="G18" s="100"/>
+      <c r="H18" s="100"/>
+      <c r="I18" s="100"/>
+      <c r="J18" s="100"/>
+      <c r="K18" s="100"/>
+      <c r="L18" s="100"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" s="97" t="s">
+        <v>421</v>
+      </c>
+      <c r="B19" s="98"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="101" t="s">
+        <v>416</v>
+      </c>
+      <c r="E19" s="98"/>
+      <c r="F19" s="98"/>
+      <c r="G19" s="98"/>
+      <c r="H19" s="98"/>
+      <c r="I19" s="98"/>
+      <c r="J19" s="98"/>
+      <c r="K19" s="98"/>
+      <c r="L19" s="98"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:L19"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:L17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:L18"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:L15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1266,7 +2799,7 @@
     <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1281,7 +2814,7 @@
     </row>
     <row r="2" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="27" t="s">
-        <v>63</v>
+        <v>214</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -1296,7 +2829,7 @@
     </row>
     <row r="3" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B3" s="25"/>
       <c r="C3" s="25"/>
@@ -1346,7 +2879,7 @@
     </row>
     <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="24" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B5" s="25"/>
       <c r="C5" s="25"/>
@@ -1410,20 +2943,20 @@
       <c r="E7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="42" t="s">
+        <v>235</v>
+      </c>
+      <c r="G7" s="16" t="s">
         <v>26</v>
-      </c>
-      <c r="G7" s="16" t="s">
-        <v>27</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>18</v>
       </c>
       <c r="I7" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="18" t="s">
         <v>28</v>
-      </c>
-      <c r="J7" s="18" t="s">
-        <v>29</v>
       </c>
       <c r="K7" s="8" t="s">
         <v>21</v>
@@ -1434,31 +2967,31 @@
         <v>11</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="G8" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="19" t="s">
+      <c r="I8" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="J8" s="11" t="s">
         <v>36</v>
-      </c>
-      <c r="J8" s="11" t="s">
-        <v>37</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>21</v>
@@ -1469,19 +3002,19 @@
         <v>11</v>
       </c>
       <c r="B9" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="E9" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="F9" s="15" t="s">
         <v>41</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>42</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>17</v>
@@ -1490,18 +3023,18 @@
         <v>18</v>
       </c>
       <c r="I9" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="18" t="s">
         <v>43</v>
-      </c>
-      <c r="J9" s="18" t="s">
-        <v>44</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="30" t="s">
-        <v>102</v>
+      <c r="A10" s="29" t="s">
+        <v>94</v>
       </c>
       <c r="B10" s="25"/>
       <c r="C10" s="25"/>
@@ -1515,183 +3048,183 @@
       <c r="K10" s="25"/>
     </row>
     <row r="11" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="32" t="s">
+      <c r="F11" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="G11" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="J11" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="33" t="s">
+      <c r="K11" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="C12" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="G11" s="36" t="s">
+      <c r="D12" s="41" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="40" t="s">
+        <v>73</v>
+      </c>
+      <c r="F12" s="42" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" s="44" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" s="45" t="s">
+        <v>76</v>
+      </c>
+      <c r="K12" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="F13" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="H13" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="I13" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="J13" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="K13" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="42" t="s">
+        <v>319</v>
+      </c>
+      <c r="G14" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I14" s="44" t="s">
+        <v>88</v>
+      </c>
+      <c r="J14" s="45" t="s">
+        <v>216</v>
+      </c>
+      <c r="K14" s="43" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>217</v>
+      </c>
+      <c r="D15" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="I11" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="J11" s="39" t="s">
-        <v>73</v>
-      </c>
-      <c r="K11" s="36" t="s">
+      <c r="H15" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="I15" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="J15" s="38" t="s">
+        <v>93</v>
+      </c>
+      <c r="K15" s="35" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="40" t="s">
-        <v>74</v>
-      </c>
-      <c r="C12" s="41" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="42" t="s">
-        <v>76</v>
-      </c>
-      <c r="E12" s="41" t="s">
-        <v>77</v>
-      </c>
-      <c r="F12" s="43" t="s">
-        <v>78</v>
-      </c>
-      <c r="G12" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="I12" s="45" t="s">
-        <v>79</v>
-      </c>
-      <c r="J12" s="46" t="s">
-        <v>80</v>
-      </c>
-      <c r="K12" s="36" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B13" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="C13" s="33" t="s">
-        <v>82</v>
-      </c>
-      <c r="D13" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="E13" s="33" t="s">
-        <v>84</v>
-      </c>
-      <c r="F13" s="35" t="s">
-        <v>85</v>
-      </c>
-      <c r="G13" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="H13" s="48" t="s">
-        <v>87</v>
-      </c>
-      <c r="I13" s="38" t="s">
-        <v>88</v>
-      </c>
-      <c r="J13" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="K13" s="47" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B14" s="40" t="s">
-        <v>91</v>
-      </c>
-      <c r="C14" s="41" t="s">
-        <v>92</v>
-      </c>
-      <c r="D14" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="43" t="s">
-        <v>93</v>
-      </c>
-      <c r="G14" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="I14" s="45" t="s">
-        <v>94</v>
-      </c>
-      <c r="J14" s="46" t="s">
-        <v>95</v>
-      </c>
-      <c r="K14" s="44" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="C15" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="D15" s="34" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="G15" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="H15" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="I15" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="J15" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="K15" s="36" t="s">
-        <v>21</v>
-      </c>
-    </row>
     <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="50" t="s">
-        <v>118</v>
+      <c r="A16" s="51" t="s">
+        <v>163</v>
       </c>
       <c r="B16" s="25"/>
       <c r="C16" s="25"/>
@@ -1705,167 +3238,790 @@
       <c r="K16" s="25"/>
     </row>
     <row r="17" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="51" t="s">
+      <c r="A17" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="E17" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="F17" s="34" t="s">
+        <v>236</v>
+      </c>
+      <c r="G17" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I17" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="J17" s="38" t="s">
+        <v>156</v>
+      </c>
+      <c r="K17" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B18" s="39" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" s="40" t="s">
+        <v>218</v>
+      </c>
+      <c r="D18" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>159</v>
+      </c>
+      <c r="F18" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="G18" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H18" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" s="44" t="s">
+        <v>161</v>
+      </c>
+      <c r="J18" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="K18" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="C19" s="32" t="s">
+        <v>165</v>
+      </c>
+      <c r="D19" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="E19" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="F19" s="34" t="s">
+        <v>168</v>
+      </c>
+      <c r="G19" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="H19" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="I19" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="J19" s="38" t="s">
+        <v>219</v>
+      </c>
+      <c r="K19" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>169</v>
+      </c>
+      <c r="C20" s="40" t="s">
+        <v>220</v>
+      </c>
+      <c r="D20" s="41" t="s">
+        <v>170</v>
+      </c>
+      <c r="E20" s="40" t="s">
+        <v>171</v>
+      </c>
+      <c r="F20" s="42" t="s">
+        <v>172</v>
+      </c>
+      <c r="G20" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="H20" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="I20" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="J20" s="45" t="s">
+        <v>221</v>
+      </c>
+      <c r="K20" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="53" t="s">
+        <v>193</v>
+      </c>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="25"/>
+    </row>
+    <row r="22" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="54" t="s">
+        <v>175</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>176</v>
+      </c>
+      <c r="C22" s="32" t="s">
+        <v>177</v>
+      </c>
+      <c r="D22" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="G22" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="I22" s="37" t="s">
+        <v>222</v>
+      </c>
+      <c r="J22" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="K22" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="54" t="s">
+        <v>175</v>
+      </c>
+      <c r="B23" s="39" t="s">
+        <v>180</v>
+      </c>
+      <c r="C23" s="40" t="s">
+        <v>223</v>
+      </c>
+      <c r="D23" s="41" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="G23" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="I23" s="44" t="s">
+        <v>182</v>
+      </c>
+      <c r="J23" s="45" t="s">
+        <v>183</v>
+      </c>
+      <c r="K23" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="54" t="s">
+        <v>175</v>
+      </c>
+      <c r="B24" s="31" t="s">
+        <v>184</v>
+      </c>
+      <c r="C24" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="D24" s="33" t="s">
+        <v>186</v>
+      </c>
+      <c r="E24" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="F24" s="34" t="s">
+        <v>188</v>
+      </c>
+      <c r="G24" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H24" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I24" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="J24" s="38" t="s">
+        <v>224</v>
+      </c>
+      <c r="K24" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="54" t="s">
+        <v>175</v>
+      </c>
+      <c r="B25" s="39" t="s">
+        <v>190</v>
+      </c>
+      <c r="C25" s="40" t="s">
+        <v>191</v>
+      </c>
+      <c r="D25" s="41" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="42" t="s">
+        <v>320</v>
+      </c>
+      <c r="G25" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H25" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="I25" s="44" t="s">
+        <v>192</v>
+      </c>
+      <c r="J25" s="45" t="s">
+        <v>225</v>
+      </c>
+      <c r="K25" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="49" t="s">
+        <v>149</v>
+      </c>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="25"/>
+      <c r="K26" s="25"/>
+    </row>
+    <row r="27" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B27" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="D27" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="E27" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="F27" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="G27" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I27" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="J27" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="K27" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B28" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="32" t="s">
+      <c r="C28" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="D28" s="41" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28" s="40" t="s">
         <v>105</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="F28" s="42" t="s">
         <v>106</v>
       </c>
-      <c r="E17" s="33" t="s">
+      <c r="G28" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I28" s="44" t="s">
         <v>107</v>
       </c>
-      <c r="F17" s="35" t="s">
+      <c r="J28" s="45" t="s">
         <v>108</v>
       </c>
-      <c r="G17" s="36" t="s">
+      <c r="K28" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="C29" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="D29" s="33" t="s">
+        <v>111</v>
+      </c>
+      <c r="E29" s="32" t="s">
+        <v>112</v>
+      </c>
+      <c r="F29" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="G29" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H29" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I29" s="37" t="s">
+        <v>114</v>
+      </c>
+      <c r="J29" s="38" t="s">
+        <v>115</v>
+      </c>
+      <c r="K29" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B30" s="39" t="s">
+        <v>116</v>
+      </c>
+      <c r="C30" s="40" t="s">
+        <v>226</v>
+      </c>
+      <c r="D30" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="E30" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="F30" s="42" t="s">
+        <v>119</v>
+      </c>
+      <c r="G30" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="H17" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="I17" s="38" t="s">
-        <v>109</v>
-      </c>
-      <c r="J17" s="39" t="s">
-        <v>110</v>
-      </c>
-      <c r="K17" s="36" t="s">
+      <c r="H30" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I30" s="44" t="s">
+        <v>120</v>
+      </c>
+      <c r="J30" s="45" t="s">
+        <v>121</v>
+      </c>
+      <c r="K30" s="35" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="B18" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="C18" s="41" t="s">
-        <v>112</v>
-      </c>
-      <c r="D18" s="42" t="s">
-        <v>113</v>
-      </c>
-      <c r="E18" s="41" t="s">
-        <v>114</v>
-      </c>
-      <c r="F18" s="43" t="s">
-        <v>115</v>
-      </c>
-      <c r="G18" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="H18" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="I18" s="45" t="s">
-        <v>116</v>
-      </c>
-      <c r="J18" s="46" t="s">
-        <v>117</v>
-      </c>
-      <c r="K18" s="36" t="s">
+    <row r="31" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B31" s="39" t="s">
+        <v>122</v>
+      </c>
+      <c r="C31" s="40" t="s">
+        <v>123</v>
+      </c>
+      <c r="D31" s="41" t="s">
+        <v>124</v>
+      </c>
+      <c r="E31" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="F31" s="42" t="s">
+        <v>126</v>
+      </c>
+      <c r="G31" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="H31" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="I31" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="J31" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="K31" s="35" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="B19" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="C19" s="33" t="s">
-        <v>120</v>
-      </c>
-      <c r="D19" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="E19" s="33" t="s">
-        <v>122</v>
-      </c>
-      <c r="F19" s="35" t="s">
-        <v>123</v>
-      </c>
-      <c r="G19" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="H19" s="48" t="s">
-        <v>87</v>
-      </c>
-      <c r="I19" s="38" t="s">
+    <row r="32" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" s="40" t="s">
+        <v>228</v>
+      </c>
+      <c r="D32" s="41" t="s">
         <v>129</v>
       </c>
-      <c r="J19" s="39" t="s">
+      <c r="E32" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="K19" s="47" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="B20" s="40" t="s">
-        <v>124</v>
-      </c>
-      <c r="C20" s="41" t="s">
-        <v>125</v>
-      </c>
-      <c r="D20" s="42" t="s">
-        <v>126</v>
-      </c>
-      <c r="E20" s="41" t="s">
-        <v>127</v>
-      </c>
-      <c r="F20" s="43" t="s">
-        <v>128</v>
-      </c>
-      <c r="G20" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="H20" s="49" t="s">
+      <c r="F32" s="42" t="s">
+        <v>131</v>
+      </c>
+      <c r="G32" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H32" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I32" s="44" t="s">
+        <v>132</v>
+      </c>
+      <c r="J32" s="45" t="s">
+        <v>133</v>
+      </c>
+      <c r="K32" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B33" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="32" t="s">
+        <v>229</v>
+      </c>
+      <c r="D33" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="E33" s="32" t="s">
+        <v>136</v>
+      </c>
+      <c r="F33" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="G33" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H33" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="I20" s="45" t="s">
-        <v>131</v>
-      </c>
-      <c r="J20" s="46" t="s">
-        <v>132</v>
-      </c>
-      <c r="K20" s="36" t="s">
+      <c r="I33" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="J33" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="K33" s="35" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="72" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B34" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="C34" s="40" t="s">
+        <v>230</v>
+      </c>
+      <c r="D34" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="E34" s="40" t="s">
+        <v>141</v>
+      </c>
+      <c r="F34" s="42" t="s">
+        <v>142</v>
+      </c>
+      <c r="G34" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="H34" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="I34" s="44" t="s">
+        <v>143</v>
+      </c>
+      <c r="J34" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="K34" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="B35" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="C35" s="32" t="s">
+        <v>145</v>
+      </c>
+      <c r="D35" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="E35" s="32" t="s">
+        <v>136</v>
+      </c>
+      <c r="F35" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="G35" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H35" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="37" t="s">
+        <v>147</v>
+      </c>
+      <c r="J35" s="38" t="s">
+        <v>148</v>
+      </c>
+      <c r="K35" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="55" t="s">
+        <v>213</v>
+      </c>
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="25"/>
+      <c r="K36" s="25"/>
+    </row>
+    <row r="37" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="56" t="s">
+        <v>194</v>
+      </c>
+      <c r="B37" s="31" t="s">
+        <v>195</v>
+      </c>
+      <c r="C37" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="D37" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="E37" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="F37" s="34" t="s">
+        <v>199</v>
+      </c>
+      <c r="G37" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H37" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I37" s="37" t="s">
+        <v>200</v>
+      </c>
+      <c r="J37" s="38" t="s">
+        <v>201</v>
+      </c>
+      <c r="K37" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="56" t="s">
+        <v>194</v>
+      </c>
+      <c r="B38" s="39" t="s">
+        <v>202</v>
+      </c>
+      <c r="C38" s="40" t="s">
+        <v>232</v>
+      </c>
+      <c r="D38" s="41" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" s="42" t="s">
+        <v>181</v>
+      </c>
+      <c r="G38" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H38" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="I38" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="J38" s="45" t="s">
+        <v>233</v>
+      </c>
+      <c r="K38" s="43" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="56" t="s">
+        <v>194</v>
+      </c>
+      <c r="B39" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="C39" s="32" t="s">
+        <v>205</v>
+      </c>
+      <c r="D39" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F39" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="G39" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H39" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I39" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="J39" s="38" t="s">
+        <v>207</v>
+      </c>
+      <c r="K39" s="35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="56" t="s">
+        <v>194</v>
+      </c>
+      <c r="B40" s="39" t="s">
+        <v>208</v>
+      </c>
+      <c r="C40" s="40" t="s">
+        <v>209</v>
+      </c>
+      <c r="D40" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" s="40" t="s">
+        <v>210</v>
+      </c>
+      <c r="F40" s="42" t="s">
+        <v>211</v>
+      </c>
+      <c r="G40" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="H40" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="I40" s="44" t="s">
+        <v>212</v>
+      </c>
+      <c r="J40" s="45" t="s">
+        <v>234</v>
+      </c>
+      <c r="K40" s="46" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="8">
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A36:K36"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A2:K2"/>
@@ -1876,12 +4032,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
@@ -1889,12 +4045,13 @@
     <col min="6" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="27.6640625" customWidth="1"/>
     <col min="9" max="9" width="0.1640625" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="29" t="s">
-        <v>61</v>
+    <row r="1" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="28" t="s">
+        <v>296</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -1905,85 +4062,1115 @@
       <c r="H2" s="25"/>
       <c r="I2" s="25"/>
     </row>
-    <row r="3" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-    </row>
-    <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="82" t="s">
+        <v>297</v>
+      </c>
+      <c r="B3" s="83"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
+    </row>
+    <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="C4" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="E4" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="G4" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="23" t="s">
+    </row>
+    <row r="5" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="21" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="21" t="s">
+      <c r="B5" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="D5" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="F5" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="H5" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="8" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="10" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="13" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2"/>
+    </row>
+    <row r="6" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="73" t="s">
+        <v>298</v>
+      </c>
+      <c r="B6" s="74" t="s">
+        <v>299</v>
+      </c>
+      <c r="C6" s="75" t="s">
+        <v>315</v>
+      </c>
+      <c r="D6" s="74" t="s">
+        <v>316</v>
+      </c>
+      <c r="E6" s="74" t="s">
+        <v>300</v>
+      </c>
+      <c r="F6" s="74" t="s">
+        <v>301</v>
+      </c>
+      <c r="G6" s="74" t="s">
+        <v>302</v>
+      </c>
+      <c r="H6" s="74" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="76" t="s">
+        <v>304</v>
+      </c>
+      <c r="B7" s="77" t="s">
+        <v>305</v>
+      </c>
+      <c r="C7" s="78" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="77" t="s">
+        <v>317</v>
+      </c>
+      <c r="E7" s="77" t="s">
+        <v>306</v>
+      </c>
+      <c r="F7" s="77" t="s">
+        <v>301</v>
+      </c>
+      <c r="G7" s="77" t="s">
+        <v>307</v>
+      </c>
+      <c r="H7" s="77" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="79" t="s">
+        <v>309</v>
+      </c>
+      <c r="B8" s="74" t="s">
+        <v>310</v>
+      </c>
+      <c r="C8" s="80" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="74" t="s">
+        <v>318</v>
+      </c>
+      <c r="E8" s="74" t="s">
+        <v>311</v>
+      </c>
+      <c r="F8" s="74" t="s">
+        <v>312</v>
+      </c>
+      <c r="G8" s="74" t="s">
+        <v>313</v>
+      </c>
+      <c r="H8" s="74" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="89" t="s">
+        <v>321</v>
+      </c>
+      <c r="B10" s="90"/>
+      <c r="C10" s="90"/>
+      <c r="D10" s="90"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="90"/>
+      <c r="G10" s="90"/>
+      <c r="H10" s="90"/>
+      <c r="I10" s="90"/>
+      <c r="J10" s="91"/>
+    </row>
+    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="88" t="s">
+        <v>322</v>
+      </c>
+      <c r="B11" s="88" t="s">
+        <v>323</v>
+      </c>
+      <c r="C11" s="88" t="s">
+        <v>324</v>
+      </c>
+      <c r="D11" s="88" t="s">
+        <v>325</v>
+      </c>
+      <c r="E11" s="88" t="s">
+        <v>326</v>
+      </c>
+      <c r="F11" s="88" t="s">
+        <v>327</v>
+      </c>
+      <c r="G11" s="88" t="s">
+        <v>328</v>
+      </c>
+      <c r="H11" s="88" t="s">
+        <v>329</v>
+      </c>
+      <c r="I11" s="88" t="s">
+        <v>330</v>
+      </c>
+      <c r="J11" s="88" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="84" t="s">
+        <v>331</v>
+      </c>
+      <c r="B12" s="77" t="s">
+        <v>363</v>
+      </c>
+      <c r="C12" s="77" t="s">
+        <v>332</v>
+      </c>
+      <c r="D12" s="77" t="s">
+        <v>333</v>
+      </c>
+      <c r="E12" s="77" t="s">
+        <v>334</v>
+      </c>
+      <c r="F12" s="77" t="s">
+        <v>335</v>
+      </c>
+      <c r="G12" s="77" t="s">
+        <v>336</v>
+      </c>
+      <c r="H12" s="77" t="s">
+        <v>337</v>
+      </c>
+      <c r="I12" s="77" t="s">
+        <v>338</v>
+      </c>
+      <c r="J12" s="77" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="85" t="s">
+        <v>339</v>
+      </c>
+      <c r="B13" s="74" t="s">
+        <v>364</v>
+      </c>
+      <c r="C13" s="74" t="s">
+        <v>340</v>
+      </c>
+      <c r="D13" s="74" t="s">
+        <v>341</v>
+      </c>
+      <c r="E13" s="74" t="s">
+        <v>342</v>
+      </c>
+      <c r="F13" s="74" t="s">
+        <v>343</v>
+      </c>
+      <c r="G13" s="74" t="s">
+        <v>344</v>
+      </c>
+      <c r="H13" s="74" t="s">
+        <v>345</v>
+      </c>
+      <c r="I13" s="74" t="s">
+        <v>346</v>
+      </c>
+      <c r="J13" s="74" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="86" t="s">
+        <v>347</v>
+      </c>
+      <c r="B14" s="77" t="s">
+        <v>365</v>
+      </c>
+      <c r="C14" s="77" t="s">
+        <v>348</v>
+      </c>
+      <c r="D14" s="77" t="s">
+        <v>349</v>
+      </c>
+      <c r="E14" s="77" t="s">
+        <v>350</v>
+      </c>
+      <c r="F14" s="77" t="s">
+        <v>351</v>
+      </c>
+      <c r="G14" s="77" t="s">
+        <v>352</v>
+      </c>
+      <c r="H14" s="77" t="s">
+        <v>353</v>
+      </c>
+      <c r="I14" s="77" t="s">
+        <v>354</v>
+      </c>
+      <c r="J14" s="77" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="87" t="s">
+        <v>355</v>
+      </c>
+      <c r="B15" s="74" t="s">
+        <v>366</v>
+      </c>
+      <c r="C15" s="74" t="s">
+        <v>356</v>
+      </c>
+      <c r="D15" s="74" t="s">
+        <v>357</v>
+      </c>
+      <c r="E15" s="74" t="s">
+        <v>358</v>
+      </c>
+      <c r="F15" s="74" t="s">
+        <v>359</v>
+      </c>
+      <c r="G15" s="74" t="s">
+        <v>360</v>
+      </c>
+      <c r="H15" s="74" t="s">
+        <v>361</v>
+      </c>
+      <c r="I15" s="74" t="s">
+        <v>362</v>
+      </c>
+      <c r="J15" s="74" t="s">
+        <v>362</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A10:I10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D072851C-E33D-3E4C-9E1E-B705D90C883D}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="21.83203125" customWidth="1"/>
+    <col min="5" max="5" width="39" customWidth="1"/>
+    <col min="6" max="6" width="28.5" customWidth="1"/>
+    <col min="7" max="7" width="24.5" customWidth="1"/>
+    <col min="8" max="8" width="38" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="95" t="s">
+        <v>405</v>
+      </c>
+      <c r="B2" s="96"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="89" t="s">
+        <v>406</v>
+      </c>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="88" t="s">
+        <v>367</v>
+      </c>
+      <c r="B4" s="88" t="s">
+        <v>368</v>
+      </c>
+      <c r="C4" s="88" t="s">
+        <v>369</v>
+      </c>
+      <c r="D4" s="88" t="s">
+        <v>370</v>
+      </c>
+      <c r="E4" s="88" t="s">
+        <v>371</v>
+      </c>
+      <c r="F4" s="88" t="s">
+        <v>372</v>
+      </c>
+      <c r="G4" s="88" t="s">
+        <v>373</v>
+      </c>
+      <c r="H4" s="88" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="92" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="77" t="s">
+        <v>375</v>
+      </c>
+      <c r="C5" s="77" t="s">
+        <v>376</v>
+      </c>
+      <c r="D5" s="77" t="s">
+        <v>404</v>
+      </c>
+      <c r="E5" s="77" t="s">
+        <v>377</v>
+      </c>
+      <c r="F5" s="77" t="s">
+        <v>378</v>
+      </c>
+      <c r="G5" s="93" t="s">
+        <v>379</v>
+      </c>
+      <c r="H5" s="80" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="71" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="94" t="s">
+        <v>380</v>
+      </c>
+      <c r="B6" s="74" t="s">
+        <v>381</v>
+      </c>
+      <c r="C6" s="74" t="s">
+        <v>382</v>
+      </c>
+      <c r="D6" s="74" t="s">
+        <v>408</v>
+      </c>
+      <c r="E6" s="74" t="s">
+        <v>383</v>
+      </c>
+      <c r="F6" s="74" t="s">
+        <v>384</v>
+      </c>
+      <c r="G6" s="93" t="s">
+        <v>385</v>
+      </c>
+      <c r="H6" s="80" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="92" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="77" t="s">
+        <v>387</v>
+      </c>
+      <c r="C7" s="77" t="s">
+        <v>388</v>
+      </c>
+      <c r="D7" s="77" t="s">
+        <v>409</v>
+      </c>
+      <c r="E7" s="77" t="s">
+        <v>389</v>
+      </c>
+      <c r="F7" s="77" t="s">
+        <v>390</v>
+      </c>
+      <c r="G7" s="93" t="s">
+        <v>391</v>
+      </c>
+      <c r="H7" s="80" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="94" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" s="74" t="s">
+        <v>410</v>
+      </c>
+      <c r="C8" s="74" t="s">
+        <v>393</v>
+      </c>
+      <c r="D8" s="74" t="s">
+        <v>411</v>
+      </c>
+      <c r="E8" s="74" t="s">
+        <v>394</v>
+      </c>
+      <c r="F8" s="74" t="s">
+        <v>395</v>
+      </c>
+      <c r="G8" s="93" t="s">
+        <v>396</v>
+      </c>
+      <c r="H8" s="80" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="92" t="s">
+        <v>398</v>
+      </c>
+      <c r="B9" s="77" t="s">
+        <v>399</v>
+      </c>
+      <c r="C9" s="77" t="s">
+        <v>382</v>
+      </c>
+      <c r="D9" s="77" t="s">
+        <v>412</v>
+      </c>
+      <c r="E9" s="77" t="s">
+        <v>400</v>
+      </c>
+      <c r="F9" s="77" t="s">
+        <v>401</v>
+      </c>
+      <c r="G9" s="93" t="s">
+        <v>402</v>
+      </c>
+      <c r="H9" s="80" t="s">
+        <v>403</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9578EDDF-5D6A-9145-9892-C45CF7563863}">
+  <dimension ref="A1:G46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="57" t="s">
+        <v>291</v>
+      </c>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="58" t="s">
+        <v>237</v>
+      </c>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="63" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="60" t="s">
+        <v>238</v>
+      </c>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="64" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="60" t="s">
+        <v>239</v>
+      </c>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="65" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="60" t="s">
+        <v>240</v>
+      </c>
+      <c r="C7" s="59"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="66" t="s">
+        <v>150</v>
+      </c>
+      <c r="B8" s="60" t="s">
+        <v>241</v>
+      </c>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="67" t="s">
+        <v>175</v>
+      </c>
+      <c r="B9" s="60" t="s">
+        <v>242</v>
+      </c>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="68" t="s">
+        <v>194</v>
+      </c>
+      <c r="B10" s="60" t="s">
+        <v>243</v>
+      </c>
+      <c r="C10" s="59"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="59"/>
+      <c r="G10" s="59"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="58" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="63" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="60" t="s">
+        <v>245</v>
+      </c>
+      <c r="C13" s="59"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="59"/>
+    </row>
+    <row r="14" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="69" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="60" t="s">
+        <v>246</v>
+      </c>
+      <c r="C14" s="59"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
+      <c r="G14" s="59"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="70" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="60" t="s">
+        <v>247</v>
+      </c>
+      <c r="C15" s="59"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="59"/>
+      <c r="G15" s="59"/>
+    </row>
+    <row r="16" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="71" t="s">
+        <v>248</v>
+      </c>
+      <c r="B16" s="60" t="s">
+        <v>249</v>
+      </c>
+      <c r="C16" s="59"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="59"/>
+      <c r="G16" s="59"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="58" t="s">
+        <v>250</v>
+      </c>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="70" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="60" t="s">
+        <v>292</v>
+      </c>
+      <c r="C19" s="59"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="59"/>
+      <c r="F19" s="59"/>
+      <c r="G19" s="59"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="69" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="60" t="s">
+        <v>251</v>
+      </c>
+      <c r="C20" s="59"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="71" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="59"/>
+      <c r="G21" s="59"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="58" t="s">
+        <v>253</v>
+      </c>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="71" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="60" t="s">
+        <v>293</v>
+      </c>
+      <c r="C24" s="59"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="59"/>
+      <c r="G24" s="59"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="70" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="60" t="s">
+        <v>294</v>
+      </c>
+      <c r="C25" s="59"/>
+      <c r="D25" s="59"/>
+      <c r="E25" s="59"/>
+      <c r="F25" s="59"/>
+      <c r="G25" s="59"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="69" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="60" t="s">
+        <v>295</v>
+      </c>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="59"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="58" t="s">
+        <v>254</v>
+      </c>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="72" t="s">
+        <v>255</v>
+      </c>
+      <c r="B29" s="61" t="s">
+        <v>256</v>
+      </c>
+      <c r="C29" s="59"/>
+      <c r="D29" s="59"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="59"/>
+      <c r="G29" s="59"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="72" t="s">
+        <v>257</v>
+      </c>
+      <c r="B30" s="61" t="s">
+        <v>258</v>
+      </c>
+      <c r="C30" s="59"/>
+      <c r="D30" s="59"/>
+      <c r="E30" s="59"/>
+      <c r="F30" s="59"/>
+      <c r="G30" s="59"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="72" t="s">
+        <v>259</v>
+      </c>
+      <c r="B31" s="61" t="s">
+        <v>260</v>
+      </c>
+      <c r="C31" s="59"/>
+      <c r="D31" s="59"/>
+      <c r="E31" s="59"/>
+      <c r="F31" s="59"/>
+      <c r="G31" s="59"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="72" t="s">
+        <v>261</v>
+      </c>
+      <c r="B32" s="61" t="s">
+        <v>262</v>
+      </c>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="59"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="72" t="s">
+        <v>263</v>
+      </c>
+      <c r="B33" s="61" t="s">
+        <v>264</v>
+      </c>
+      <c r="C33" s="59"/>
+      <c r="D33" s="59"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="59"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="72" t="s">
+        <v>265</v>
+      </c>
+      <c r="B34" s="61" t="s">
+        <v>266</v>
+      </c>
+      <c r="C34" s="59"/>
+      <c r="D34" s="59"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="59"/>
+      <c r="G34" s="59"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="72" t="s">
+        <v>267</v>
+      </c>
+      <c r="B35" s="61" t="s">
+        <v>268</v>
+      </c>
+      <c r="C35" s="59"/>
+      <c r="D35" s="59"/>
+      <c r="E35" s="59"/>
+      <c r="F35" s="59"/>
+      <c r="G35" s="59"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="72" t="s">
+        <v>269</v>
+      </c>
+      <c r="B36" s="61" t="s">
+        <v>270</v>
+      </c>
+      <c r="C36" s="59"/>
+      <c r="D36" s="59"/>
+      <c r="E36" s="59"/>
+      <c r="F36" s="59"/>
+      <c r="G36" s="59"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="72" t="s">
+        <v>271</v>
+      </c>
+      <c r="B37" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="C37" s="59"/>
+      <c r="D37" s="59"/>
+      <c r="E37" s="59"/>
+      <c r="F37" s="59"/>
+      <c r="G37" s="59"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="72" t="s">
+        <v>273</v>
+      </c>
+      <c r="B38" s="61" t="s">
+        <v>274</v>
+      </c>
+      <c r="C38" s="59"/>
+      <c r="D38" s="59"/>
+      <c r="E38" s="59"/>
+      <c r="F38" s="59"/>
+      <c r="G38" s="59"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="72" t="s">
+        <v>275</v>
+      </c>
+      <c r="B39" s="61" t="s">
+        <v>276</v>
+      </c>
+      <c r="C39" s="59"/>
+      <c r="D39" s="59"/>
+      <c r="E39" s="59"/>
+      <c r="F39" s="59"/>
+      <c r="G39" s="59"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="72" t="s">
+        <v>277</v>
+      </c>
+      <c r="B40" s="61" t="s">
+        <v>278</v>
+      </c>
+      <c r="C40" s="59"/>
+      <c r="D40" s="59"/>
+      <c r="E40" s="59"/>
+      <c r="F40" s="59"/>
+      <c r="G40" s="59"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="72" t="s">
+        <v>279</v>
+      </c>
+      <c r="B41" s="61" t="s">
+        <v>280</v>
+      </c>
+      <c r="C41" s="59"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="59"/>
+      <c r="F41" s="59"/>
+      <c r="G41" s="59"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="B42" s="61" t="s">
+        <v>282</v>
+      </c>
+      <c r="C42" s="59"/>
+      <c r="D42" s="59"/>
+      <c r="E42" s="59"/>
+      <c r="F42" s="59"/>
+      <c r="G42" s="59"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="72" t="s">
+        <v>283</v>
+      </c>
+      <c r="B43" s="61" t="s">
+        <v>284</v>
+      </c>
+      <c r="C43" s="59"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="59"/>
+      <c r="F43" s="59"/>
+      <c r="G43" s="59"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="72" t="s">
+        <v>285</v>
+      </c>
+      <c r="B44" s="61" t="s">
+        <v>286</v>
+      </c>
+      <c r="C44" s="59"/>
+      <c r="D44" s="59"/>
+      <c r="E44" s="59"/>
+      <c r="F44" s="59"/>
+      <c r="G44" s="59"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="72" t="s">
+        <v>287</v>
+      </c>
+      <c r="B45" s="61" t="s">
+        <v>288</v>
+      </c>
+      <c r="C45" s="59"/>
+      <c r="D45" s="59"/>
+      <c r="E45" s="59"/>
+      <c r="F45" s="59"/>
+      <c r="G45" s="59"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="72" t="s">
+        <v>289</v>
+      </c>
+      <c r="B46" s="61" t="s">
+        <v>290</v>
+      </c>
+      <c r="C46" s="59"/>
+      <c r="D46" s="59"/>
+      <c r="E46" s="59"/>
+      <c r="F46" s="59"/>
+      <c r="G46" s="59"/>
+    </row>
+  </sheetData>
+  <mergeCells count="40">
+    <mergeCell ref="B43:G43"/>
+    <mergeCell ref="B44:G44"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B46:G46"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B33:G33"/>
+    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added more recommendations to Gap analysis sheet
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33965CD0-53FF-7941-9B2F-435832F3C15D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CF56B6-EEC7-6C4A-9F23-25A227757FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="463">
   <si>
     <t>CSCRF
 Function</t>
@@ -1537,6 +1537,114 @@
   </si>
   <si>
     <t>LinkedIn: https://www.linkedin.com/in/nilisha-wandile/</t>
+  </si>
+  <si>
+    <t>CIS Control</t>
+  </si>
+  <si>
+    <t>CIS Safeguard</t>
+  </si>
+  <si>
+    <t>Why It Matters for Indian BFSI</t>
+  </si>
+  <si>
+    <t>CSCRF Status</t>
+  </si>
+  <si>
+    <t>Recommendation</t>
+  </si>
+  <si>
+    <t>IG Level</t>
+  </si>
+  <si>
+    <t>Estimated Effort</t>
+  </si>
+  <si>
+    <t>Business Value</t>
+  </si>
+  <si>
+    <t>CIS 9</t>
+  </si>
+  <si>
+    <t>Email &amp; Web Browser Protections (9.1–9.7)</t>
+  </si>
+  <si>
+    <t>BFSI is a top phishing target. DMARC/DKIM/SPF + browser isolation provides critical protection against Business Email Compromise (BEC) and credential theft.</t>
+  </si>
+  <si>
+    <t>Not addressed in CSCRF</t>
+  </si>
+  <si>
+    <t>Implement DMARC (enforcement), DKIM, SPF for all email domains. Deploy email security gateway with sandboxing. Consider browser isolation for trading staff.</t>
+  </si>
+  <si>
+    <t>Low–Medium</t>
+  </si>
+  <si>
+    <t>Reduces phishing success rate significantly; protects broker trading credentials</t>
+  </si>
+  <si>
+    <t>CIS 10.5</t>
+  </si>
+  <si>
+    <t>Anti-Exploitation Features (DEP/ASLR)</t>
+  </si>
+  <si>
+    <t>Algo trading terminals and OMS platforms are high-value targets for exploitation. Memory protection features reduce attack surface.</t>
+  </si>
+  <si>
+    <t>Partially implied under PR.PS but not specific</t>
+  </si>
+  <si>
+    <t>Enable DEP, ASLR, and Control Flow Guard on all trading terminals, OMS servers, and risk management systems. Validate via config baseline audit.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Reduces exploitation risk on high-value financial infrastructure</t>
+  </si>
+  <si>
+    <t>CIS 4.6</t>
+  </si>
+  <si>
+    <t>Unencrypted Sensitive Data Discovery</t>
+  </si>
+  <si>
+    <t>UPSI and client financial data inadvertently stored unencrypted poses insider threat and breach risk under SEBI PIT Regulations.</t>
+  </si>
+  <si>
+    <t>Not explicitly in CSCRF</t>
+  </si>
+  <si>
+    <t>Deploy automated sensitive data discovery tool (e.g., Varonis, Spirion) to scan file systems, shares, and endpoints for unencrypted UPSI/PAN/financial data.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Critical for UPSI protection; reduces PIT Regulation exposure; investor data breach risk</t>
+  </si>
+  <si>
+    <t>CIS 14.5</t>
+  </si>
+  <si>
+    <t>Train Workforce on Causes of Unintended Exposure</t>
+  </si>
+  <si>
+    <t>Insider threat (intentional and accidental) is particularly relevant in capital markets for UPSI mishandling.</t>
+  </si>
+  <si>
+    <t>Add dedicated insider threat awareness module to annual training programme. Include UPSI handling, data classification responsibilities, and whistleblower processes.</t>
+  </si>
+  <si>
+    <t>Reduces UPSI leakage risk; strengthens SEBI PIT compliance culture</t>
+  </si>
+  <si>
+    <t>SECTION B - CIS Controls That Exceed CSCRF (Global Best Practice - Recommended)</t>
+  </si>
+  <si>
+    <t>CSCRF covers general awareness - not insider threat specifically</t>
   </si>
 </sst>
 </file>
@@ -4391,7 +4499,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D072851C-E33D-3E4C-9E1E-B705D90C883D}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -4594,10 +4702,153 @@
         <v>403</v>
       </c>
     </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="89" t="s">
+        <v>461</v>
+      </c>
+      <c r="B12" s="90"/>
+      <c r="C12" s="90"/>
+      <c r="D12" s="90"/>
+      <c r="E12" s="90"/>
+      <c r="F12" s="90"/>
+      <c r="G12" s="90"/>
+      <c r="H12" s="90"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="88" t="s">
+        <v>427</v>
+      </c>
+      <c r="B13" s="88" t="s">
+        <v>428</v>
+      </c>
+      <c r="C13" s="88" t="s">
+        <v>429</v>
+      </c>
+      <c r="D13" s="88" t="s">
+        <v>430</v>
+      </c>
+      <c r="E13" s="88" t="s">
+        <v>431</v>
+      </c>
+      <c r="F13" s="88" t="s">
+        <v>432</v>
+      </c>
+      <c r="G13" s="88" t="s">
+        <v>433</v>
+      </c>
+      <c r="H13" s="88" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="78" x14ac:dyDescent="0.2">
+      <c r="A14" s="92" t="s">
+        <v>435</v>
+      </c>
+      <c r="B14" s="77" t="s">
+        <v>436</v>
+      </c>
+      <c r="C14" s="77" t="s">
+        <v>437</v>
+      </c>
+      <c r="D14" s="77" t="s">
+        <v>438</v>
+      </c>
+      <c r="E14" s="77" t="s">
+        <v>439</v>
+      </c>
+      <c r="F14" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="H14" s="77" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="52" x14ac:dyDescent="0.2">
+      <c r="A15" s="94" t="s">
+        <v>442</v>
+      </c>
+      <c r="B15" s="74" t="s">
+        <v>443</v>
+      </c>
+      <c r="C15" s="74" t="s">
+        <v>444</v>
+      </c>
+      <c r="D15" s="74" t="s">
+        <v>445</v>
+      </c>
+      <c r="E15" s="74" t="s">
+        <v>446</v>
+      </c>
+      <c r="F15" s="74" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="74" t="s">
+        <v>447</v>
+      </c>
+      <c r="H15" s="74" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="52" x14ac:dyDescent="0.2">
+      <c r="A16" s="92" t="s">
+        <v>449</v>
+      </c>
+      <c r="B16" s="77" t="s">
+        <v>450</v>
+      </c>
+      <c r="C16" s="77" t="s">
+        <v>451</v>
+      </c>
+      <c r="D16" s="77" t="s">
+        <v>452</v>
+      </c>
+      <c r="E16" s="77" t="s">
+        <v>453</v>
+      </c>
+      <c r="F16" s="77" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="77" t="s">
+        <v>454</v>
+      </c>
+      <c r="H16" s="77" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="52" x14ac:dyDescent="0.2">
+      <c r="A17" s="94" t="s">
+        <v>456</v>
+      </c>
+      <c r="B17" s="74" t="s">
+        <v>457</v>
+      </c>
+      <c r="C17" s="74" t="s">
+        <v>458</v>
+      </c>
+      <c r="D17" s="74" t="s">
+        <v>462</v>
+      </c>
+      <c r="E17" s="74" t="s">
+        <v>459</v>
+      </c>
+      <c r="F17" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="74" t="s">
+        <v>447</v>
+      </c>
+      <c r="H17" s="74" t="s">
+        <v>460</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A12:H12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed Implementation Roadmap completion dates
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CF56B6-EEC7-6C4A-9F23-25A227757FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E06E2CF-9E18-FE42-B461-9EB1EA4942D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="8" r:id="rId1"/>
@@ -1078,10 +1078,6 @@
 • CERT-In reporting workflow</t>
   </si>
   <si>
-    <t>Year 1 baseline by Jan 2025
-Year 2 by Dec 2025</t>
-  </si>
-  <si>
     <t>Mid-Size Regulated Entities</t>
   </si>
   <si>
@@ -1645,6 +1641,10 @@
   </si>
   <si>
     <t>CSCRF covers general awareness - not insider threat specifically</t>
+  </si>
+  <si>
+    <t>Year 1 baseline by Q1
+Year 2 Jan every year</t>
   </si>
 </sst>
 </file>
@@ -2745,7 +2745,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="62" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B10" s="62"/>
       <c r="C10" s="62"/>
@@ -2755,11 +2755,11 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="62" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B11" s="62"/>
       <c r="C11" s="62" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D11" s="62"/>
       <c r="E11" s="62"/>
@@ -2767,7 +2767,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="102" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B14" s="81"/>
       <c r="C14" s="81"/>
@@ -2783,12 +2783,12 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="97" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B15" s="98"/>
       <c r="C15" s="98"/>
       <c r="D15" s="101" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E15" s="98"/>
       <c r="F15" s="98"/>
@@ -2801,12 +2801,12 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="99" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B16" s="100"/>
       <c r="C16" s="100"/>
       <c r="D16" s="61" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E16" s="100"/>
       <c r="F16" s="100"/>
@@ -2819,12 +2819,12 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="97" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B17" s="98"/>
       <c r="C17" s="98"/>
       <c r="D17" s="101" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E17" s="98"/>
       <c r="F17" s="98"/>
@@ -2837,12 +2837,12 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="99" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B18" s="100"/>
       <c r="C18" s="100"/>
       <c r="D18" s="61" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E18" s="100"/>
       <c r="F18" s="100"/>
@@ -2855,12 +2855,12 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="97" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B19" s="98"/>
       <c r="C19" s="98"/>
       <c r="D19" s="101" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E19" s="98"/>
       <c r="F19" s="98"/>
@@ -3277,7 +3277,7 @@
         <v>32</v>
       </c>
       <c r="F14" s="42" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G14" s="43" t="s">
         <v>26</v>
@@ -3622,7 +3622,7 @@
         <v>15</v>
       </c>
       <c r="F25" s="42" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G25" s="43" t="s">
         <v>26</v>
@@ -4156,7 +4156,16 @@
     <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
     <row r="2" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="28" t="s">
         <v>296</v>
@@ -4243,10 +4252,10 @@
         <v>299</v>
       </c>
       <c r="C6" s="75" t="s">
+        <v>314</v>
+      </c>
+      <c r="D6" s="74" t="s">
         <v>315</v>
-      </c>
-      <c r="D6" s="74" t="s">
-        <v>316</v>
       </c>
       <c r="E6" s="74" t="s">
         <v>300</v>
@@ -4258,64 +4267,64 @@
         <v>302</v>
       </c>
       <c r="H6" s="74" t="s">
-        <v>303</v>
+        <v>462</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="76" t="s">
+        <v>303</v>
+      </c>
+      <c r="B7" s="77" t="s">
         <v>304</v>
-      </c>
-      <c r="B7" s="77" t="s">
-        <v>305</v>
       </c>
       <c r="C7" s="78" t="s">
         <v>26</v>
       </c>
       <c r="D7" s="77" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E7" s="77" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F7" s="77" t="s">
         <v>301</v>
       </c>
       <c r="G7" s="77" t="s">
+        <v>306</v>
+      </c>
+      <c r="H7" s="77" t="s">
         <v>307</v>
-      </c>
-      <c r="H7" s="77" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="79" t="s">
+        <v>308</v>
+      </c>
+      <c r="B8" s="74" t="s">
         <v>309</v>
-      </c>
-      <c r="B8" s="74" t="s">
-        <v>310</v>
       </c>
       <c r="C8" s="80" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="74" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E8" s="74" t="s">
+        <v>310</v>
+      </c>
+      <c r="F8" s="74" t="s">
         <v>311</v>
       </c>
-      <c r="F8" s="74" t="s">
+      <c r="G8" s="74" t="s">
         <v>312</v>
       </c>
-      <c r="G8" s="74" t="s">
+      <c r="H8" s="74" t="s">
         <v>313</v>
-      </c>
-      <c r="H8" s="74" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="89" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B10" s="90"/>
       <c r="C10" s="90"/>
@@ -4329,162 +4338,162 @@
     </row>
     <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="88" t="s">
+        <v>321</v>
+      </c>
+      <c r="B11" s="88" t="s">
         <v>322</v>
       </c>
-      <c r="B11" s="88" t="s">
+      <c r="C11" s="88" t="s">
         <v>323</v>
       </c>
-      <c r="C11" s="88" t="s">
+      <c r="D11" s="88" t="s">
         <v>324</v>
       </c>
-      <c r="D11" s="88" t="s">
+      <c r="E11" s="88" t="s">
         <v>325</v>
       </c>
-      <c r="E11" s="88" t="s">
+      <c r="F11" s="88" t="s">
         <v>326</v>
       </c>
-      <c r="F11" s="88" t="s">
+      <c r="G11" s="88" t="s">
         <v>327</v>
       </c>
-      <c r="G11" s="88" t="s">
+      <c r="H11" s="88" t="s">
         <v>328</v>
       </c>
-      <c r="H11" s="88" t="s">
+      <c r="I11" s="88" t="s">
         <v>329</v>
       </c>
-      <c r="I11" s="88" t="s">
-        <v>330</v>
-      </c>
       <c r="J11" s="88" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="84" t="s">
+        <v>330</v>
+      </c>
+      <c r="B12" s="77" t="s">
+        <v>362</v>
+      </c>
+      <c r="C12" s="77" t="s">
         <v>331</v>
       </c>
-      <c r="B12" s="77" t="s">
-        <v>363</v>
-      </c>
-      <c r="C12" s="77" t="s">
+      <c r="D12" s="77" t="s">
         <v>332</v>
       </c>
-      <c r="D12" s="77" t="s">
+      <c r="E12" s="77" t="s">
         <v>333</v>
       </c>
-      <c r="E12" s="77" t="s">
+      <c r="F12" s="77" t="s">
         <v>334</v>
       </c>
-      <c r="F12" s="77" t="s">
+      <c r="G12" s="77" t="s">
         <v>335</v>
       </c>
-      <c r="G12" s="77" t="s">
+      <c r="H12" s="77" t="s">
         <v>336</v>
       </c>
-      <c r="H12" s="77" t="s">
+      <c r="I12" s="77" t="s">
         <v>337</v>
       </c>
-      <c r="I12" s="77" t="s">
-        <v>338</v>
-      </c>
       <c r="J12" s="77" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="85" t="s">
+        <v>338</v>
+      </c>
+      <c r="B13" s="74" t="s">
+        <v>363</v>
+      </c>
+      <c r="C13" s="74" t="s">
         <v>339</v>
       </c>
-      <c r="B13" s="74" t="s">
-        <v>364</v>
-      </c>
-      <c r="C13" s="74" t="s">
+      <c r="D13" s="74" t="s">
         <v>340</v>
       </c>
-      <c r="D13" s="74" t="s">
+      <c r="E13" s="74" t="s">
         <v>341</v>
       </c>
-      <c r="E13" s="74" t="s">
+      <c r="F13" s="74" t="s">
         <v>342</v>
       </c>
-      <c r="F13" s="74" t="s">
+      <c r="G13" s="74" t="s">
         <v>343</v>
       </c>
-      <c r="G13" s="74" t="s">
+      <c r="H13" s="74" t="s">
         <v>344</v>
       </c>
-      <c r="H13" s="74" t="s">
+      <c r="I13" s="74" t="s">
         <v>345</v>
       </c>
-      <c r="I13" s="74" t="s">
-        <v>346</v>
-      </c>
       <c r="J13" s="74" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="86" t="s">
+        <v>346</v>
+      </c>
+      <c r="B14" s="77" t="s">
+        <v>364</v>
+      </c>
+      <c r="C14" s="77" t="s">
         <v>347</v>
       </c>
-      <c r="B14" s="77" t="s">
-        <v>365</v>
-      </c>
-      <c r="C14" s="77" t="s">
+      <c r="D14" s="77" t="s">
         <v>348</v>
       </c>
-      <c r="D14" s="77" t="s">
+      <c r="E14" s="77" t="s">
         <v>349</v>
       </c>
-      <c r="E14" s="77" t="s">
+      <c r="F14" s="77" t="s">
         <v>350</v>
       </c>
-      <c r="F14" s="77" t="s">
+      <c r="G14" s="77" t="s">
         <v>351</v>
       </c>
-      <c r="G14" s="77" t="s">
+      <c r="H14" s="77" t="s">
         <v>352</v>
       </c>
-      <c r="H14" s="77" t="s">
+      <c r="I14" s="77" t="s">
         <v>353</v>
       </c>
-      <c r="I14" s="77" t="s">
-        <v>354</v>
-      </c>
       <c r="J14" s="77" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="87" t="s">
+        <v>354</v>
+      </c>
+      <c r="B15" s="74" t="s">
+        <v>365</v>
+      </c>
+      <c r="C15" s="74" t="s">
         <v>355</v>
       </c>
-      <c r="B15" s="74" t="s">
-        <v>366</v>
-      </c>
-      <c r="C15" s="74" t="s">
+      <c r="D15" s="74" t="s">
         <v>356</v>
       </c>
-      <c r="D15" s="74" t="s">
+      <c r="E15" s="74" t="s">
         <v>357</v>
       </c>
-      <c r="E15" s="74" t="s">
+      <c r="F15" s="74" t="s">
         <v>358</v>
       </c>
-      <c r="F15" s="74" t="s">
+      <c r="G15" s="74" t="s">
         <v>359</v>
       </c>
-      <c r="G15" s="74" t="s">
+      <c r="H15" s="74" t="s">
         <v>360</v>
       </c>
-      <c r="H15" s="74" t="s">
+      <c r="I15" s="74" t="s">
         <v>361</v>
       </c>
-      <c r="I15" s="74" t="s">
-        <v>362</v>
-      </c>
       <c r="J15" s="74" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -4524,7 +4533,7 @@
     </row>
     <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="95" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B2" s="96"/>
       <c r="C2" s="96"/>
@@ -4536,7 +4545,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="89" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B3" s="90"/>
       <c r="C3" s="90"/>
@@ -4548,28 +4557,28 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="88" t="s">
+        <v>366</v>
+      </c>
+      <c r="B4" s="88" t="s">
         <v>367</v>
       </c>
-      <c r="B4" s="88" t="s">
+      <c r="C4" s="88" t="s">
         <v>368</v>
       </c>
-      <c r="C4" s="88" t="s">
+      <c r="D4" s="88" t="s">
         <v>369</v>
       </c>
-      <c r="D4" s="88" t="s">
+      <c r="E4" s="88" t="s">
         <v>370</v>
       </c>
-      <c r="E4" s="88" t="s">
+      <c r="F4" s="88" t="s">
         <v>371</v>
       </c>
-      <c r="F4" s="88" t="s">
+      <c r="G4" s="88" t="s">
         <v>372</v>
       </c>
-      <c r="G4" s="88" t="s">
+      <c r="H4" s="88" t="s">
         <v>373</v>
-      </c>
-      <c r="H4" s="88" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -4577,51 +4586,51 @@
         <v>77</v>
       </c>
       <c r="B5" s="77" t="s">
+        <v>374</v>
+      </c>
+      <c r="C5" s="77" t="s">
         <v>375</v>
       </c>
-      <c r="C5" s="77" t="s">
+      <c r="D5" s="77" t="s">
+        <v>403</v>
+      </c>
+      <c r="E5" s="77" t="s">
         <v>376</v>
       </c>
-      <c r="D5" s="77" t="s">
-        <v>404</v>
-      </c>
-      <c r="E5" s="77" t="s">
+      <c r="F5" s="77" t="s">
         <v>377</v>
       </c>
-      <c r="F5" s="77" t="s">
+      <c r="G5" s="93" t="s">
         <v>378</v>
       </c>
-      <c r="G5" s="93" t="s">
-        <v>379</v>
-      </c>
       <c r="H5" s="80" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="71" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="94" t="s">
+        <v>379</v>
+      </c>
+      <c r="B6" s="74" t="s">
         <v>380</v>
       </c>
-      <c r="B6" s="74" t="s">
+      <c r="C6" s="74" t="s">
         <v>381</v>
       </c>
-      <c r="C6" s="74" t="s">
+      <c r="D6" s="74" t="s">
+        <v>407</v>
+      </c>
+      <c r="E6" s="74" t="s">
         <v>382</v>
       </c>
-      <c r="D6" s="74" t="s">
-        <v>408</v>
-      </c>
-      <c r="E6" s="74" t="s">
+      <c r="F6" s="74" t="s">
         <v>383</v>
       </c>
-      <c r="F6" s="74" t="s">
+      <c r="G6" s="93" t="s">
         <v>384</v>
       </c>
-      <c r="G6" s="93" t="s">
+      <c r="H6" s="80" t="s">
         <v>385</v>
-      </c>
-      <c r="H6" s="80" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4629,25 +4638,25 @@
         <v>140</v>
       </c>
       <c r="B7" s="77" t="s">
+        <v>386</v>
+      </c>
+      <c r="C7" s="77" t="s">
         <v>387</v>
       </c>
-      <c r="C7" s="77" t="s">
+      <c r="D7" s="77" t="s">
+        <v>408</v>
+      </c>
+      <c r="E7" s="77" t="s">
         <v>388</v>
       </c>
-      <c r="D7" s="77" t="s">
-        <v>409</v>
-      </c>
-      <c r="E7" s="77" t="s">
+      <c r="F7" s="77" t="s">
         <v>389</v>
       </c>
-      <c r="F7" s="77" t="s">
+      <c r="G7" s="93" t="s">
         <v>390</v>
       </c>
-      <c r="G7" s="93" t="s">
+      <c r="H7" s="80" t="s">
         <v>391</v>
-      </c>
-      <c r="H7" s="80" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -4655,56 +4664,56 @@
         <v>164</v>
       </c>
       <c r="B8" s="74" t="s">
+        <v>409</v>
+      </c>
+      <c r="C8" s="74" t="s">
+        <v>392</v>
+      </c>
+      <c r="D8" s="74" t="s">
         <v>410</v>
       </c>
-      <c r="C8" s="74" t="s">
+      <c r="E8" s="74" t="s">
         <v>393</v>
       </c>
-      <c r="D8" s="74" t="s">
-        <v>411</v>
-      </c>
-      <c r="E8" s="74" t="s">
+      <c r="F8" s="74" t="s">
         <v>394</v>
       </c>
-      <c r="F8" s="74" t="s">
+      <c r="G8" s="93" t="s">
         <v>395</v>
       </c>
-      <c r="G8" s="93" t="s">
+      <c r="H8" s="80" t="s">
         <v>396</v>
-      </c>
-      <c r="H8" s="80" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="92" t="s">
+        <v>397</v>
+      </c>
+      <c r="B9" s="77" t="s">
         <v>398</v>
       </c>
-      <c r="B9" s="77" t="s">
+      <c r="C9" s="77" t="s">
+        <v>381</v>
+      </c>
+      <c r="D9" s="77" t="s">
+        <v>411</v>
+      </c>
+      <c r="E9" s="77" t="s">
         <v>399</v>
       </c>
-      <c r="C9" s="77" t="s">
-        <v>382</v>
-      </c>
-      <c r="D9" s="77" t="s">
-        <v>412</v>
-      </c>
-      <c r="E9" s="77" t="s">
+      <c r="F9" s="77" t="s">
         <v>400</v>
       </c>
-      <c r="F9" s="77" t="s">
+      <c r="G9" s="93" t="s">
         <v>401</v>
       </c>
-      <c r="G9" s="93" t="s">
+      <c r="H9" s="80" t="s">
         <v>402</v>
-      </c>
-      <c r="H9" s="80" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="89" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B12" s="90"/>
       <c r="C12" s="90"/>
@@ -4716,132 +4725,132 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="88" t="s">
+        <v>426</v>
+      </c>
+      <c r="B13" s="88" t="s">
         <v>427</v>
       </c>
-      <c r="B13" s="88" t="s">
+      <c r="C13" s="88" t="s">
         <v>428</v>
       </c>
-      <c r="C13" s="88" t="s">
+      <c r="D13" s="88" t="s">
         <v>429</v>
       </c>
-      <c r="D13" s="88" t="s">
+      <c r="E13" s="88" t="s">
         <v>430</v>
       </c>
-      <c r="E13" s="88" t="s">
+      <c r="F13" s="88" t="s">
         <v>431</v>
       </c>
-      <c r="F13" s="88" t="s">
+      <c r="G13" s="88" t="s">
         <v>432</v>
       </c>
-      <c r="G13" s="88" t="s">
+      <c r="H13" s="88" t="s">
         <v>433</v>
-      </c>
-      <c r="H13" s="88" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="78" x14ac:dyDescent="0.2">
       <c r="A14" s="92" t="s">
+        <v>434</v>
+      </c>
+      <c r="B14" s="77" t="s">
         <v>435</v>
       </c>
-      <c r="B14" s="77" t="s">
+      <c r="C14" s="77" t="s">
         <v>436</v>
       </c>
-      <c r="C14" s="77" t="s">
+      <c r="D14" s="77" t="s">
         <v>437</v>
       </c>
-      <c r="D14" s="77" t="s">
+      <c r="E14" s="77" t="s">
         <v>438</v>
-      </c>
-      <c r="E14" s="77" t="s">
-        <v>439</v>
       </c>
       <c r="F14" s="77" t="s">
         <v>17</v>
       </c>
       <c r="G14" s="77" t="s">
+        <v>439</v>
+      </c>
+      <c r="H14" s="77" t="s">
         <v>440</v>
-      </c>
-      <c r="H14" s="77" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="52" x14ac:dyDescent="0.2">
       <c r="A15" s="94" t="s">
+        <v>441</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>442</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="74" t="s">
         <v>443</v>
       </c>
-      <c r="C15" s="74" t="s">
+      <c r="D15" s="74" t="s">
         <v>444</v>
       </c>
-      <c r="D15" s="74" t="s">
+      <c r="E15" s="74" t="s">
         <v>445</v>
-      </c>
-      <c r="E15" s="74" t="s">
-        <v>446</v>
       </c>
       <c r="F15" s="74" t="s">
         <v>26</v>
       </c>
       <c r="G15" s="74" t="s">
+        <v>446</v>
+      </c>
+      <c r="H15" s="74" t="s">
         <v>447</v>
-      </c>
-      <c r="H15" s="74" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="52" x14ac:dyDescent="0.2">
       <c r="A16" s="92" t="s">
+        <v>448</v>
+      </c>
+      <c r="B16" s="77" t="s">
         <v>449</v>
       </c>
-      <c r="B16" s="77" t="s">
+      <c r="C16" s="77" t="s">
         <v>450</v>
       </c>
-      <c r="C16" s="77" t="s">
+      <c r="D16" s="77" t="s">
         <v>451</v>
       </c>
-      <c r="D16" s="77" t="s">
+      <c r="E16" s="77" t="s">
         <v>452</v>
-      </c>
-      <c r="E16" s="77" t="s">
-        <v>453</v>
       </c>
       <c r="F16" s="77" t="s">
         <v>26</v>
       </c>
       <c r="G16" s="77" t="s">
+        <v>453</v>
+      </c>
+      <c r="H16" s="77" t="s">
         <v>454</v>
-      </c>
-      <c r="H16" s="77" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="52" x14ac:dyDescent="0.2">
       <c r="A17" s="94" t="s">
+        <v>455</v>
+      </c>
+      <c r="B17" s="74" t="s">
         <v>456</v>
       </c>
-      <c r="B17" s="74" t="s">
+      <c r="C17" s="74" t="s">
         <v>457</v>
       </c>
-      <c r="C17" s="74" t="s">
+      <c r="D17" s="74" t="s">
+        <v>461</v>
+      </c>
+      <c r="E17" s="74" t="s">
         <v>458</v>
-      </c>
-      <c r="D17" s="74" t="s">
-        <v>462</v>
-      </c>
-      <c r="E17" s="74" t="s">
-        <v>459</v>
       </c>
       <c r="F17" s="74" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="74" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="H17" s="74" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Cover and Evidence tracker (Needs working)
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E06E2CF-9E18-FE42-B461-9EB1EA4942D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71BCDAFF-82A0-0541-9DB6-D4537FB017B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="8" r:id="rId1"/>
     <sheet name="Crosswalk" sheetId="2" r:id="rId2"/>
-    <sheet name="Implementation Roadmap" sheetId="4" r:id="rId3"/>
-    <sheet name="Gap Analysis" sheetId="7" r:id="rId4"/>
-    <sheet name="Legend" sheetId="6" r:id="rId5"/>
+    <sheet name="Gap Analysis" sheetId="7" r:id="rId3"/>
+    <sheet name="Implementation Roadmap" sheetId="4" r:id="rId4"/>
+    <sheet name="Evidence tracker" sheetId="9" r:id="rId5"/>
+    <sheet name="Legend" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="472">
   <si>
     <t>CSCRF
 Function</t>
@@ -1140,9 +1141,6 @@
     <t>17.1-17.7 Full IR Set</t>
   </si>
   <si>
-    <t>SECTION B — 12-Month Implementation Roadmap (Qualified RE Reference Model)</t>
-  </si>
-  <si>
     <t>Phase</t>
   </si>
   <si>
@@ -1526,15 +1524,6 @@
     <t>RE Tier : CIS Implementation Group alignment and 12-month phased roadmap</t>
   </si>
   <si>
-    <t>Prepared By: Ronit Yadav &lt;ronit.yadav@sbicapsec.com&gt;</t>
-  </si>
-  <si>
-    <t>Reviewed by: Nilisha Wandile</t>
-  </si>
-  <si>
-    <t>LinkedIn: https://www.linkedin.com/in/nilisha-wandile/</t>
-  </si>
-  <si>
     <t>CIS Control</t>
   </si>
   <si>
@@ -1645,13 +1634,52 @@
   <si>
     <t>Year 1 baseline by Q1
 Year 2 Jan every year</t>
+  </si>
+  <si>
+    <t>Crosswalk &amp; Companion Guide for Indian Capital Market Regulated Entities</t>
+  </si>
+  <si>
+    <t>Reference Framework</t>
+  </si>
+  <si>
+    <t>Target Standard</t>
+  </si>
+  <si>
+    <t>Document Version</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF  :  CIS Controls v8.1</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF 2024 - Circular No. SEBI/HO/ITD-LE/CYS/P/CIR/2024/163 dated August 20, 2024</t>
+  </si>
+  <si>
+    <t>CIS Controls v8.1 (2024) - Center for Internet Security</t>
+  </si>
+  <si>
+    <t>v0.1 - Community Draft (May 2026)</t>
+  </si>
+  <si>
+    <t>Prepared by</t>
+  </si>
+  <si>
+    <t>Ronit Yadav&lt;Ronit.Yadav@sbicapsec.com&gt;</t>
+  </si>
+  <si>
+    <t>Reviewed by</t>
+  </si>
+  <si>
+    <t>Nilisha Wandile &lt;LinkedIn: https://www.linkedin.com/in/nilisha-wandile/&gt;</t>
+  </si>
+  <si>
+    <t>SECTION B - 12-Month Implementation Roadmap (Qualified RE Reference Model)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="51" x14ac:knownFonts="1">
+  <fonts count="56" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1985,18 +2013,46 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFE8C97A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="28"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0B1F3A"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -2127,38 +2183,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2172,7 +2201,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2181,26 +2213,47 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2209,35 +2262,11 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2251,7 +2280,10 @@
     <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2260,157 +2292,198 @@
     <xf numFmtId="0" fontId="27" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="47" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="50" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="50" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="42" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="47" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="50" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="53" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="51" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="50" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2715,7 +2788,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB9251F8-4A3E-BF4A-BD2B-E73CDC9A5F26}">
-  <dimension ref="A3:L19"/>
+  <dimension ref="A2:M27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.1640625" customWidth="1"/>
@@ -2727,105 +2800,260 @@
     <col min="12" max="12" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="62"/>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="62"/>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="62" t="s">
-        <v>423</v>
-      </c>
-      <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
-      <c r="D10" s="62"/>
-      <c r="E10" s="62"/>
-      <c r="F10" s="62"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="62" t="s">
-        <v>424</v>
-      </c>
-      <c r="B11" s="62"/>
-      <c r="C11" s="62" t="s">
-        <v>425</v>
-      </c>
-      <c r="D11" s="62"/>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="102" t="s">
-        <v>412</v>
-      </c>
-      <c r="B14" s="81"/>
-      <c r="C14" s="81"/>
-      <c r="D14" s="81"/>
-      <c r="E14" s="81"/>
-      <c r="F14" s="81"/>
-      <c r="G14" s="81"/>
-      <c r="H14" s="81"/>
-      <c r="I14" s="81"/>
-      <c r="J14" s="81"/>
-      <c r="K14" s="81"/>
-      <c r="L14" s="81"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="97" t="s">
-        <v>416</v>
-      </c>
-      <c r="B15" s="98"/>
-      <c r="C15" s="98"/>
-      <c r="D15" s="101" t="s">
-        <v>421</v>
-      </c>
-      <c r="E15" s="98"/>
-      <c r="F15" s="98"/>
-      <c r="G15" s="98"/>
-      <c r="H15" s="98"/>
-      <c r="I15" s="98"/>
-      <c r="J15" s="98"/>
-      <c r="K15" s="98"/>
-      <c r="L15" s="98"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" s="99" t="s">
-        <v>417</v>
-      </c>
-      <c r="B16" s="100"/>
-      <c r="C16" s="100"/>
-      <c r="D16" s="61" t="s">
-        <v>413</v>
-      </c>
-      <c r="E16" s="100"/>
-      <c r="F16" s="100"/>
-      <c r="G16" s="100"/>
-      <c r="H16" s="100"/>
-      <c r="I16" s="100"/>
-      <c r="J16" s="100"/>
-      <c r="K16" s="100"/>
-      <c r="L16" s="100"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="97" t="s">
-        <v>418</v>
-      </c>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="98"/>
+      <c r="B2" s="98"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="98"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="98"/>
+      <c r="B3" s="103" t="s">
+        <v>463</v>
+      </c>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="98"/>
+      <c r="B4" s="80"/>
+      <c r="C4" s="80"/>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="80"/>
+      <c r="H4" s="80"/>
+      <c r="I4" s="80"/>
+      <c r="J4" s="80"/>
+      <c r="K4" s="80"/>
+      <c r="L4" s="80"/>
+      <c r="M4" s="80"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="98"/>
+      <c r="B5" s="80"/>
+      <c r="C5" s="80"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="80"/>
+      <c r="F5" s="80"/>
+      <c r="G5" s="80"/>
+      <c r="H5" s="80"/>
+      <c r="I5" s="80"/>
+      <c r="J5" s="80"/>
+      <c r="K5" s="80"/>
+      <c r="L5" s="80"/>
+      <c r="M5" s="80"/>
+    </row>
+    <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="98"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
+      <c r="D6" s="80"/>
+      <c r="E6" s="80"/>
+      <c r="F6" s="80"/>
+      <c r="G6" s="80"/>
+      <c r="H6" s="80"/>
+      <c r="I6" s="80"/>
+      <c r="J6" s="80"/>
+      <c r="K6" s="80"/>
+      <c r="L6" s="80"/>
+      <c r="M6" s="80"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="98"/>
+      <c r="B7" s="99" t="s">
+        <v>459</v>
+      </c>
+      <c r="C7" s="100"/>
+      <c r="D7" s="100"/>
+      <c r="E7" s="100"/>
+      <c r="F7" s="100"/>
+      <c r="G7" s="100"/>
+      <c r="H7" s="100"/>
+      <c r="I7" s="100"/>
+      <c r="J7" s="100"/>
+      <c r="K7" s="100"/>
+      <c r="L7" s="100"/>
+      <c r="M7" s="100"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="98"/>
+      <c r="B8" s="100"/>
+      <c r="C8" s="100"/>
+      <c r="D8" s="100"/>
+      <c r="E8" s="100"/>
+      <c r="F8" s="100"/>
+      <c r="G8" s="100"/>
+      <c r="H8" s="100"/>
+      <c r="I8" s="100"/>
+      <c r="J8" s="100"/>
+      <c r="K8" s="100"/>
+      <c r="L8" s="100"/>
+      <c r="M8" s="100"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="98"/>
+      <c r="B9" s="100"/>
+      <c r="C9" s="100"/>
+      <c r="D9" s="100"/>
+      <c r="E9" s="100"/>
+      <c r="F9" s="100"/>
+      <c r="G9" s="100"/>
+      <c r="H9" s="100"/>
+      <c r="I9" s="100"/>
+      <c r="J9" s="100"/>
+      <c r="K9" s="100"/>
+      <c r="L9" s="100"/>
+      <c r="M9" s="100"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="98"/>
+      <c r="B10" s="98"/>
+      <c r="C10" s="98"/>
+      <c r="D10" s="98"/>
+      <c r="E10" s="98"/>
+      <c r="F10" s="98"/>
+      <c r="G10" s="98"/>
+      <c r="H10" s="98"/>
+      <c r="I10" s="98"/>
+      <c r="J10" s="98"/>
+      <c r="K10" s="98"/>
+      <c r="L10" s="98"/>
+      <c r="M10" s="98"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" s="98"/>
+      <c r="B11" s="104" t="s">
+        <v>460</v>
+      </c>
+      <c r="C11" s="80"/>
+      <c r="D11" s="80"/>
+      <c r="E11" s="102" t="s">
+        <v>464</v>
+      </c>
+      <c r="F11" s="78"/>
+      <c r="G11" s="78"/>
+      <c r="H11" s="78"/>
+      <c r="I11" s="78"/>
+      <c r="J11" s="78"/>
+      <c r="K11" s="78"/>
+      <c r="L11" s="78"/>
+      <c r="M11" s="78"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" s="98"/>
+      <c r="B12" s="104" t="s">
+        <v>461</v>
+      </c>
+      <c r="C12" s="80"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="102" t="s">
+        <v>465</v>
+      </c>
+      <c r="F12" s="78"/>
+      <c r="G12" s="78"/>
+      <c r="H12" s="78"/>
+      <c r="I12" s="78"/>
+      <c r="J12" s="78"/>
+      <c r="K12" s="78"/>
+      <c r="L12" s="78"/>
+      <c r="M12" s="78"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="98"/>
+      <c r="B13" s="104" t="s">
+        <v>462</v>
+      </c>
+      <c r="C13" s="80"/>
+      <c r="D13" s="80"/>
+      <c r="E13" s="102" t="s">
+        <v>466</v>
+      </c>
+      <c r="F13" s="78"/>
+      <c r="G13" s="78"/>
+      <c r="H13" s="78"/>
+      <c r="I13" s="78"/>
+      <c r="J13" s="78"/>
+      <c r="K13" s="78"/>
+      <c r="L13" s="78"/>
+      <c r="M13" s="78"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="98"/>
+      <c r="B14" s="104" t="s">
+        <v>467</v>
+      </c>
+      <c r="C14" s="80"/>
+      <c r="D14" s="80"/>
+      <c r="E14" s="102" t="s">
+        <v>468</v>
+      </c>
+      <c r="F14" s="78"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="78"/>
+      <c r="I14" s="78"/>
+      <c r="J14" s="78"/>
+      <c r="K14" s="78"/>
+      <c r="L14" s="78"/>
+      <c r="M14" s="78"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" s="98"/>
+      <c r="B15" s="104" t="s">
+        <v>469</v>
+      </c>
+      <c r="C15" s="80"/>
+      <c r="D15" s="80"/>
+      <c r="E15" s="102" t="s">
+        <v>470</v>
+      </c>
+      <c r="F15" s="78"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="78"/>
+      <c r="J15" s="78"/>
+      <c r="K15" s="78"/>
+      <c r="L15" s="78"/>
+      <c r="M15" s="78"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" s="98"/>
+      <c r="B16" s="101"/>
+      <c r="C16" s="78"/>
+      <c r="D16" s="78"/>
+      <c r="E16" s="102"/>
+      <c r="F16" s="78"/>
+      <c r="G16" s="78"/>
+      <c r="H16" s="78"/>
+      <c r="I16" s="78"/>
+      <c r="J16" s="78"/>
+      <c r="K16" s="78"/>
+      <c r="L16" s="78"/>
+      <c r="M16" s="78"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" s="98"/>
       <c r="B17" s="98"/>
       <c r="C17" s="98"/>
-      <c r="D17" s="101" t="s">
-        <v>422</v>
-      </c>
+      <c r="D17" s="98"/>
       <c r="E17" s="98"/>
       <c r="F17" s="98"/>
       <c r="G17" s="98"/>
@@ -2834,34 +3062,28 @@
       <c r="J17" s="98"/>
       <c r="K17" s="98"/>
       <c r="L17" s="98"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="99" t="s">
-        <v>419</v>
-      </c>
-      <c r="B18" s="100"/>
-      <c r="C18" s="100"/>
-      <c r="D18" s="61" t="s">
-        <v>414</v>
-      </c>
-      <c r="E18" s="100"/>
-      <c r="F18" s="100"/>
-      <c r="G18" s="100"/>
-      <c r="H18" s="100"/>
-      <c r="I18" s="100"/>
-      <c r="J18" s="100"/>
-      <c r="K18" s="100"/>
-      <c r="L18" s="100"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="97" t="s">
-        <v>420</v>
-      </c>
+      <c r="M17" s="98"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" s="98"/>
+      <c r="B18" s="98"/>
+      <c r="C18" s="98"/>
+      <c r="D18" s="98"/>
+      <c r="E18" s="98"/>
+      <c r="F18" s="98"/>
+      <c r="G18" s="98"/>
+      <c r="H18" s="98"/>
+      <c r="I18" s="98"/>
+      <c r="J18" s="98"/>
+      <c r="K18" s="98"/>
+      <c r="L18" s="98"/>
+      <c r="M18" s="98"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" s="98"/>
       <c r="B19" s="98"/>
       <c r="C19" s="98"/>
-      <c r="D19" s="101" t="s">
-        <v>415</v>
-      </c>
+      <c r="D19" s="98"/>
       <c r="E19" s="98"/>
       <c r="F19" s="98"/>
       <c r="G19" s="98"/>
@@ -2870,20 +3092,156 @@
       <c r="J19" s="98"/>
       <c r="K19" s="98"/>
       <c r="L19" s="98"/>
+      <c r="M19" s="98"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" s="98"/>
+      <c r="B20" s="98"/>
+      <c r="C20" s="98"/>
+      <c r="D20" s="98"/>
+      <c r="E20" s="98"/>
+      <c r="F20" s="98"/>
+      <c r="G20" s="98"/>
+      <c r="H20" s="98"/>
+      <c r="I20" s="98"/>
+      <c r="J20" s="98"/>
+      <c r="K20" s="98"/>
+      <c r="L20" s="98"/>
+      <c r="M20" s="98"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" s="97" t="s">
+        <v>411</v>
+      </c>
+      <c r="B22" s="97"/>
+      <c r="C22" s="97"/>
+      <c r="D22" s="97"/>
+      <c r="E22" s="97"/>
+      <c r="F22" s="97"/>
+      <c r="G22" s="97"/>
+      <c r="H22" s="97"/>
+      <c r="I22" s="97"/>
+      <c r="J22" s="97"/>
+      <c r="K22" s="97"/>
+      <c r="L22" s="97"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" s="94" t="s">
+        <v>415</v>
+      </c>
+      <c r="B23" s="94"/>
+      <c r="C23" s="94"/>
+      <c r="D23" s="96" t="s">
+        <v>420</v>
+      </c>
+      <c r="E23" s="96"/>
+      <c r="F23" s="96"/>
+      <c r="G23" s="96"/>
+      <c r="H23" s="96"/>
+      <c r="I23" s="96"/>
+      <c r="J23" s="96"/>
+      <c r="K23" s="96"/>
+      <c r="L23" s="96"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" s="95" t="s">
+        <v>416</v>
+      </c>
+      <c r="B24" s="95"/>
+      <c r="C24" s="95"/>
+      <c r="D24" s="59" t="s">
+        <v>412</v>
+      </c>
+      <c r="E24" s="59"/>
+      <c r="F24" s="59"/>
+      <c r="G24" s="59"/>
+      <c r="H24" s="59"/>
+      <c r="I24" s="59"/>
+      <c r="J24" s="59"/>
+      <c r="K24" s="59"/>
+      <c r="L24" s="59"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="94" t="s">
+        <v>417</v>
+      </c>
+      <c r="B25" s="94"/>
+      <c r="C25" s="94"/>
+      <c r="D25" s="96" t="s">
+        <v>421</v>
+      </c>
+      <c r="E25" s="96"/>
+      <c r="F25" s="96"/>
+      <c r="G25" s="96"/>
+      <c r="H25" s="96"/>
+      <c r="I25" s="96"/>
+      <c r="J25" s="96"/>
+      <c r="K25" s="96"/>
+      <c r="L25" s="96"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" s="95" t="s">
+        <v>418</v>
+      </c>
+      <c r="B26" s="95"/>
+      <c r="C26" s="95"/>
+      <c r="D26" s="59" t="s">
+        <v>413</v>
+      </c>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="59"/>
+      <c r="J26" s="59"/>
+      <c r="K26" s="59"/>
+      <c r="L26" s="59"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A27" s="94" t="s">
+        <v>419</v>
+      </c>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="96" t="s">
+        <v>414</v>
+      </c>
+      <c r="E27" s="96"/>
+      <c r="F27" s="96"/>
+      <c r="G27" s="96"/>
+      <c r="H27" s="96"/>
+      <c r="I27" s="96"/>
+      <c r="J27" s="96"/>
+      <c r="K27" s="96"/>
+      <c r="L27" s="96"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:L19"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:L16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:L17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:L18"/>
-    <mergeCell ref="A14:L14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:L15"/>
+  <mergeCells count="25">
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:M16"/>
+    <mergeCell ref="E14:M14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:M15"/>
+    <mergeCell ref="B3:M6"/>
+    <mergeCell ref="B7:M9"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E11:M11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="E12:M12"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:L27"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:L24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="D25:L25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="D26:L26"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D23:L23"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:M13"/>
+    <mergeCell ref="B14:D14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2921,1207 +3279,1207 @@
       <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
     </row>
     <row r="3" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
     </row>
     <row r="4" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="105" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="105" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="105" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="105" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="105" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="105" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="105" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="105" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="105" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="105" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="25"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
     </row>
     <row r="6" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="42" t="s">
+      <c r="F7" s="41" t="s">
         <v>235</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="17" t="s">
+      <c r="I7" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="J7" s="18" t="s">
+      <c r="J7" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="K7" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="16" t="s">
+      <c r="G8" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="17" t="s">
+      <c r="I9" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="J9" s="18" t="s">
+      <c r="J9" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="K9" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="25"/>
-      <c r="K10" s="25"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
     </row>
     <row r="11" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="32" t="s">
+      <c r="C11" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="33" t="s">
+      <c r="D11" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="E11" s="32" t="s">
+      <c r="E11" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="F11" s="34" t="s">
+      <c r="F11" s="33" t="s">
         <v>67</v>
       </c>
-      <c r="G11" s="35" t="s">
+      <c r="G11" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="36" t="s">
+      <c r="H11" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I11" s="37" t="s">
+      <c r="I11" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="J11" s="38" t="s">
+      <c r="J11" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="K11" s="35" t="s">
+      <c r="K11" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="39" t="s">
+      <c r="B12" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="40" t="s">
+      <c r="C12" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="E12" s="40" t="s">
+      <c r="E12" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="42" t="s">
+      <c r="F12" s="41" t="s">
         <v>74</v>
       </c>
-      <c r="G12" s="43" t="s">
+      <c r="G12" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="H12" s="36" t="s">
+      <c r="H12" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I12" s="44" t="s">
+      <c r="I12" s="43" t="s">
         <v>75</v>
       </c>
-      <c r="J12" s="45" t="s">
+      <c r="J12" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="K12" s="35" t="s">
+      <c r="K12" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="33" t="s">
+      <c r="D13" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="E13" s="32" t="s">
+      <c r="E13" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="F13" s="34" t="s">
+      <c r="F13" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="G13" s="46" t="s">
+      <c r="G13" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="47" t="s">
+      <c r="H13" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="I13" s="37" t="s">
+      <c r="I13" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="J13" s="38" t="s">
+      <c r="J13" s="37" t="s">
         <v>215</v>
       </c>
-      <c r="K13" s="46" t="s">
+      <c r="K13" s="45" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="39" t="s">
+      <c r="B14" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="C14" s="40" t="s">
+      <c r="C14" s="39" t="s">
         <v>87</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="40" t="s">
+      <c r="E14" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="F14" s="42" t="s">
+      <c r="F14" s="41" t="s">
         <v>318</v>
       </c>
-      <c r="G14" s="43" t="s">
+      <c r="G14" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="H14" s="36" t="s">
+      <c r="H14" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I14" s="44" t="s">
+      <c r="I14" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="J14" s="45" t="s">
+      <c r="J14" s="44" t="s">
         <v>216</v>
       </c>
-      <c r="K14" s="43" t="s">
+      <c r="K14" s="42" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="31" t="s">
         <v>217</v>
       </c>
-      <c r="D15" s="33" t="s">
+      <c r="D15" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="32" t="s">
+      <c r="E15" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="34" t="s">
+      <c r="F15" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="G15" s="35" t="s">
+      <c r="G15" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="48" t="s">
+      <c r="H15" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="37" t="s">
+      <c r="I15" s="36" t="s">
         <v>92</v>
       </c>
-      <c r="J15" s="38" t="s">
+      <c r="J15" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="K15" s="35" t="s">
+      <c r="K15" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="51" t="s">
+      <c r="A16" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
     </row>
     <row r="17" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="52" t="s">
+      <c r="A17" s="51" t="s">
         <v>150</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="D17" s="33" t="s">
+      <c r="D17" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="E17" s="32" t="s">
+      <c r="E17" s="31" t="s">
         <v>154</v>
       </c>
-      <c r="F17" s="34" t="s">
+      <c r="F17" s="33" t="s">
         <v>236</v>
       </c>
-      <c r="G17" s="35" t="s">
+      <c r="G17" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H17" s="36" t="s">
+      <c r="H17" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="37" t="s">
+      <c r="I17" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="J17" s="38" t="s">
+      <c r="J17" s="37" t="s">
         <v>156</v>
       </c>
-      <c r="K17" s="35" t="s">
+      <c r="K17" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="52" t="s">
+      <c r="A18" s="51" t="s">
         <v>150</v>
       </c>
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="C18" s="40" t="s">
+      <c r="C18" s="39" t="s">
         <v>218</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="40" t="s">
         <v>158</v>
       </c>
-      <c r="E18" s="40" t="s">
+      <c r="E18" s="39" t="s">
         <v>159</v>
       </c>
-      <c r="F18" s="42" t="s">
+      <c r="F18" s="41" t="s">
         <v>160</v>
       </c>
-      <c r="G18" s="43" t="s">
+      <c r="G18" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="H18" s="36" t="s">
+      <c r="H18" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I18" s="44" t="s">
+      <c r="I18" s="43" t="s">
         <v>161</v>
       </c>
-      <c r="J18" s="45" t="s">
+      <c r="J18" s="44" t="s">
         <v>162</v>
       </c>
-      <c r="K18" s="35" t="s">
+      <c r="K18" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="52" t="s">
+      <c r="A19" s="51" t="s">
         <v>150</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="C19" s="32" t="s">
+      <c r="C19" s="31" t="s">
         <v>165</v>
       </c>
-      <c r="D19" s="33" t="s">
+      <c r="D19" s="32" t="s">
         <v>166</v>
       </c>
-      <c r="E19" s="32" t="s">
+      <c r="E19" s="31" t="s">
         <v>167</v>
       </c>
-      <c r="F19" s="34" t="s">
+      <c r="F19" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="G19" s="46" t="s">
+      <c r="G19" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="H19" s="47" t="s">
+      <c r="H19" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="I19" s="37" t="s">
+      <c r="I19" s="36" t="s">
         <v>173</v>
       </c>
-      <c r="J19" s="38" t="s">
+      <c r="J19" s="37" t="s">
         <v>219</v>
       </c>
-      <c r="K19" s="46" t="s">
+      <c r="K19" s="45" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="52" t="s">
+      <c r="A20" s="51" t="s">
         <v>150</v>
       </c>
-      <c r="B20" s="39" t="s">
+      <c r="B20" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="C20" s="40" t="s">
+      <c r="C20" s="39" t="s">
         <v>220</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="40" t="s">
         <v>170</v>
       </c>
-      <c r="E20" s="40" t="s">
+      <c r="E20" s="39" t="s">
         <v>171</v>
       </c>
-      <c r="F20" s="42" t="s">
+      <c r="F20" s="41" t="s">
         <v>172</v>
       </c>
-      <c r="G20" s="46" t="s">
+      <c r="G20" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="H20" s="48" t="s">
+      <c r="H20" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="I20" s="44" t="s">
+      <c r="I20" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="J20" s="45" t="s">
+      <c r="J20" s="44" t="s">
         <v>221</v>
       </c>
-      <c r="K20" s="35" t="s">
+      <c r="K20" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="53" t="s">
+      <c r="A21" s="52" t="s">
         <v>193</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
     </row>
     <row r="22" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="B22" s="31" t="s">
+      <c r="B22" s="30" t="s">
         <v>176</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="31" t="s">
         <v>177</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="E22" s="32" t="s">
+      <c r="E22" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="F22" s="34" t="s">
+      <c r="F22" s="33" t="s">
         <v>178</v>
       </c>
-      <c r="G22" s="35" t="s">
+      <c r="G22" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H22" s="48" t="s">
+      <c r="H22" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="I22" s="37" t="s">
+      <c r="I22" s="36" t="s">
         <v>222</v>
       </c>
-      <c r="J22" s="38" t="s">
+      <c r="J22" s="37" t="s">
         <v>179</v>
       </c>
-      <c r="K22" s="46" t="s">
+      <c r="K22" s="45" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="54" t="s">
+      <c r="A23" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="B23" s="38" t="s">
         <v>180</v>
       </c>
-      <c r="C23" s="40" t="s">
+      <c r="C23" s="39" t="s">
         <v>223</v>
       </c>
-      <c r="D23" s="41" t="s">
+      <c r="D23" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="E23" s="40" t="s">
+      <c r="E23" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="F23" s="42" t="s">
+      <c r="F23" s="41" t="s">
         <v>181</v>
       </c>
-      <c r="G23" s="35" t="s">
+      <c r="G23" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H23" s="47" t="s">
+      <c r="H23" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="I23" s="44" t="s">
+      <c r="I23" s="43" t="s">
         <v>182</v>
       </c>
-      <c r="J23" s="45" t="s">
+      <c r="J23" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="K23" s="46" t="s">
+      <c r="K23" s="45" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="54" t="s">
+      <c r="A24" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="C24" s="32" t="s">
+      <c r="C24" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="D24" s="33" t="s">
+      <c r="D24" s="32" t="s">
         <v>186</v>
       </c>
-      <c r="E24" s="32" t="s">
+      <c r="E24" s="31" t="s">
         <v>187</v>
       </c>
-      <c r="F24" s="34" t="s">
+      <c r="F24" s="33" t="s">
         <v>188</v>
       </c>
-      <c r="G24" s="43" t="s">
+      <c r="G24" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="H24" s="36" t="s">
+      <c r="H24" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I24" s="37" t="s">
+      <c r="I24" s="36" t="s">
         <v>189</v>
       </c>
-      <c r="J24" s="38" t="s">
+      <c r="J24" s="37" t="s">
         <v>224</v>
       </c>
-      <c r="K24" s="35" t="s">
+      <c r="K24" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="54" t="s">
+      <c r="A25" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="B25" s="39" t="s">
+      <c r="B25" s="38" t="s">
         <v>190</v>
       </c>
-      <c r="C25" s="40" t="s">
+      <c r="C25" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="E25" s="40" t="s">
+      <c r="E25" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="F25" s="42" t="s">
+      <c r="F25" s="41" t="s">
         <v>319</v>
       </c>
-      <c r="G25" s="43" t="s">
+      <c r="G25" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="H25" s="47" t="s">
+      <c r="H25" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="I25" s="44" t="s">
+      <c r="I25" s="43" t="s">
         <v>192</v>
       </c>
-      <c r="J25" s="45" t="s">
+      <c r="J25" s="44" t="s">
         <v>225</v>
       </c>
-      <c r="K25" s="46" t="s">
+      <c r="K25" s="45" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="49" t="s">
+      <c r="A26" s="48" t="s">
         <v>149</v>
       </c>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="25"/>
-      <c r="J26" s="25"/>
-      <c r="K26" s="25"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
     </row>
     <row r="27" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="50" t="s">
+      <c r="A27" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="30" t="s">
         <v>96</v>
       </c>
-      <c r="C27" s="32" t="s">
+      <c r="C27" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="E27" s="32" t="s">
+      <c r="E27" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="F27" s="34" t="s">
+      <c r="F27" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="G27" s="35" t="s">
+      <c r="G27" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H27" s="36" t="s">
+      <c r="H27" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I27" s="37" t="s">
+      <c r="I27" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="J27" s="38" t="s">
+      <c r="J27" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="K27" s="46" t="s">
+      <c r="K27" s="45" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B28" s="39" t="s">
+      <c r="B28" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="C28" s="40" t="s">
+      <c r="C28" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="E28" s="40" t="s">
+      <c r="E28" s="39" t="s">
         <v>105</v>
       </c>
-      <c r="F28" s="42" t="s">
+      <c r="F28" s="41" t="s">
         <v>106</v>
       </c>
-      <c r="G28" s="35" t="s">
+      <c r="G28" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H28" s="36" t="s">
+      <c r="H28" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I28" s="44" t="s">
+      <c r="I28" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="J28" s="45" t="s">
+      <c r="J28" s="44" t="s">
         <v>108</v>
       </c>
-      <c r="K28" s="35" t="s">
+      <c r="K28" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="50" t="s">
+      <c r="A29" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B29" s="31" t="s">
+      <c r="B29" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="C29" s="32" t="s">
+      <c r="C29" s="31" t="s">
         <v>110</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="E29" s="32" t="s">
+      <c r="E29" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="F29" s="34" t="s">
+      <c r="F29" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="G29" s="43" t="s">
+      <c r="G29" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="H29" s="36" t="s">
+      <c r="H29" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I29" s="37" t="s">
+      <c r="I29" s="36" t="s">
         <v>114</v>
       </c>
-      <c r="J29" s="38" t="s">
+      <c r="J29" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="K29" s="46" t="s">
+      <c r="K29" s="45" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="50" t="s">
+      <c r="A30" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B30" s="39" t="s">
+      <c r="B30" s="38" t="s">
         <v>116</v>
       </c>
-      <c r="C30" s="40" t="s">
+      <c r="C30" s="39" t="s">
         <v>226</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="40" t="s">
         <v>117</v>
       </c>
-      <c r="E30" s="40" t="s">
+      <c r="E30" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="F30" s="42" t="s">
+      <c r="F30" s="41" t="s">
         <v>119</v>
       </c>
-      <c r="G30" s="35" t="s">
+      <c r="G30" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H30" s="36" t="s">
+      <c r="H30" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I30" s="44" t="s">
+      <c r="I30" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="J30" s="45" t="s">
+      <c r="J30" s="44" t="s">
         <v>121</v>
       </c>
-      <c r="K30" s="35" t="s">
+      <c r="K30" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="50" t="s">
+      <c r="A31" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B31" s="39" t="s">
+      <c r="B31" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="C31" s="40" t="s">
+      <c r="C31" s="39" t="s">
         <v>123</v>
       </c>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="40" t="s">
         <v>124</v>
       </c>
-      <c r="E31" s="40" t="s">
+      <c r="E31" s="39" t="s">
         <v>125</v>
       </c>
-      <c r="F31" s="42" t="s">
+      <c r="F31" s="41" t="s">
         <v>126</v>
       </c>
-      <c r="G31" s="35" t="s">
+      <c r="G31" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="H31" s="36" t="s">
+      <c r="H31" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="I31" s="44" t="s">
+      <c r="I31" s="43" t="s">
         <v>127</v>
       </c>
-      <c r="J31" s="45" t="s">
+      <c r="J31" s="44" t="s">
         <v>227</v>
       </c>
-      <c r="K31" s="35" t="s">
+      <c r="K31" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="50" t="s">
+      <c r="A32" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B32" s="39" t="s">
+      <c r="B32" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="C32" s="40" t="s">
+      <c r="C32" s="39" t="s">
         <v>228</v>
       </c>
-      <c r="D32" s="41" t="s">
+      <c r="D32" s="40" t="s">
         <v>129</v>
       </c>
-      <c r="E32" s="40" t="s">
+      <c r="E32" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="F32" s="42" t="s">
+      <c r="F32" s="41" t="s">
         <v>131</v>
       </c>
-      <c r="G32" s="35" t="s">
+      <c r="G32" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H32" s="36" t="s">
+      <c r="H32" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I32" s="44" t="s">
+      <c r="I32" s="43" t="s">
         <v>132</v>
       </c>
-      <c r="J32" s="45" t="s">
+      <c r="J32" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="K32" s="35" t="s">
+      <c r="K32" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="50" t="s">
+      <c r="A33" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B33" s="31" t="s">
+      <c r="B33" s="30" t="s">
         <v>134</v>
       </c>
-      <c r="C33" s="32" t="s">
+      <c r="C33" s="31" t="s">
         <v>229</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="32" t="s">
         <v>135</v>
       </c>
-      <c r="E33" s="32" t="s">
+      <c r="E33" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="F33" s="34" t="s">
+      <c r="F33" s="33" t="s">
         <v>137</v>
       </c>
-      <c r="G33" s="43" t="s">
+      <c r="G33" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="H33" s="48" t="s">
+      <c r="H33" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="I33" s="37" t="s">
+      <c r="I33" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="J33" s="38" t="s">
+      <c r="J33" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="K33" s="35" t="s">
+      <c r="K33" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="50" t="s">
+      <c r="A34" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B34" s="39" t="s">
+      <c r="B34" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="C34" s="40" t="s">
+      <c r="C34" s="39" t="s">
         <v>230</v>
       </c>
-      <c r="D34" s="41" t="s">
+      <c r="D34" s="40" t="s">
         <v>135</v>
       </c>
-      <c r="E34" s="40" t="s">
+      <c r="E34" s="39" t="s">
         <v>141</v>
       </c>
-      <c r="F34" s="42" t="s">
+      <c r="F34" s="41" t="s">
         <v>142</v>
       </c>
-      <c r="G34" s="46" t="s">
+      <c r="G34" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="H34" s="47" t="s">
+      <c r="H34" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="I34" s="44" t="s">
+      <c r="I34" s="43" t="s">
         <v>143</v>
       </c>
-      <c r="J34" s="45" t="s">
+      <c r="J34" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="K34" s="46" t="s">
+      <c r="K34" s="45" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="50" t="s">
+      <c r="A35" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="B35" s="31" t="s">
+      <c r="B35" s="30" t="s">
         <v>144</v>
       </c>
-      <c r="C35" s="32" t="s">
+      <c r="C35" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="D35" s="33" t="s">
+      <c r="D35" s="32" t="s">
         <v>135</v>
       </c>
-      <c r="E35" s="32" t="s">
+      <c r="E35" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="F35" s="34" t="s">
+      <c r="F35" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="G35" s="43" t="s">
+      <c r="G35" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="H35" s="48" t="s">
+      <c r="H35" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="I35" s="37" t="s">
+      <c r="I35" s="36" t="s">
         <v>147</v>
       </c>
-      <c r="J35" s="38" t="s">
+      <c r="J35" s="37" t="s">
         <v>148</v>
       </c>
-      <c r="K35" s="35" t="s">
+      <c r="K35" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="55" t="s">
+      <c r="A36" s="54" t="s">
         <v>213</v>
       </c>
-      <c r="B36" s="25"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="25"/>
-      <c r="E36" s="25"/>
-      <c r="F36" s="25"/>
-      <c r="G36" s="25"/>
-      <c r="H36" s="25"/>
-      <c r="I36" s="25"/>
-      <c r="J36" s="25"/>
-      <c r="K36" s="25"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="24"/>
+      <c r="J36" s="24"/>
+      <c r="K36" s="24"/>
     </row>
     <row r="37" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="56" t="s">
+      <c r="A37" s="55" t="s">
         <v>194</v>
       </c>
-      <c r="B37" s="31" t="s">
+      <c r="B37" s="30" t="s">
         <v>195</v>
       </c>
-      <c r="C37" s="32" t="s">
+      <c r="C37" s="31" t="s">
         <v>196</v>
       </c>
-      <c r="D37" s="33" t="s">
+      <c r="D37" s="32" t="s">
         <v>197</v>
       </c>
-      <c r="E37" s="32" t="s">
+      <c r="E37" s="31" t="s">
         <v>198</v>
       </c>
-      <c r="F37" s="34" t="s">
+      <c r="F37" s="33" t="s">
         <v>199</v>
       </c>
-      <c r="G37" s="35" t="s">
+      <c r="G37" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H37" s="36" t="s">
+      <c r="H37" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I37" s="37" t="s">
+      <c r="I37" s="36" t="s">
         <v>200</v>
       </c>
-      <c r="J37" s="38" t="s">
+      <c r="J37" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="K37" s="35" t="s">
+      <c r="K37" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="56" t="s">
+      <c r="A38" s="55" t="s">
         <v>194</v>
       </c>
-      <c r="B38" s="39" t="s">
+      <c r="B38" s="38" t="s">
         <v>202</v>
       </c>
-      <c r="C38" s="40" t="s">
+      <c r="C38" s="39" t="s">
         <v>232</v>
       </c>
-      <c r="D38" s="41" t="s">
+      <c r="D38" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="E38" s="40" t="s">
+      <c r="E38" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="F38" s="42" t="s">
+      <c r="F38" s="41" t="s">
         <v>181</v>
       </c>
-      <c r="G38" s="35" t="s">
+      <c r="G38" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H38" s="48" t="s">
+      <c r="H38" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="I38" s="44" t="s">
+      <c r="I38" s="43" t="s">
         <v>203</v>
       </c>
-      <c r="J38" s="45" t="s">
+      <c r="J38" s="44" t="s">
         <v>233</v>
       </c>
-      <c r="K38" s="43" t="s">
+      <c r="K38" s="42" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="56" t="s">
+      <c r="A39" s="55" t="s">
         <v>194</v>
       </c>
-      <c r="B39" s="31" t="s">
+      <c r="B39" s="30" t="s">
         <v>204</v>
       </c>
-      <c r="C39" s="32" t="s">
+      <c r="C39" s="31" t="s">
         <v>205</v>
       </c>
-      <c r="D39" s="33" t="s">
+      <c r="D39" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="E39" s="32" t="s">
+      <c r="E39" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="F39" s="34" t="s">
+      <c r="F39" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="G39" s="35" t="s">
+      <c r="G39" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="H39" s="36" t="s">
+      <c r="H39" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="I39" s="37" t="s">
+      <c r="I39" s="36" t="s">
         <v>206</v>
       </c>
-      <c r="J39" s="38" t="s">
+      <c r="J39" s="37" t="s">
         <v>207</v>
       </c>
-      <c r="K39" s="35" t="s">
+      <c r="K39" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="56" t="s">
+      <c r="A40" s="55" t="s">
         <v>194</v>
       </c>
-      <c r="B40" s="39" t="s">
+      <c r="B40" s="38" t="s">
         <v>208</v>
       </c>
-      <c r="C40" s="40" t="s">
+      <c r="C40" s="39" t="s">
         <v>209</v>
       </c>
-      <c r="D40" s="41" t="s">
+      <c r="D40" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="E40" s="40" t="s">
+      <c r="E40" s="39" t="s">
         <v>210</v>
       </c>
-      <c r="F40" s="42" t="s">
+      <c r="F40" s="41" t="s">
         <v>211</v>
       </c>
-      <c r="G40" s="46" t="s">
+      <c r="G40" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="H40" s="47" t="s">
+      <c r="H40" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="I40" s="44" t="s">
+      <c r="I40" s="43" t="s">
         <v>212</v>
       </c>
-      <c r="J40" s="45" t="s">
+      <c r="J40" s="44" t="s">
         <v>234</v>
       </c>
-      <c r="K40" s="46" t="s">
+      <c r="K40" s="45" t="s">
         <v>85</v>
       </c>
     </row>
@@ -4141,6 +4499,363 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D072851C-E33D-3E4C-9E1E-B705D90C883D}">
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="21.83203125" customWidth="1"/>
+    <col min="5" max="5" width="39" customWidth="1"/>
+    <col min="6" max="6" width="28.5" customWidth="1"/>
+    <col min="7" max="7" width="24.5" customWidth="1"/>
+    <col min="8" max="8" width="38" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="92" t="s">
+        <v>403</v>
+      </c>
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="86" t="s">
+        <v>404</v>
+      </c>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="85" t="s">
+        <v>365</v>
+      </c>
+      <c r="B4" s="85" t="s">
+        <v>366</v>
+      </c>
+      <c r="C4" s="85" t="s">
+        <v>367</v>
+      </c>
+      <c r="D4" s="85" t="s">
+        <v>368</v>
+      </c>
+      <c r="E4" s="85" t="s">
+        <v>369</v>
+      </c>
+      <c r="F4" s="85" t="s">
+        <v>370</v>
+      </c>
+      <c r="G4" s="85" t="s">
+        <v>371</v>
+      </c>
+      <c r="H4" s="85" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="89" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="74" t="s">
+        <v>373</v>
+      </c>
+      <c r="C5" s="74" t="s">
+        <v>374</v>
+      </c>
+      <c r="D5" s="74" t="s">
+        <v>402</v>
+      </c>
+      <c r="E5" s="74" t="s">
+        <v>375</v>
+      </c>
+      <c r="F5" s="74" t="s">
+        <v>376</v>
+      </c>
+      <c r="G5" s="90" t="s">
+        <v>377</v>
+      </c>
+      <c r="H5" s="77" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="71" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="91" t="s">
+        <v>378</v>
+      </c>
+      <c r="B6" s="71" t="s">
+        <v>379</v>
+      </c>
+      <c r="C6" s="71" t="s">
+        <v>380</v>
+      </c>
+      <c r="D6" s="71" t="s">
+        <v>406</v>
+      </c>
+      <c r="E6" s="71" t="s">
+        <v>381</v>
+      </c>
+      <c r="F6" s="71" t="s">
+        <v>382</v>
+      </c>
+      <c r="G6" s="90" t="s">
+        <v>383</v>
+      </c>
+      <c r="H6" s="77" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="89" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="74" t="s">
+        <v>385</v>
+      </c>
+      <c r="C7" s="74" t="s">
+        <v>386</v>
+      </c>
+      <c r="D7" s="74" t="s">
+        <v>407</v>
+      </c>
+      <c r="E7" s="74" t="s">
+        <v>387</v>
+      </c>
+      <c r="F7" s="74" t="s">
+        <v>388</v>
+      </c>
+      <c r="G7" s="90" t="s">
+        <v>389</v>
+      </c>
+      <c r="H7" s="77" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="91" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" s="71" t="s">
+        <v>408</v>
+      </c>
+      <c r="C8" s="71" t="s">
+        <v>391</v>
+      </c>
+      <c r="D8" s="71" t="s">
+        <v>409</v>
+      </c>
+      <c r="E8" s="71" t="s">
+        <v>392</v>
+      </c>
+      <c r="F8" s="71" t="s">
+        <v>393</v>
+      </c>
+      <c r="G8" s="90" t="s">
+        <v>394</v>
+      </c>
+      <c r="H8" s="77" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="89" t="s">
+        <v>396</v>
+      </c>
+      <c r="B9" s="74" t="s">
+        <v>397</v>
+      </c>
+      <c r="C9" s="74" t="s">
+        <v>380</v>
+      </c>
+      <c r="D9" s="74" t="s">
+        <v>410</v>
+      </c>
+      <c r="E9" s="74" t="s">
+        <v>398</v>
+      </c>
+      <c r="F9" s="74" t="s">
+        <v>399</v>
+      </c>
+      <c r="G9" s="90" t="s">
+        <v>400</v>
+      </c>
+      <c r="H9" s="77" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="86" t="s">
+        <v>456</v>
+      </c>
+      <c r="B12" s="87"/>
+      <c r="C12" s="87"/>
+      <c r="D12" s="87"/>
+      <c r="E12" s="87"/>
+      <c r="F12" s="87"/>
+      <c r="G12" s="87"/>
+      <c r="H12" s="87"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="85" t="s">
+        <v>422</v>
+      </c>
+      <c r="B13" s="85" t="s">
+        <v>423</v>
+      </c>
+      <c r="C13" s="85" t="s">
+        <v>424</v>
+      </c>
+      <c r="D13" s="85" t="s">
+        <v>425</v>
+      </c>
+      <c r="E13" s="85" t="s">
+        <v>426</v>
+      </c>
+      <c r="F13" s="85" t="s">
+        <v>427</v>
+      </c>
+      <c r="G13" s="85" t="s">
+        <v>428</v>
+      </c>
+      <c r="H13" s="85" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="78" x14ac:dyDescent="0.2">
+      <c r="A14" s="89" t="s">
+        <v>430</v>
+      </c>
+      <c r="B14" s="74" t="s">
+        <v>431</v>
+      </c>
+      <c r="C14" s="74" t="s">
+        <v>432</v>
+      </c>
+      <c r="D14" s="74" t="s">
+        <v>433</v>
+      </c>
+      <c r="E14" s="74" t="s">
+        <v>434</v>
+      </c>
+      <c r="F14" s="74" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="74" t="s">
+        <v>435</v>
+      </c>
+      <c r="H14" s="74" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="52" x14ac:dyDescent="0.2">
+      <c r="A15" s="91" t="s">
+        <v>437</v>
+      </c>
+      <c r="B15" s="71" t="s">
+        <v>438</v>
+      </c>
+      <c r="C15" s="71" t="s">
+        <v>439</v>
+      </c>
+      <c r="D15" s="71" t="s">
+        <v>440</v>
+      </c>
+      <c r="E15" s="71" t="s">
+        <v>441</v>
+      </c>
+      <c r="F15" s="71" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="71" t="s">
+        <v>442</v>
+      </c>
+      <c r="H15" s="71" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="52" x14ac:dyDescent="0.2">
+      <c r="A16" s="89" t="s">
+        <v>444</v>
+      </c>
+      <c r="B16" s="74" t="s">
+        <v>445</v>
+      </c>
+      <c r="C16" s="74" t="s">
+        <v>446</v>
+      </c>
+      <c r="D16" s="74" t="s">
+        <v>447</v>
+      </c>
+      <c r="E16" s="74" t="s">
+        <v>448</v>
+      </c>
+      <c r="F16" s="74" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="74" t="s">
+        <v>449</v>
+      </c>
+      <c r="H16" s="74" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="52" x14ac:dyDescent="0.2">
+      <c r="A17" s="91" t="s">
+        <v>451</v>
+      </c>
+      <c r="B17" s="71" t="s">
+        <v>452</v>
+      </c>
+      <c r="C17" s="71" t="s">
+        <v>453</v>
+      </c>
+      <c r="D17" s="71" t="s">
+        <v>457</v>
+      </c>
+      <c r="E17" s="71" t="s">
+        <v>454</v>
+      </c>
+      <c r="F17" s="71" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="71" t="s">
+        <v>442</v>
+      </c>
+      <c r="H17" s="71" t="s">
+        <v>455</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A12:H12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4167,333 +4882,333 @@
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>296</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
     </row>
     <row r="3" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="82" t="s">
+      <c r="A3" s="79" t="s">
         <v>297</v>
       </c>
-      <c r="B3" s="83"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="G4" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="22" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="19" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="73" t="s">
+      <c r="A6" s="70" t="s">
         <v>298</v>
       </c>
-      <c r="B6" s="74" t="s">
+      <c r="B6" s="71" t="s">
         <v>299</v>
       </c>
-      <c r="C6" s="75" t="s">
+      <c r="C6" s="72" t="s">
         <v>314</v>
       </c>
-      <c r="D6" s="74" t="s">
+      <c r="D6" s="71" t="s">
         <v>315</v>
       </c>
-      <c r="E6" s="74" t="s">
+      <c r="E6" s="71" t="s">
         <v>300</v>
       </c>
-      <c r="F6" s="74" t="s">
+      <c r="F6" s="71" t="s">
         <v>301</v>
       </c>
-      <c r="G6" s="74" t="s">
+      <c r="G6" s="71" t="s">
         <v>302</v>
       </c>
-      <c r="H6" s="74" t="s">
-        <v>462</v>
+      <c r="H6" s="71" t="s">
+        <v>458</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="76" t="s">
+      <c r="A7" s="73" t="s">
         <v>303</v>
       </c>
-      <c r="B7" s="77" t="s">
+      <c r="B7" s="74" t="s">
         <v>304</v>
       </c>
-      <c r="C7" s="78" t="s">
+      <c r="C7" s="75" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="77" t="s">
+      <c r="D7" s="74" t="s">
         <v>316</v>
       </c>
-      <c r="E7" s="77" t="s">
+      <c r="E7" s="74" t="s">
         <v>305</v>
       </c>
-      <c r="F7" s="77" t="s">
+      <c r="F7" s="74" t="s">
         <v>301</v>
       </c>
-      <c r="G7" s="77" t="s">
+      <c r="G7" s="74" t="s">
         <v>306</v>
       </c>
-      <c r="H7" s="77" t="s">
+      <c r="H7" s="74" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="79" t="s">
+      <c r="A8" s="76" t="s">
         <v>308</v>
       </c>
-      <c r="B8" s="74" t="s">
+      <c r="B8" s="71" t="s">
         <v>309</v>
       </c>
-      <c r="C8" s="80" t="s">
+      <c r="C8" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="74" t="s">
+      <c r="D8" s="71" t="s">
         <v>317</v>
       </c>
-      <c r="E8" s="74" t="s">
+      <c r="E8" s="71" t="s">
         <v>310</v>
       </c>
-      <c r="F8" s="74" t="s">
+      <c r="F8" s="71" t="s">
         <v>311</v>
       </c>
-      <c r="G8" s="74" t="s">
+      <c r="G8" s="71" t="s">
         <v>312</v>
       </c>
-      <c r="H8" s="74" t="s">
+      <c r="H8" s="71" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="89" t="s">
+      <c r="A10" s="86" t="s">
+        <v>471</v>
+      </c>
+      <c r="B10" s="87"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="87"/>
+      <c r="E10" s="87"/>
+      <c r="F10" s="87"/>
+      <c r="G10" s="87"/>
+      <c r="H10" s="87"/>
+      <c r="I10" s="87"/>
+      <c r="J10" s="88"/>
+    </row>
+    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="85" t="s">
         <v>320</v>
       </c>
-      <c r="B10" s="90"/>
-      <c r="C10" s="90"/>
-      <c r="D10" s="90"/>
-      <c r="E10" s="90"/>
-      <c r="F10" s="90"/>
-      <c r="G10" s="90"/>
-      <c r="H10" s="90"/>
-      <c r="I10" s="90"/>
-      <c r="J10" s="91"/>
-    </row>
-    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="88" t="s">
+      <c r="B11" s="85" t="s">
         <v>321</v>
       </c>
-      <c r="B11" s="88" t="s">
+      <c r="C11" s="85" t="s">
         <v>322</v>
       </c>
-      <c r="C11" s="88" t="s">
+      <c r="D11" s="85" t="s">
         <v>323</v>
       </c>
-      <c r="D11" s="88" t="s">
+      <c r="E11" s="85" t="s">
         <v>324</v>
       </c>
-      <c r="E11" s="88" t="s">
+      <c r="F11" s="85" t="s">
         <v>325</v>
       </c>
-      <c r="F11" s="88" t="s">
+      <c r="G11" s="85" t="s">
         <v>326</v>
       </c>
-      <c r="G11" s="88" t="s">
+      <c r="H11" s="85" t="s">
         <v>327</v>
       </c>
-      <c r="H11" s="88" t="s">
+      <c r="I11" s="85" t="s">
         <v>328</v>
       </c>
-      <c r="I11" s="88" t="s">
+      <c r="J11" s="85" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="81" t="s">
         <v>329</v>
       </c>
-      <c r="J11" s="88" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="84" t="s">
+      <c r="B12" s="74" t="s">
+        <v>361</v>
+      </c>
+      <c r="C12" s="74" t="s">
         <v>330</v>
       </c>
-      <c r="B12" s="77" t="s">
+      <c r="D12" s="74" t="s">
+        <v>331</v>
+      </c>
+      <c r="E12" s="74" t="s">
+        <v>332</v>
+      </c>
+      <c r="F12" s="74" t="s">
+        <v>333</v>
+      </c>
+      <c r="G12" s="74" t="s">
+        <v>334</v>
+      </c>
+      <c r="H12" s="74" t="s">
+        <v>335</v>
+      </c>
+      <c r="I12" s="74" t="s">
+        <v>336</v>
+      </c>
+      <c r="J12" s="74" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="82" t="s">
+        <v>337</v>
+      </c>
+      <c r="B13" s="71" t="s">
         <v>362</v>
       </c>
-      <c r="C12" s="77" t="s">
-        <v>331</v>
-      </c>
-      <c r="D12" s="77" t="s">
-        <v>332</v>
-      </c>
-      <c r="E12" s="77" t="s">
-        <v>333</v>
-      </c>
-      <c r="F12" s="77" t="s">
-        <v>334</v>
-      </c>
-      <c r="G12" s="77" t="s">
-        <v>335</v>
-      </c>
-      <c r="H12" s="77" t="s">
-        <v>336</v>
-      </c>
-      <c r="I12" s="77" t="s">
-        <v>337</v>
-      </c>
-      <c r="J12" s="77" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="85" t="s">
+      <c r="C13" s="71" t="s">
         <v>338</v>
       </c>
-      <c r="B13" s="74" t="s">
+      <c r="D13" s="71" t="s">
+        <v>339</v>
+      </c>
+      <c r="E13" s="71" t="s">
+        <v>340</v>
+      </c>
+      <c r="F13" s="71" t="s">
+        <v>341</v>
+      </c>
+      <c r="G13" s="71" t="s">
+        <v>342</v>
+      </c>
+      <c r="H13" s="71" t="s">
+        <v>343</v>
+      </c>
+      <c r="I13" s="71" t="s">
+        <v>344</v>
+      </c>
+      <c r="J13" s="71" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="83" t="s">
+        <v>345</v>
+      </c>
+      <c r="B14" s="74" t="s">
         <v>363</v>
       </c>
-      <c r="C13" s="74" t="s">
-        <v>339</v>
-      </c>
-      <c r="D13" s="74" t="s">
-        <v>340</v>
-      </c>
-      <c r="E13" s="74" t="s">
-        <v>341</v>
-      </c>
-      <c r="F13" s="74" t="s">
-        <v>342</v>
-      </c>
-      <c r="G13" s="74" t="s">
-        <v>343</v>
-      </c>
-      <c r="H13" s="74" t="s">
-        <v>344</v>
-      </c>
-      <c r="I13" s="74" t="s">
-        <v>345</v>
-      </c>
-      <c r="J13" s="74" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="86" t="s">
+      <c r="C14" s="74" t="s">
         <v>346</v>
       </c>
-      <c r="B14" s="77" t="s">
+      <c r="D14" s="74" t="s">
+        <v>347</v>
+      </c>
+      <c r="E14" s="74" t="s">
+        <v>348</v>
+      </c>
+      <c r="F14" s="74" t="s">
+        <v>349</v>
+      </c>
+      <c r="G14" s="74" t="s">
+        <v>350</v>
+      </c>
+      <c r="H14" s="74" t="s">
+        <v>351</v>
+      </c>
+      <c r="I14" s="74" t="s">
+        <v>352</v>
+      </c>
+      <c r="J14" s="74" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="84" t="s">
+        <v>353</v>
+      </c>
+      <c r="B15" s="71" t="s">
         <v>364</v>
       </c>
-      <c r="C14" s="77" t="s">
-        <v>347</v>
-      </c>
-      <c r="D14" s="77" t="s">
-        <v>348</v>
-      </c>
-      <c r="E14" s="77" t="s">
-        <v>349</v>
-      </c>
-      <c r="F14" s="77" t="s">
-        <v>350</v>
-      </c>
-      <c r="G14" s="77" t="s">
-        <v>351</v>
-      </c>
-      <c r="H14" s="77" t="s">
-        <v>352</v>
-      </c>
-      <c r="I14" s="77" t="s">
-        <v>353</v>
-      </c>
-      <c r="J14" s="77" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="87" t="s">
+      <c r="C15" s="71" t="s">
         <v>354</v>
       </c>
-      <c r="B15" s="74" t="s">
-        <v>365</v>
-      </c>
-      <c r="C15" s="74" t="s">
+      <c r="D15" s="71" t="s">
         <v>355</v>
       </c>
-      <c r="D15" s="74" t="s">
+      <c r="E15" s="71" t="s">
         <v>356</v>
       </c>
-      <c r="E15" s="74" t="s">
+      <c r="F15" s="71" t="s">
         <v>357</v>
       </c>
-      <c r="F15" s="74" t="s">
+      <c r="G15" s="71" t="s">
         <v>358</v>
       </c>
-      <c r="G15" s="74" t="s">
+      <c r="H15" s="71" t="s">
         <v>359</v>
       </c>
-      <c r="H15" s="74" t="s">
+      <c r="I15" s="71" t="s">
         <v>360</v>
       </c>
-      <c r="I15" s="74" t="s">
-        <v>361</v>
-      </c>
-      <c r="J15" s="74" t="s">
-        <v>361</v>
+      <c r="J15" s="71" t="s">
+        <v>360</v>
       </c>
     </row>
   </sheetData>
@@ -4506,364 +5221,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D072851C-E33D-3E4C-9E1E-B705D90C883D}">
-  <dimension ref="A1:H17"/>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B78A3055-C56F-CB41-83BE-657DC6F2B5A1}">
+  <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.6640625" customWidth="1"/>
-    <col min="2" max="2" width="24.1640625" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="21.83203125" customWidth="1"/>
-    <col min="5" max="5" width="39" customWidth="1"/>
-    <col min="6" max="6" width="28.5" customWidth="1"/>
-    <col min="7" max="7" width="24.5" customWidth="1"/>
-    <col min="8" max="8" width="38" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="95" t="s">
-        <v>404</v>
-      </c>
-      <c r="B2" s="96"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="89" t="s">
-        <v>405</v>
-      </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="88" t="s">
-        <v>366</v>
-      </c>
-      <c r="B4" s="88" t="s">
-        <v>367</v>
-      </c>
-      <c r="C4" s="88" t="s">
-        <v>368</v>
-      </c>
-      <c r="D4" s="88" t="s">
-        <v>369</v>
-      </c>
-      <c r="E4" s="88" t="s">
-        <v>370</v>
-      </c>
-      <c r="F4" s="88" t="s">
-        <v>371</v>
-      </c>
-      <c r="G4" s="88" t="s">
-        <v>372</v>
-      </c>
-      <c r="H4" s="88" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="92" t="s">
-        <v>77</v>
-      </c>
-      <c r="B5" s="77" t="s">
-        <v>374</v>
-      </c>
-      <c r="C5" s="77" t="s">
-        <v>375</v>
-      </c>
-      <c r="D5" s="77" t="s">
-        <v>403</v>
-      </c>
-      <c r="E5" s="77" t="s">
-        <v>376</v>
-      </c>
-      <c r="F5" s="77" t="s">
-        <v>377</v>
-      </c>
-      <c r="G5" s="93" t="s">
-        <v>378</v>
-      </c>
-      <c r="H5" s="80" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="71" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="94" t="s">
-        <v>379</v>
-      </c>
-      <c r="B6" s="74" t="s">
-        <v>380</v>
-      </c>
-      <c r="C6" s="74" t="s">
-        <v>381</v>
-      </c>
-      <c r="D6" s="74" t="s">
-        <v>407</v>
-      </c>
-      <c r="E6" s="74" t="s">
-        <v>382</v>
-      </c>
-      <c r="F6" s="74" t="s">
-        <v>383</v>
-      </c>
-      <c r="G6" s="93" t="s">
-        <v>384</v>
-      </c>
-      <c r="H6" s="80" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="92" t="s">
-        <v>140</v>
-      </c>
-      <c r="B7" s="77" t="s">
-        <v>386</v>
-      </c>
-      <c r="C7" s="77" t="s">
-        <v>387</v>
-      </c>
-      <c r="D7" s="77" t="s">
-        <v>408</v>
-      </c>
-      <c r="E7" s="77" t="s">
-        <v>388</v>
-      </c>
-      <c r="F7" s="77" t="s">
-        <v>389</v>
-      </c>
-      <c r="G7" s="93" t="s">
-        <v>390</v>
-      </c>
-      <c r="H7" s="80" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="94" t="s">
-        <v>164</v>
-      </c>
-      <c r="B8" s="74" t="s">
-        <v>409</v>
-      </c>
-      <c r="C8" s="74" t="s">
-        <v>392</v>
-      </c>
-      <c r="D8" s="74" t="s">
-        <v>410</v>
-      </c>
-      <c r="E8" s="74" t="s">
-        <v>393</v>
-      </c>
-      <c r="F8" s="74" t="s">
-        <v>394</v>
-      </c>
-      <c r="G8" s="93" t="s">
-        <v>395</v>
-      </c>
-      <c r="H8" s="80" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="92" t="s">
-        <v>397</v>
-      </c>
-      <c r="B9" s="77" t="s">
-        <v>398</v>
-      </c>
-      <c r="C9" s="77" t="s">
-        <v>381</v>
-      </c>
-      <c r="D9" s="77" t="s">
-        <v>411</v>
-      </c>
-      <c r="E9" s="77" t="s">
-        <v>399</v>
-      </c>
-      <c r="F9" s="77" t="s">
-        <v>400</v>
-      </c>
-      <c r="G9" s="93" t="s">
-        <v>401</v>
-      </c>
-      <c r="H9" s="80" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="89" t="s">
-        <v>460</v>
-      </c>
-      <c r="B12" s="90"/>
-      <c r="C12" s="90"/>
-      <c r="D12" s="90"/>
-      <c r="E12" s="90"/>
-      <c r="F12" s="90"/>
-      <c r="G12" s="90"/>
-      <c r="H12" s="90"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="88" t="s">
-        <v>426</v>
-      </c>
-      <c r="B13" s="88" t="s">
-        <v>427</v>
-      </c>
-      <c r="C13" s="88" t="s">
-        <v>428</v>
-      </c>
-      <c r="D13" s="88" t="s">
-        <v>429</v>
-      </c>
-      <c r="E13" s="88" t="s">
-        <v>430</v>
-      </c>
-      <c r="F13" s="88" t="s">
-        <v>431</v>
-      </c>
-      <c r="G13" s="88" t="s">
-        <v>432</v>
-      </c>
-      <c r="H13" s="88" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="78" x14ac:dyDescent="0.2">
-      <c r="A14" s="92" t="s">
-        <v>434</v>
-      </c>
-      <c r="B14" s="77" t="s">
-        <v>435</v>
-      </c>
-      <c r="C14" s="77" t="s">
-        <v>436</v>
-      </c>
-      <c r="D14" s="77" t="s">
-        <v>437</v>
-      </c>
-      <c r="E14" s="77" t="s">
-        <v>438</v>
-      </c>
-      <c r="F14" s="77" t="s">
-        <v>17</v>
-      </c>
-      <c r="G14" s="77" t="s">
-        <v>439</v>
-      </c>
-      <c r="H14" s="77" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="52" x14ac:dyDescent="0.2">
-      <c r="A15" s="94" t="s">
-        <v>441</v>
-      </c>
-      <c r="B15" s="74" t="s">
-        <v>442</v>
-      </c>
-      <c r="C15" s="74" t="s">
-        <v>443</v>
-      </c>
-      <c r="D15" s="74" t="s">
-        <v>444</v>
-      </c>
-      <c r="E15" s="74" t="s">
-        <v>445</v>
-      </c>
-      <c r="F15" s="74" t="s">
-        <v>26</v>
-      </c>
-      <c r="G15" s="74" t="s">
-        <v>446</v>
-      </c>
-      <c r="H15" s="74" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="52" x14ac:dyDescent="0.2">
-      <c r="A16" s="92" t="s">
-        <v>448</v>
-      </c>
-      <c r="B16" s="77" t="s">
-        <v>449</v>
-      </c>
-      <c r="C16" s="77" t="s">
-        <v>450</v>
-      </c>
-      <c r="D16" s="77" t="s">
-        <v>451</v>
-      </c>
-      <c r="E16" s="77" t="s">
-        <v>452</v>
-      </c>
-      <c r="F16" s="77" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16" s="77" t="s">
-        <v>453</v>
-      </c>
-      <c r="H16" s="77" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="52" x14ac:dyDescent="0.2">
-      <c r="A17" s="94" t="s">
-        <v>455</v>
-      </c>
-      <c r="B17" s="74" t="s">
-        <v>456</v>
-      </c>
-      <c r="C17" s="74" t="s">
-        <v>457</v>
-      </c>
-      <c r="D17" s="74" t="s">
-        <v>461</v>
-      </c>
-      <c r="E17" s="74" t="s">
-        <v>458</v>
-      </c>
-      <c r="F17" s="74" t="s">
-        <v>17</v>
-      </c>
-      <c r="G17" s="74" t="s">
-        <v>446</v>
-      </c>
-      <c r="H17" s="74" t="s">
-        <v>459</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A12:H12"/>
-  </mergeCells>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9578EDDF-5D6A-9145-9892-C45CF7563863}">
   <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4881,512 +5248,512 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="107" t="s">
         <v>291</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="56" t="s">
         <v>237</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="60" t="s">
+      <c r="B5" s="58" t="s">
         <v>238</v>
       </c>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="61" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="60" t="s">
+      <c r="B6" s="58" t="s">
         <v>239</v>
       </c>
-      <c r="C6" s="59"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
-      <c r="F6" s="59"/>
-      <c r="G6" s="59"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="65" t="s">
+      <c r="A7" s="62" t="s">
         <v>95</v>
       </c>
-      <c r="B7" s="60" t="s">
+      <c r="B7" s="58" t="s">
         <v>240</v>
       </c>
-      <c r="C7" s="59"/>
-      <c r="D7" s="59"/>
-      <c r="E7" s="59"/>
-      <c r="F7" s="59"/>
-      <c r="G7" s="59"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="57"/>
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="57"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="66" t="s">
+      <c r="A8" s="63" t="s">
         <v>150</v>
       </c>
-      <c r="B8" s="60" t="s">
+      <c r="B8" s="58" t="s">
         <v>241</v>
       </c>
-      <c r="C8" s="59"/>
-      <c r="D8" s="59"/>
-      <c r="E8" s="59"/>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="57"/>
+      <c r="E8" s="57"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="57"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="67" t="s">
+      <c r="A9" s="64" t="s">
         <v>175</v>
       </c>
-      <c r="B9" s="60" t="s">
+      <c r="B9" s="58" t="s">
         <v>242</v>
       </c>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="57"/>
+      <c r="E9" s="57"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="57"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="65" t="s">
         <v>194</v>
       </c>
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="58" t="s">
         <v>243</v>
       </c>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="57"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="58" t="s">
+      <c r="A12" s="106" t="s">
         <v>244</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
+      <c r="B12" s="78"/>
+      <c r="C12" s="78"/>
+      <c r="D12" s="78"/>
+      <c r="E12" s="78"/>
+      <c r="F12" s="78"/>
+      <c r="G12" s="78"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="60" t="s">
+      <c r="B13" s="58" t="s">
         <v>245</v>
       </c>
-      <c r="C13" s="59"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="59"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="57"/>
+      <c r="F13" s="57"/>
+      <c r="G13" s="57"/>
     </row>
     <row r="14" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="69" t="s">
+      <c r="A14" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="60" t="s">
+      <c r="B14" s="58" t="s">
         <v>246</v>
       </c>
-      <c r="C14" s="59"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="59"/>
-      <c r="F14" s="59"/>
-      <c r="G14" s="59"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="70" t="s">
+      <c r="A15" s="67" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="60" t="s">
+      <c r="B15" s="58" t="s">
         <v>247</v>
       </c>
-      <c r="C15" s="59"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="59"/>
-      <c r="F15" s="59"/>
-      <c r="G15" s="59"/>
+      <c r="C15" s="57"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="57"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
     </row>
     <row r="16" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="71" t="s">
+      <c r="A16" s="68" t="s">
         <v>248</v>
       </c>
-      <c r="B16" s="60" t="s">
+      <c r="B16" s="58" t="s">
         <v>249</v>
       </c>
-      <c r="C16" s="59"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="59"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="59"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="57"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="57"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="58" t="s">
+      <c r="A18" s="106" t="s">
         <v>250</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
+      <c r="B18" s="78"/>
+      <c r="C18" s="78"/>
+      <c r="D18" s="78"/>
+      <c r="E18" s="78"/>
+      <c r="F18" s="78"/>
+      <c r="G18" s="78"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="70" t="s">
+      <c r="A19" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="58" t="s">
         <v>292</v>
       </c>
-      <c r="C19" s="59"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="59"/>
-      <c r="F19" s="59"/>
-      <c r="G19" s="59"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="57"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="69" t="s">
+      <c r="A20" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="60" t="s">
+      <c r="B20" s="58" t="s">
         <v>251</v>
       </c>
-      <c r="C20" s="59"/>
-      <c r="D20" s="59"/>
-      <c r="E20" s="59"/>
-      <c r="F20" s="59"/>
-      <c r="G20" s="59"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="57"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="71" t="s">
+      <c r="A21" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="60" t="s">
+      <c r="B21" s="58" t="s">
         <v>252</v>
       </c>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="59"/>
+      <c r="C21" s="57"/>
+      <c r="D21" s="57"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="58" t="s">
+      <c r="A23" s="106" t="s">
         <v>253</v>
       </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
+      <c r="B23" s="78"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
+      <c r="G23" s="78"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" s="71" t="s">
+      <c r="A24" s="68" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="60" t="s">
+      <c r="B24" s="58" t="s">
         <v>293</v>
       </c>
-      <c r="C24" s="59"/>
-      <c r="D24" s="59"/>
-      <c r="E24" s="59"/>
-      <c r="F24" s="59"/>
-      <c r="G24" s="59"/>
+      <c r="C24" s="57"/>
+      <c r="D24" s="57"/>
+      <c r="E24" s="57"/>
+      <c r="F24" s="57"/>
+      <c r="G24" s="57"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" s="70" t="s">
+      <c r="A25" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="60" t="s">
+      <c r="B25" s="58" t="s">
         <v>294</v>
       </c>
-      <c r="C25" s="59"/>
-      <c r="D25" s="59"/>
-      <c r="E25" s="59"/>
-      <c r="F25" s="59"/>
-      <c r="G25" s="59"/>
+      <c r="C25" s="57"/>
+      <c r="D25" s="57"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="57"/>
+      <c r="G25" s="57"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="69" t="s">
+      <c r="A26" s="66" t="s">
         <v>89</v>
       </c>
-      <c r="B26" s="60" t="s">
+      <c r="B26" s="58" t="s">
         <v>295</v>
       </c>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="59"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="58" t="s">
+      <c r="A28" s="106" t="s">
         <v>254</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="78"/>
+      <c r="F28" s="78"/>
+      <c r="G28" s="78"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="72" t="s">
+      <c r="A29" s="69" t="s">
         <v>255</v>
       </c>
-      <c r="B29" s="61" t="s">
+      <c r="B29" s="59" t="s">
         <v>256</v>
       </c>
-      <c r="C29" s="59"/>
-      <c r="D29" s="59"/>
-      <c r="E29" s="59"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="59"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="57"/>
+      <c r="E29" s="57"/>
+      <c r="F29" s="57"/>
+      <c r="G29" s="57"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" s="72" t="s">
+      <c r="A30" s="69" t="s">
         <v>257</v>
       </c>
-      <c r="B30" s="61" t="s">
+      <c r="B30" s="59" t="s">
         <v>258</v>
       </c>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="59"/>
-      <c r="F30" s="59"/>
-      <c r="G30" s="59"/>
+      <c r="C30" s="57"/>
+      <c r="D30" s="57"/>
+      <c r="E30" s="57"/>
+      <c r="F30" s="57"/>
+      <c r="G30" s="57"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" s="72" t="s">
+      <c r="A31" s="69" t="s">
         <v>259</v>
       </c>
-      <c r="B31" s="61" t="s">
+      <c r="B31" s="59" t="s">
         <v>260</v>
       </c>
-      <c r="C31" s="59"/>
-      <c r="D31" s="59"/>
-      <c r="E31" s="59"/>
-      <c r="F31" s="59"/>
-      <c r="G31" s="59"/>
+      <c r="C31" s="57"/>
+      <c r="D31" s="57"/>
+      <c r="E31" s="57"/>
+      <c r="F31" s="57"/>
+      <c r="G31" s="57"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A32" s="72" t="s">
+      <c r="A32" s="69" t="s">
         <v>261</v>
       </c>
-      <c r="B32" s="61" t="s">
+      <c r="B32" s="59" t="s">
         <v>262</v>
       </c>
-      <c r="C32" s="59"/>
-      <c r="D32" s="59"/>
-      <c r="E32" s="59"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="59"/>
+      <c r="C32" s="57"/>
+      <c r="D32" s="57"/>
+      <c r="E32" s="57"/>
+      <c r="F32" s="57"/>
+      <c r="G32" s="57"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" s="72" t="s">
+      <c r="A33" s="69" t="s">
         <v>263</v>
       </c>
-      <c r="B33" s="61" t="s">
+      <c r="B33" s="59" t="s">
         <v>264</v>
       </c>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-      <c r="E33" s="59"/>
-      <c r="F33" s="59"/>
-      <c r="G33" s="59"/>
+      <c r="C33" s="57"/>
+      <c r="D33" s="57"/>
+      <c r="E33" s="57"/>
+      <c r="F33" s="57"/>
+      <c r="G33" s="57"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="72" t="s">
+      <c r="A34" s="69" t="s">
         <v>265</v>
       </c>
-      <c r="B34" s="61" t="s">
+      <c r="B34" s="59" t="s">
         <v>266</v>
       </c>
-      <c r="C34" s="59"/>
-      <c r="D34" s="59"/>
-      <c r="E34" s="59"/>
-      <c r="F34" s="59"/>
-      <c r="G34" s="59"/>
+      <c r="C34" s="57"/>
+      <c r="D34" s="57"/>
+      <c r="E34" s="57"/>
+      <c r="F34" s="57"/>
+      <c r="G34" s="57"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="72" t="s">
+      <c r="A35" s="69" t="s">
         <v>267</v>
       </c>
-      <c r="B35" s="61" t="s">
+      <c r="B35" s="59" t="s">
         <v>268</v>
       </c>
-      <c r="C35" s="59"/>
-      <c r="D35" s="59"/>
-      <c r="E35" s="59"/>
-      <c r="F35" s="59"/>
-      <c r="G35" s="59"/>
+      <c r="C35" s="57"/>
+      <c r="D35" s="57"/>
+      <c r="E35" s="57"/>
+      <c r="F35" s="57"/>
+      <c r="G35" s="57"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="72" t="s">
+      <c r="A36" s="69" t="s">
         <v>269</v>
       </c>
-      <c r="B36" s="61" t="s">
+      <c r="B36" s="59" t="s">
         <v>270</v>
       </c>
-      <c r="C36" s="59"/>
-      <c r="D36" s="59"/>
-      <c r="E36" s="59"/>
-      <c r="F36" s="59"/>
-      <c r="G36" s="59"/>
+      <c r="C36" s="57"/>
+      <c r="D36" s="57"/>
+      <c r="E36" s="57"/>
+      <c r="F36" s="57"/>
+      <c r="G36" s="57"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="72" t="s">
+      <c r="A37" s="69" t="s">
         <v>271</v>
       </c>
-      <c r="B37" s="61" t="s">
+      <c r="B37" s="59" t="s">
         <v>272</v>
       </c>
-      <c r="C37" s="59"/>
-      <c r="D37" s="59"/>
-      <c r="E37" s="59"/>
-      <c r="F37" s="59"/>
-      <c r="G37" s="59"/>
+      <c r="C37" s="57"/>
+      <c r="D37" s="57"/>
+      <c r="E37" s="57"/>
+      <c r="F37" s="57"/>
+      <c r="G37" s="57"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="72" t="s">
+      <c r="A38" s="69" t="s">
         <v>273</v>
       </c>
-      <c r="B38" s="61" t="s">
+      <c r="B38" s="59" t="s">
         <v>274</v>
       </c>
-      <c r="C38" s="59"/>
-      <c r="D38" s="59"/>
-      <c r="E38" s="59"/>
-      <c r="F38" s="59"/>
-      <c r="G38" s="59"/>
+      <c r="C38" s="57"/>
+      <c r="D38" s="57"/>
+      <c r="E38" s="57"/>
+      <c r="F38" s="57"/>
+      <c r="G38" s="57"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="72" t="s">
+      <c r="A39" s="69" t="s">
         <v>275</v>
       </c>
-      <c r="B39" s="61" t="s">
+      <c r="B39" s="59" t="s">
         <v>276</v>
       </c>
-      <c r="C39" s="59"/>
-      <c r="D39" s="59"/>
-      <c r="E39" s="59"/>
-      <c r="F39" s="59"/>
-      <c r="G39" s="59"/>
+      <c r="C39" s="57"/>
+      <c r="D39" s="57"/>
+      <c r="E39" s="57"/>
+      <c r="F39" s="57"/>
+      <c r="G39" s="57"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" s="72" t="s">
+      <c r="A40" s="69" t="s">
         <v>277</v>
       </c>
-      <c r="B40" s="61" t="s">
+      <c r="B40" s="59" t="s">
         <v>278</v>
       </c>
-      <c r="C40" s="59"/>
-      <c r="D40" s="59"/>
-      <c r="E40" s="59"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="59"/>
+      <c r="C40" s="57"/>
+      <c r="D40" s="57"/>
+      <c r="E40" s="57"/>
+      <c r="F40" s="57"/>
+      <c r="G40" s="57"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="72" t="s">
+      <c r="A41" s="69" t="s">
         <v>279</v>
       </c>
-      <c r="B41" s="61" t="s">
+      <c r="B41" s="59" t="s">
         <v>280</v>
       </c>
-      <c r="C41" s="59"/>
-      <c r="D41" s="59"/>
-      <c r="E41" s="59"/>
-      <c r="F41" s="59"/>
-      <c r="G41" s="59"/>
+      <c r="C41" s="57"/>
+      <c r="D41" s="57"/>
+      <c r="E41" s="57"/>
+      <c r="F41" s="57"/>
+      <c r="G41" s="57"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="72" t="s">
+      <c r="A42" s="69" t="s">
         <v>281</v>
       </c>
-      <c r="B42" s="61" t="s">
+      <c r="B42" s="59" t="s">
         <v>282</v>
       </c>
-      <c r="C42" s="59"/>
-      <c r="D42" s="59"/>
-      <c r="E42" s="59"/>
-      <c r="F42" s="59"/>
-      <c r="G42" s="59"/>
+      <c r="C42" s="57"/>
+      <c r="D42" s="57"/>
+      <c r="E42" s="57"/>
+      <c r="F42" s="57"/>
+      <c r="G42" s="57"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="72" t="s">
+      <c r="A43" s="69" t="s">
         <v>283</v>
       </c>
-      <c r="B43" s="61" t="s">
+      <c r="B43" s="59" t="s">
         <v>284</v>
       </c>
-      <c r="C43" s="59"/>
-      <c r="D43" s="59"/>
-      <c r="E43" s="59"/>
-      <c r="F43" s="59"/>
-      <c r="G43" s="59"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="57"/>
+      <c r="E43" s="57"/>
+      <c r="F43" s="57"/>
+      <c r="G43" s="57"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="72" t="s">
+      <c r="A44" s="69" t="s">
         <v>285</v>
       </c>
-      <c r="B44" s="61" t="s">
+      <c r="B44" s="59" t="s">
         <v>286</v>
       </c>
-      <c r="C44" s="59"/>
-      <c r="D44" s="59"/>
-      <c r="E44" s="59"/>
-      <c r="F44" s="59"/>
-      <c r="G44" s="59"/>
+      <c r="C44" s="57"/>
+      <c r="D44" s="57"/>
+      <c r="E44" s="57"/>
+      <c r="F44" s="57"/>
+      <c r="G44" s="57"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" s="72" t="s">
+      <c r="A45" s="69" t="s">
         <v>287</v>
       </c>
-      <c r="B45" s="61" t="s">
+      <c r="B45" s="59" t="s">
         <v>288</v>
       </c>
-      <c r="C45" s="59"/>
-      <c r="D45" s="59"/>
-      <c r="E45" s="59"/>
-      <c r="F45" s="59"/>
-      <c r="G45" s="59"/>
+      <c r="C45" s="57"/>
+      <c r="D45" s="57"/>
+      <c r="E45" s="57"/>
+      <c r="F45" s="57"/>
+      <c r="G45" s="57"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" s="72" t="s">
+      <c r="A46" s="69" t="s">
         <v>289</v>
       </c>
-      <c r="B46" s="61" t="s">
+      <c r="B46" s="59" t="s">
         <v>290</v>
       </c>
-      <c r="C46" s="59"/>
-      <c r="D46" s="59"/>
-      <c r="E46" s="59"/>
-      <c r="F46" s="59"/>
-      <c r="G46" s="59"/>
+      <c r="C46" s="57"/>
+      <c r="D46" s="57"/>
+      <c r="E46" s="57"/>
+      <c r="F46" s="57"/>
+      <c r="G46" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="40">

</xml_diff>

<commit_message>
Fixed Evidence Tracker sheet
</commit_message>
<xml_diff>
--- a/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
+++ b/SEBI_CSCRF_CIS_Controls_Crosswalk_v1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\CSCRF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronityadav/Documents/CSCRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06845035-913A-471C-A090-B82E57D77338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{986ED400-1590-CE44-970F-61FFB0076C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="8" r:id="rId1"/>
@@ -1651,9 +1651,6 @@
     <t>SEBI CSCRF  :  CIS Controls v8.1</t>
   </si>
   <si>
-    <t>SEBI CSCRF 2024 - Circular No. SEBI/HO/ITD-LE/CYS/P/CIR/2024/163 dated August 20, 2024</t>
-  </si>
-  <si>
     <t>CIS Controls v8.1 (2024) - Center for Internet Security</t>
   </si>
   <si>
@@ -1794,6 +1791,9 @@
   <si>
     <t>Instructions: Complete one row per control mapping. 
 Status: Not Started | In Progress | Evidence Collected | Auditor Reviewed | Closed</t>
+  </si>
+  <si>
+    <t>SEBI CSCRF 2024 - Circular No. SEBI/HO/ ITD-1/ITD_CSC_EXT/P/CIR/2024/113 dated August 20, 2024</t>
   </si>
 </sst>
 </file>
@@ -1813,73 +1813,86 @@
       <sz val="9"/>
       <color rgb="FF0B1F3A"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF6B7F93"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF1C2B3A"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF1A3A5C"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF4A6480"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF1C5C1C"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color rgb="FF7C4A00"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF1C2B3A"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF7C4A00"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color rgb="FF1A3A5C"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8.5"/>
       <color rgb="FF1C2B3A"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8.5"/>
       <color rgb="FF1A3A5C"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -2542,42 +2555,66 @@
     <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="57" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="52" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="51" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="52" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="54" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="32" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2588,15 +2625,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2613,35 +2641,20 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="41" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2951,18 +2964,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB9251F8-4A3E-BF4A-BD2B-E73CDC9A5F26}">
   <dimension ref="A2:M27"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.109375" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="1" max="1" width="16.1640625" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" customWidth="1"/>
+    <col min="5" max="5" width="17.1640625" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" customWidth="1"/>
-    <col min="11" max="11" width="15.109375" customWidth="1"/>
-    <col min="12" max="12" width="13.109375" customWidth="1"/>
+    <col min="11" max="11" width="15.1640625" customWidth="1"/>
+    <col min="12" max="12" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="64"/>
       <c r="B2" s="64"/>
       <c r="C2" s="64"/>
@@ -2977,116 +2990,116 @@
       <c r="L2" s="64"/>
       <c r="M2" s="64"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="64"/>
-      <c r="B3" s="80" t="s">
+      <c r="B3" s="89" t="s">
         <v>463</v>
       </c>
-      <c r="C3" s="79"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79"/>
-      <c r="L3" s="79"/>
-      <c r="M3" s="79"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="84"/>
+      <c r="I3" s="84"/>
+      <c r="J3" s="84"/>
+      <c r="K3" s="84"/>
+      <c r="L3" s="84"/>
+      <c r="M3" s="84"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="64"/>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
-      <c r="L4" s="79"/>
-      <c r="M4" s="79"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B4" s="84"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="84"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="84"/>
+      <c r="H4" s="84"/>
+      <c r="I4" s="84"/>
+      <c r="J4" s="84"/>
+      <c r="K4" s="84"/>
+      <c r="L4" s="84"/>
+      <c r="M4" s="84"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="64"/>
-      <c r="B5" s="79"/>
-      <c r="C5" s="79"/>
-      <c r="D5" s="79"/>
-      <c r="E5" s="79"/>
-      <c r="F5" s="79"/>
-      <c r="G5" s="79"/>
-      <c r="H5" s="79"/>
-      <c r="I5" s="79"/>
-      <c r="J5" s="79"/>
-      <c r="K5" s="79"/>
-      <c r="L5" s="79"/>
-      <c r="M5" s="79"/>
-    </row>
-    <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="84"/>
+      <c r="C5" s="84"/>
+      <c r="D5" s="84"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+      <c r="I5" s="84"/>
+      <c r="J5" s="84"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="84"/>
+    </row>
+    <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="64"/>
-      <c r="B6" s="79"/>
-      <c r="C6" s="79"/>
-      <c r="D6" s="79"/>
-      <c r="E6" s="79"/>
-      <c r="F6" s="79"/>
-      <c r="G6" s="79"/>
-      <c r="H6" s="79"/>
-      <c r="I6" s="79"/>
-      <c r="J6" s="79"/>
-      <c r="K6" s="79"/>
-      <c r="L6" s="79"/>
-      <c r="M6" s="79"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="84"/>
+      <c r="C6" s="84"/>
+      <c r="D6" s="84"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="84"/>
+      <c r="G6" s="84"/>
+      <c r="H6" s="84"/>
+      <c r="I6" s="84"/>
+      <c r="J6" s="84"/>
+      <c r="K6" s="84"/>
+      <c r="L6" s="84"/>
+      <c r="M6" s="84"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="64"/>
-      <c r="B7" s="81" t="s">
+      <c r="B7" s="90" t="s">
         <v>459</v>
       </c>
-      <c r="C7" s="76"/>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
-      <c r="I7" s="76"/>
-      <c r="J7" s="76"/>
-      <c r="K7" s="76"/>
-      <c r="L7" s="76"/>
-      <c r="M7" s="76"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C7" s="86"/>
+      <c r="D7" s="86"/>
+      <c r="E7" s="86"/>
+      <c r="F7" s="86"/>
+      <c r="G7" s="86"/>
+      <c r="H7" s="86"/>
+      <c r="I7" s="86"/>
+      <c r="J7" s="86"/>
+      <c r="K7" s="86"/>
+      <c r="L7" s="86"/>
+      <c r="M7" s="86"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="64"/>
-      <c r="B8" s="76"/>
-      <c r="C8" s="76"/>
-      <c r="D8" s="76"/>
-      <c r="E8" s="76"/>
-      <c r="F8" s="76"/>
-      <c r="G8" s="76"/>
-      <c r="H8" s="76"/>
-      <c r="I8" s="76"/>
-      <c r="J8" s="76"/>
-      <c r="K8" s="76"/>
-      <c r="L8" s="76"/>
-      <c r="M8" s="76"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B8" s="86"/>
+      <c r="C8" s="86"/>
+      <c r="D8" s="86"/>
+      <c r="E8" s="86"/>
+      <c r="F8" s="86"/>
+      <c r="G8" s="86"/>
+      <c r="H8" s="86"/>
+      <c r="I8" s="86"/>
+      <c r="J8" s="86"/>
+      <c r="K8" s="86"/>
+      <c r="L8" s="86"/>
+      <c r="M8" s="86"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="64"/>
-      <c r="B9" s="76"/>
-      <c r="C9" s="76"/>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
-      <c r="F9" s="76"/>
-      <c r="G9" s="76"/>
-      <c r="H9" s="76"/>
-      <c r="I9" s="76"/>
-      <c r="J9" s="76"/>
-      <c r="K9" s="76"/>
-      <c r="L9" s="76"/>
-      <c r="M9" s="76"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B9" s="86"/>
+      <c r="C9" s="86"/>
+      <c r="D9" s="86"/>
+      <c r="E9" s="86"/>
+      <c r="F9" s="86"/>
+      <c r="G9" s="86"/>
+      <c r="H9" s="86"/>
+      <c r="I9" s="86"/>
+      <c r="J9" s="86"/>
+      <c r="K9" s="86"/>
+      <c r="L9" s="86"/>
+      <c r="M9" s="86"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="64"/>
       <c r="B10" s="64"/>
       <c r="C10" s="64"/>
@@ -3101,115 +3114,115 @@
       <c r="L10" s="64"/>
       <c r="M10" s="64"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="64"/>
-      <c r="B11" s="78" t="s">
+      <c r="B11" s="83" t="s">
         <v>460</v>
       </c>
-      <c r="C11" s="79"/>
-      <c r="D11" s="79"/>
-      <c r="E11" s="77" t="s">
+      <c r="C11" s="84"/>
+      <c r="D11" s="84"/>
+      <c r="E11" s="85" t="s">
+        <v>511</v>
+      </c>
+      <c r="F11" s="86"/>
+      <c r="G11" s="86"/>
+      <c r="H11" s="86"/>
+      <c r="I11" s="86"/>
+      <c r="J11" s="86"/>
+      <c r="K11" s="86"/>
+      <c r="L11" s="86"/>
+      <c r="M11" s="86"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" s="64"/>
+      <c r="B12" s="83" t="s">
+        <v>461</v>
+      </c>
+      <c r="C12" s="84"/>
+      <c r="D12" s="84"/>
+      <c r="E12" s="85" t="s">
         <v>464</v>
       </c>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="76"/>
-      <c r="I11" s="76"/>
-      <c r="J11" s="76"/>
-      <c r="K11" s="76"/>
-      <c r="L11" s="76"/>
-      <c r="M11" s="76"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="64"/>
-      <c r="B12" s="78" t="s">
-        <v>461</v>
-      </c>
-      <c r="C12" s="79"/>
-      <c r="D12" s="79"/>
-      <c r="E12" s="77" t="s">
+      <c r="F12" s="86"/>
+      <c r="G12" s="86"/>
+      <c r="H12" s="86"/>
+      <c r="I12" s="86"/>
+      <c r="J12" s="86"/>
+      <c r="K12" s="86"/>
+      <c r="L12" s="86"/>
+      <c r="M12" s="86"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="64"/>
+      <c r="B13" s="83" t="s">
+        <v>462</v>
+      </c>
+      <c r="C13" s="84"/>
+      <c r="D13" s="84"/>
+      <c r="E13" s="85" t="s">
         <v>465</v>
       </c>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="76"/>
-      <c r="I12" s="76"/>
-      <c r="J12" s="76"/>
-      <c r="K12" s="76"/>
-      <c r="L12" s="76"/>
-      <c r="M12" s="76"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="64"/>
-      <c r="B13" s="78" t="s">
-        <v>462</v>
-      </c>
-      <c r="C13" s="79"/>
-      <c r="D13" s="79"/>
-      <c r="E13" s="77" t="s">
+      <c r="F13" s="86"/>
+      <c r="G13" s="86"/>
+      <c r="H13" s="86"/>
+      <c r="I13" s="86"/>
+      <c r="J13" s="86"/>
+      <c r="K13" s="86"/>
+      <c r="L13" s="86"/>
+      <c r="M13" s="86"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="64"/>
+      <c r="B14" s="83" t="s">
         <v>466</v>
       </c>
-      <c r="F13" s="76"/>
-      <c r="G13" s="76"/>
-      <c r="H13" s="76"/>
-      <c r="I13" s="76"/>
-      <c r="J13" s="76"/>
-      <c r="K13" s="76"/>
-      <c r="L13" s="76"/>
-      <c r="M13" s="76"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="64"/>
-      <c r="B14" s="78" t="s">
+      <c r="C14" s="84"/>
+      <c r="D14" s="84"/>
+      <c r="E14" s="85" t="s">
+        <v>469</v>
+      </c>
+      <c r="F14" s="86"/>
+      <c r="G14" s="86"/>
+      <c r="H14" s="86"/>
+      <c r="I14" s="86"/>
+      <c r="J14" s="86"/>
+      <c r="K14" s="86"/>
+      <c r="L14" s="86"/>
+      <c r="M14" s="86"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" s="64"/>
+      <c r="B15" s="83" t="s">
         <v>467</v>
       </c>
-      <c r="C14" s="79"/>
-      <c r="D14" s="79"/>
-      <c r="E14" s="77" t="s">
-        <v>470</v>
-      </c>
-      <c r="F14" s="76"/>
-      <c r="G14" s="76"/>
-      <c r="H14" s="76"/>
-      <c r="I14" s="76"/>
-      <c r="J14" s="76"/>
-      <c r="K14" s="76"/>
-      <c r="L14" s="76"/>
-      <c r="M14" s="76"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="64"/>
-      <c r="B15" s="78" t="s">
-        <v>468</v>
-      </c>
-      <c r="C15" s="79"/>
-      <c r="D15" s="79"/>
-      <c r="E15" s="77"/>
-      <c r="F15" s="76"/>
-      <c r="G15" s="76"/>
-      <c r="H15" s="76"/>
-      <c r="I15" s="76"/>
-      <c r="J15" s="76"/>
-      <c r="K15" s="76"/>
-      <c r="L15" s="76"/>
-      <c r="M15" s="76"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C15" s="84"/>
+      <c r="D15" s="84"/>
+      <c r="E15" s="85"/>
+      <c r="F15" s="86"/>
+      <c r="G15" s="86"/>
+      <c r="H15" s="86"/>
+      <c r="I15" s="86"/>
+      <c r="J15" s="86"/>
+      <c r="K15" s="86"/>
+      <c r="L15" s="86"/>
+      <c r="M15" s="86"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="64"/>
-      <c r="B16" s="75"/>
-      <c r="C16" s="76"/>
-      <c r="D16" s="76"/>
-      <c r="E16" s="77"/>
-      <c r="F16" s="76"/>
-      <c r="G16" s="76"/>
-      <c r="H16" s="76"/>
-      <c r="I16" s="76"/>
-      <c r="J16" s="76"/>
-      <c r="K16" s="76"/>
-      <c r="L16" s="76"/>
-      <c r="M16" s="76"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B16" s="91"/>
+      <c r="C16" s="86"/>
+      <c r="D16" s="86"/>
+      <c r="E16" s="85"/>
+      <c r="F16" s="86"/>
+      <c r="G16" s="86"/>
+      <c r="H16" s="86"/>
+      <c r="I16" s="86"/>
+      <c r="J16" s="86"/>
+      <c r="K16" s="86"/>
+      <c r="L16" s="86"/>
+      <c r="M16" s="86"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="64"/>
       <c r="B17" s="64"/>
       <c r="C17" s="64"/>
@@ -3224,7 +3237,7 @@
       <c r="L17" s="64"/>
       <c r="M17" s="64"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="64"/>
       <c r="B18" s="64"/>
       <c r="C18" s="64"/>
@@ -3239,7 +3252,7 @@
       <c r="L18" s="64"/>
       <c r="M18" s="64"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="64"/>
       <c r="B19" s="64"/>
       <c r="C19" s="64"/>
@@ -3254,7 +3267,7 @@
       <c r="L19" s="64"/>
       <c r="M19" s="64"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="64"/>
       <c r="B20" s="64"/>
       <c r="C20" s="64"/>
@@ -3269,120 +3282,120 @@
       <c r="L20" s="64"/>
       <c r="M20" s="64"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="86" t="s">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" s="80" t="s">
         <v>411</v>
       </c>
-      <c r="B22" s="86"/>
-      <c r="C22" s="86"/>
-      <c r="D22" s="86"/>
-      <c r="E22" s="86"/>
-      <c r="F22" s="86"/>
-      <c r="G22" s="86"/>
-      <c r="H22" s="86"/>
-      <c r="I22" s="86"/>
-      <c r="J22" s="86"/>
-      <c r="K22" s="86"/>
-      <c r="L22" s="86"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" s="82" t="s">
+      <c r="B22" s="80"/>
+      <c r="C22" s="80"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="80"/>
+      <c r="F22" s="80"/>
+      <c r="G22" s="80"/>
+      <c r="H22" s="80"/>
+      <c r="I22" s="80"/>
+      <c r="J22" s="80"/>
+      <c r="K22" s="80"/>
+      <c r="L22" s="80"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" s="81" t="s">
         <v>415</v>
       </c>
-      <c r="B23" s="82"/>
-      <c r="C23" s="82"/>
-      <c r="D23" s="83" t="s">
+      <c r="B23" s="81"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="82" t="s">
         <v>420</v>
       </c>
-      <c r="E23" s="83"/>
-      <c r="F23" s="83"/>
-      <c r="G23" s="83"/>
-      <c r="H23" s="83"/>
-      <c r="I23" s="83"/>
-      <c r="J23" s="83"/>
-      <c r="K23" s="83"/>
-      <c r="L23" s="83"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="84" t="s">
+      <c r="E23" s="82"/>
+      <c r="F23" s="82"/>
+      <c r="G23" s="82"/>
+      <c r="H23" s="82"/>
+      <c r="I23" s="82"/>
+      <c r="J23" s="82"/>
+      <c r="K23" s="82"/>
+      <c r="L23" s="82"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" s="87" t="s">
         <v>416</v>
       </c>
-      <c r="B24" s="84"/>
-      <c r="C24" s="84"/>
-      <c r="D24" s="85" t="s">
+      <c r="B24" s="87"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="88" t="s">
         <v>412</v>
       </c>
-      <c r="E24" s="85"/>
-      <c r="F24" s="85"/>
-      <c r="G24" s="85"/>
-      <c r="H24" s="85"/>
-      <c r="I24" s="85"/>
-      <c r="J24" s="85"/>
-      <c r="K24" s="85"/>
-      <c r="L24" s="85"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="82" t="s">
+      <c r="E24" s="88"/>
+      <c r="F24" s="88"/>
+      <c r="G24" s="88"/>
+      <c r="H24" s="88"/>
+      <c r="I24" s="88"/>
+      <c r="J24" s="88"/>
+      <c r="K24" s="88"/>
+      <c r="L24" s="88"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="81" t="s">
         <v>417</v>
       </c>
-      <c r="B25" s="82"/>
-      <c r="C25" s="82"/>
-      <c r="D25" s="83" t="s">
+      <c r="B25" s="81"/>
+      <c r="C25" s="81"/>
+      <c r="D25" s="82" t="s">
         <v>421</v>
       </c>
-      <c r="E25" s="83"/>
-      <c r="F25" s="83"/>
-      <c r="G25" s="83"/>
-      <c r="H25" s="83"/>
-      <c r="I25" s="83"/>
-      <c r="J25" s="83"/>
-      <c r="K25" s="83"/>
-      <c r="L25" s="83"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="84" t="s">
+      <c r="E25" s="82"/>
+      <c r="F25" s="82"/>
+      <c r="G25" s="82"/>
+      <c r="H25" s="82"/>
+      <c r="I25" s="82"/>
+      <c r="J25" s="82"/>
+      <c r="K25" s="82"/>
+      <c r="L25" s="82"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" s="87" t="s">
         <v>418</v>
       </c>
-      <c r="B26" s="84"/>
-      <c r="C26" s="84"/>
-      <c r="D26" s="85" t="s">
+      <c r="B26" s="87"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="88" t="s">
         <v>413</v>
       </c>
-      <c r="E26" s="85"/>
-      <c r="F26" s="85"/>
-      <c r="G26" s="85"/>
-      <c r="H26" s="85"/>
-      <c r="I26" s="85"/>
-      <c r="J26" s="85"/>
-      <c r="K26" s="85"/>
-      <c r="L26" s="85"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" s="82" t="s">
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
+      <c r="G26" s="88"/>
+      <c r="H26" s="88"/>
+      <c r="I26" s="88"/>
+      <c r="J26" s="88"/>
+      <c r="K26" s="88"/>
+      <c r="L26" s="88"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A27" s="81" t="s">
         <v>419</v>
       </c>
-      <c r="B27" s="82"/>
-      <c r="C27" s="82"/>
-      <c r="D27" s="83" t="s">
+      <c r="B27" s="81"/>
+      <c r="C27" s="81"/>
+      <c r="D27" s="82" t="s">
         <v>414</v>
       </c>
-      <c r="E27" s="83"/>
-      <c r="F27" s="83"/>
-      <c r="G27" s="83"/>
-      <c r="H27" s="83"/>
-      <c r="I27" s="83"/>
-      <c r="J27" s="83"/>
-      <c r="K27" s="83"/>
-      <c r="L27" s="83"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="82"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="82"/>
+      <c r="J27" s="82"/>
+      <c r="K27" s="82"/>
+      <c r="L27" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="D23:L23"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:M13"/>
-    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B3:M6"/>
+    <mergeCell ref="B7:M9"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E11:M11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="E12:M12"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="D27:L27"/>
     <mergeCell ref="A24:C24"/>
@@ -3391,12 +3404,12 @@
     <mergeCell ref="D25:L25"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="D26:L26"/>
-    <mergeCell ref="B3:M6"/>
-    <mergeCell ref="B7:M9"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E11:M11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="E12:M12"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D23:L23"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:M13"/>
+    <mergeCell ref="B14:D14"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="E16:M16"/>
     <mergeCell ref="E14:M14"/>
@@ -3410,7 +3423,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K40"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -3425,7 +3438,7 @@
     <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3438,37 +3451,37 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="93" t="s">
+    <row r="2" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="92" t="s">
         <v>214</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
-      <c r="J2" s="88"/>
-      <c r="K2" s="88"/>
-    </row>
-    <row r="3" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="92" t="s">
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="93"/>
+    </row>
+    <row r="3" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="100" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="88"/>
-      <c r="I3" s="88"/>
-      <c r="J3" s="88"/>
-      <c r="K3" s="88"/>
-    </row>
-    <row r="4" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="93"/>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
+      <c r="J3" s="93"/>
+      <c r="K3" s="93"/>
+    </row>
+    <row r="4" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="74" t="s">
         <v>0</v>
       </c>
@@ -3503,22 +3516,22 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="91" t="s">
+    <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="99" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="88"/>
-      <c r="C5" s="88"/>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="88"/>
-      <c r="K5" s="88"/>
-    </row>
-    <row r="6" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="93"/>
+      <c r="C5" s="93"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="93"/>
+      <c r="K5" s="93"/>
+    </row>
+    <row r="6" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
@@ -3553,7 +3566,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -3588,7 +3601,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -3623,7 +3636,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -3658,22 +3671,22 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="94" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="88"/>
-      <c r="C10" s="88"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="88"/>
-      <c r="F10" s="88"/>
-      <c r="G10" s="88"/>
-      <c r="H10" s="88"/>
-      <c r="I10" s="88"/>
-      <c r="J10" s="88"/>
-      <c r="K10" s="88"/>
-    </row>
-    <row r="11" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
+      <c r="H10" s="93"/>
+      <c r="I10" s="93"/>
+      <c r="J10" s="93"/>
+      <c r="K10" s="93"/>
+    </row>
+    <row r="11" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="23" t="s">
         <v>62</v>
       </c>
@@ -3708,7 +3721,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="23" t="s">
         <v>62</v>
       </c>
@@ -3743,7 +3756,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
         <v>62</v>
       </c>
@@ -3778,7 +3791,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
         <v>62</v>
       </c>
@@ -3813,7 +3826,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
         <v>62</v>
       </c>
@@ -3848,22 +3861,22 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="95" t="s">
         <v>163</v>
       </c>
-      <c r="B16" s="88"/>
-      <c r="C16" s="88"/>
-      <c r="D16" s="88"/>
-      <c r="E16" s="88"/>
-      <c r="F16" s="88"/>
-      <c r="G16" s="88"/>
-      <c r="H16" s="88"/>
-      <c r="I16" s="88"/>
-      <c r="J16" s="88"/>
-      <c r="K16" s="88"/>
-    </row>
-    <row r="17" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="93"/>
+      <c r="C16" s="93"/>
+      <c r="D16" s="93"/>
+      <c r="E16" s="93"/>
+      <c r="F16" s="93"/>
+      <c r="G16" s="93"/>
+      <c r="H16" s="93"/>
+      <c r="I16" s="93"/>
+      <c r="J16" s="93"/>
+      <c r="K16" s="93"/>
+    </row>
+    <row r="17" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="43" t="s">
         <v>150</v>
       </c>
@@ -3898,7 +3911,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="43" t="s">
         <v>150</v>
       </c>
@@ -3933,7 +3946,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="43" t="s">
         <v>150</v>
       </c>
@@ -3968,7 +3981,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="43" t="s">
         <v>150</v>
       </c>
@@ -4003,22 +4016,22 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="87" t="s">
+    <row r="21" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="96" t="s">
         <v>193</v>
       </c>
-      <c r="B21" s="88"/>
-      <c r="C21" s="88"/>
-      <c r="D21" s="88"/>
-      <c r="E21" s="88"/>
-      <c r="F21" s="88"/>
-      <c r="G21" s="88"/>
-      <c r="H21" s="88"/>
-      <c r="I21" s="88"/>
-      <c r="J21" s="88"/>
-      <c r="K21" s="88"/>
-    </row>
-    <row r="22" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="93"/>
+      <c r="C21" s="93"/>
+      <c r="D21" s="93"/>
+      <c r="E21" s="93"/>
+      <c r="F21" s="93"/>
+      <c r="G21" s="93"/>
+      <c r="H21" s="93"/>
+      <c r="I21" s="93"/>
+      <c r="J21" s="93"/>
+      <c r="K21" s="93"/>
+    </row>
+    <row r="22" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="44" t="s">
         <v>175</v>
       </c>
@@ -4053,7 +4066,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="44" t="s">
         <v>175</v>
       </c>
@@ -4088,7 +4101,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="44" t="s">
         <v>175</v>
       </c>
@@ -4123,7 +4136,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="44" t="s">
         <v>175</v>
       </c>
@@ -4158,22 +4171,22 @@
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="89" t="s">
+    <row r="26" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="97" t="s">
         <v>149</v>
       </c>
-      <c r="B26" s="88"/>
-      <c r="C26" s="88"/>
-      <c r="D26" s="88"/>
-      <c r="E26" s="88"/>
-      <c r="F26" s="88"/>
-      <c r="G26" s="88"/>
-      <c r="H26" s="88"/>
-      <c r="I26" s="88"/>
-      <c r="J26" s="88"/>
-      <c r="K26" s="88"/>
-    </row>
-    <row r="27" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="93"/>
+      <c r="C26" s="93"/>
+      <c r="D26" s="93"/>
+      <c r="E26" s="93"/>
+      <c r="F26" s="93"/>
+      <c r="G26" s="93"/>
+      <c r="H26" s="93"/>
+      <c r="I26" s="93"/>
+      <c r="J26" s="93"/>
+      <c r="K26" s="93"/>
+    </row>
+    <row r="27" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="42" t="s">
         <v>95</v>
       </c>
@@ -4208,7 +4221,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="42" t="s">
         <v>95</v>
       </c>
@@ -4243,7 +4256,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="42" t="s">
         <v>95</v>
       </c>
@@ -4278,7 +4291,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="42" t="s">
         <v>95</v>
       </c>
@@ -4313,7 +4326,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="42" t="s">
         <v>95</v>
       </c>
@@ -4348,7 +4361,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="42" t="s">
         <v>95</v>
       </c>
@@ -4383,7 +4396,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="42" t="s">
         <v>95</v>
       </c>
@@ -4418,7 +4431,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="42" t="s">
         <v>95</v>
       </c>
@@ -4453,7 +4466,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="42" t="s">
         <v>95</v>
       </c>
@@ -4488,22 +4501,22 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="90" t="s">
+    <row r="36" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="98" t="s">
         <v>213</v>
       </c>
-      <c r="B36" s="88"/>
-      <c r="C36" s="88"/>
-      <c r="D36" s="88"/>
-      <c r="E36" s="88"/>
-      <c r="F36" s="88"/>
-      <c r="G36" s="88"/>
-      <c r="H36" s="88"/>
-      <c r="I36" s="88"/>
-      <c r="J36" s="88"/>
-      <c r="K36" s="88"/>
-    </row>
-    <row r="37" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="93"/>
+      <c r="C36" s="93"/>
+      <c r="D36" s="93"/>
+      <c r="E36" s="93"/>
+      <c r="F36" s="93"/>
+      <c r="G36" s="93"/>
+      <c r="H36" s="93"/>
+      <c r="I36" s="93"/>
+      <c r="J36" s="93"/>
+      <c r="K36" s="93"/>
+    </row>
+    <row r="37" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="45" t="s">
         <v>194</v>
       </c>
@@ -4538,7 +4551,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="45" t="s">
         <v>194</v>
       </c>
@@ -4573,7 +4586,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="45" t="s">
         <v>194</v>
       </c>
@@ -4608,7 +4621,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="45" t="s">
         <v>194</v>
       </c>
@@ -4645,14 +4658,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="A3:K3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A10:K10"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A21:K21"/>
     <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A36:K36"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4661,19 +4674,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D072851C-E33D-3E4C-9E1E-B705D90C883D}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" customWidth="1"/>
-    <col min="4" max="4" width="21.77734375" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="21.83203125" customWidth="1"/>
     <col min="5" max="5" width="39" customWidth="1"/>
-    <col min="6" max="6" width="28.44140625" customWidth="1"/>
-    <col min="7" max="7" width="24.44140625" customWidth="1"/>
+    <col min="6" max="6" width="28.5" customWidth="1"/>
+    <col min="7" max="7" width="24.5" customWidth="1"/>
     <col min="8" max="8" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4683,31 +4696,31 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="96" t="s">
+    <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="101" t="s">
         <v>403</v>
       </c>
-      <c r="B2" s="97"/>
-      <c r="C2" s="97"/>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="98" t="s">
+      <c r="B2" s="102"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="103" t="s">
         <v>404</v>
       </c>
-      <c r="B3" s="99"/>
-      <c r="C3" s="99"/>
-      <c r="D3" s="99"/>
-      <c r="E3" s="99"/>
-      <c r="F3" s="99"/>
-      <c r="G3" s="99"/>
-      <c r="H3" s="99"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B3" s="104"/>
+      <c r="C3" s="104"/>
+      <c r="D3" s="104"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="104"/>
+      <c r="H3" s="104"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="69" t="s">
         <v>365</v>
       </c>
@@ -4733,7 +4746,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="67.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="71" t="s">
         <v>77</v>
       </c>
@@ -4759,7 +4772,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="71" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="73" t="s">
         <v>378</v>
       </c>
@@ -4785,7 +4798,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="71" t="s">
         <v>140</v>
       </c>
@@ -4811,7 +4824,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="73" t="s">
         <v>164</v>
       </c>
@@ -4837,7 +4850,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="67.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="71" t="s">
         <v>396</v>
       </c>
@@ -4863,19 +4876,19 @@
         <v>401</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="98" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="103" t="s">
         <v>456</v>
       </c>
-      <c r="B12" s="99"/>
-      <c r="C12" s="99"/>
-      <c r="D12" s="99"/>
-      <c r="E12" s="99"/>
-      <c r="F12" s="99"/>
-      <c r="G12" s="99"/>
-      <c r="H12" s="99"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B12" s="104"/>
+      <c r="C12" s="104"/>
+      <c r="D12" s="104"/>
+      <c r="E12" s="104"/>
+      <c r="F12" s="104"/>
+      <c r="G12" s="104"/>
+      <c r="H12" s="104"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="69" t="s">
         <v>422</v>
       </c>
@@ -4901,7 +4914,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="64.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="78" x14ac:dyDescent="0.2">
       <c r="A14" s="71" t="s">
         <v>430</v>
       </c>
@@ -4927,7 +4940,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="52" x14ac:dyDescent="0.2">
       <c r="A15" s="73" t="s">
         <v>437</v>
       </c>
@@ -4953,7 +4966,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="52" x14ac:dyDescent="0.2">
       <c r="A16" s="71" t="s">
         <v>444</v>
       </c>
@@ -4979,7 +4992,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="52" x14ac:dyDescent="0.2">
       <c r="A17" s="73" t="s">
         <v>451</v>
       </c>
@@ -5018,20 +5031,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J15"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" customWidth="1"/>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
     <col min="6" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="27.6640625" customWidth="1"/>
-    <col min="9" max="9" width="0.109375" customWidth="1"/>
+    <col min="9" max="9" width="0.1640625" customWidth="1"/>
     <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5041,33 +5054,33 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="101" t="s">
+    <row r="2" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="106" t="s">
         <v>296</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
-    </row>
-    <row r="3" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="100" t="s">
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+    </row>
+    <row r="3" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="105" t="s">
         <v>297</v>
       </c>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-    </row>
-    <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="84"/>
+      <c r="I3" s="84"/>
+    </row>
+    <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
         <v>44</v>
       </c>
@@ -5093,7 +5106,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
         <v>52</v>
       </c>
@@ -5119,7 +5132,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="56" t="s">
         <v>298</v>
       </c>
@@ -5145,7 +5158,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="59" t="s">
         <v>303</v>
       </c>
@@ -5171,7 +5184,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="62" t="s">
         <v>308</v>
       </c>
@@ -5197,21 +5210,21 @@
         <v>313</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="98" t="s">
-        <v>469</v>
-      </c>
-      <c r="B10" s="99"/>
-      <c r="C10" s="99"/>
-      <c r="D10" s="99"/>
-      <c r="E10" s="99"/>
-      <c r="F10" s="99"/>
-      <c r="G10" s="99"/>
-      <c r="H10" s="99"/>
-      <c r="I10" s="99"/>
+    <row r="10" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="103" t="s">
+        <v>468</v>
+      </c>
+      <c r="B10" s="104"/>
+      <c r="C10" s="104"/>
+      <c r="D10" s="104"/>
+      <c r="E10" s="104"/>
+      <c r="F10" s="104"/>
+      <c r="G10" s="104"/>
+      <c r="H10" s="104"/>
+      <c r="I10" s="104"/>
       <c r="J10" s="70"/>
     </row>
-    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="69" t="s">
         <v>320</v>
       </c>
@@ -5243,7 +5256,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="65" t="s">
         <v>329</v>
       </c>
@@ -5275,7 +5288,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="66" t="s">
         <v>337</v>
       </c>
@@ -5307,7 +5320,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="67" t="s">
         <v>345</v>
       </c>
@@ -5339,7 +5352,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="68" t="s">
         <v>353</v>
       </c>
@@ -5384,88 +5397,88 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B78A3055-C56F-CB41-83BE-657DC6F2B5A1}">
   <dimension ref="A1:L17"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="25.2" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="25.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.109375" style="111" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.1640625" style="79" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="104" t="s">
+    <row r="1" spans="1:12" ht="25.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="107" t="s">
+        <v>470</v>
+      </c>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
+      <c r="K1" s="86"/>
+      <c r="L1" s="86"/>
+    </row>
+    <row r="2" spans="1:12" ht="25.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="108" t="s">
+        <v>510</v>
+      </c>
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="93"/>
+      <c r="L2" s="93"/>
+    </row>
+    <row r="3" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="78" t="s">
         <v>471</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-    </row>
-    <row r="2" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="110" t="s">
-        <v>511</v>
-      </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
-      <c r="J2" s="88"/>
-      <c r="K2" s="88"/>
-      <c r="L2" s="88"/>
-    </row>
-    <row r="3" spans="1:12" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="109" t="s">
+      <c r="B3" s="78" t="s">
         <v>472</v>
       </c>
-      <c r="B3" s="109" t="s">
+      <c r="C3" s="78" t="s">
+        <v>422</v>
+      </c>
+      <c r="D3" s="78" t="s">
         <v>473</v>
       </c>
-      <c r="C3" s="109" t="s">
-        <v>422</v>
-      </c>
-      <c r="D3" s="109" t="s">
+      <c r="E3" s="78" t="s">
         <v>474</v>
       </c>
-      <c r="E3" s="109" t="s">
+      <c r="F3" s="78" t="s">
         <v>475</v>
       </c>
-      <c r="F3" s="109" t="s">
+      <c r="G3" s="78" t="s">
         <v>476</v>
       </c>
-      <c r="G3" s="109" t="s">
+      <c r="H3" s="78" t="s">
         <v>477</v>
       </c>
-      <c r="H3" s="109" t="s">
+      <c r="I3" s="78" t="s">
+        <v>328</v>
+      </c>
+      <c r="J3" s="78" t="s">
         <v>478</v>
       </c>
-      <c r="I3" s="109" t="s">
-        <v>328</v>
-      </c>
-      <c r="J3" s="109" t="s">
+      <c r="K3" s="78" t="s">
         <v>479</v>
       </c>
-      <c r="K3" s="109" t="s">
+      <c r="L3" s="78" t="s">
         <v>480</v>
       </c>
-      <c r="L3" s="109" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="71" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C4" s="60" t="s">
         <v>14</v>
@@ -5473,27 +5486,27 @@
       <c r="D4" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="106" t="s">
+      <c r="E4" s="75" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="60" t="s">
+        <v>482</v>
+      </c>
+      <c r="G4" s="60"/>
+      <c r="H4" s="76" t="s">
         <v>483</v>
-      </c>
-      <c r="G4" s="60"/>
-      <c r="H4" s="107" t="s">
-        <v>484</v>
       </c>
       <c r="I4" s="60"/>
       <c r="J4" s="60"/>
       <c r="K4" s="60"/>
       <c r="L4" s="60"/>
     </row>
-    <row r="5" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="73" t="s">
         <v>77</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C5" s="57" t="s">
         <v>79</v>
@@ -5505,79 +5518,79 @@
         <v>85</v>
       </c>
       <c r="F5" s="57" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="G5" s="57"/>
-      <c r="H5" s="107" t="s">
-        <v>484</v>
+      <c r="H5" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I5" s="57"/>
       <c r="J5" s="57"/>
       <c r="K5" s="57"/>
       <c r="L5" s="57"/>
     </row>
-    <row r="6" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="71" t="s">
         <v>96</v>
       </c>
       <c r="B6" s="60" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C6" s="60" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="108" t="s">
+      <c r="D6" s="77" t="s">
         <v>34</v>
       </c>
       <c r="E6" s="62" t="s">
         <v>85</v>
       </c>
       <c r="F6" s="60" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G6" s="60"/>
-      <c r="H6" s="107" t="s">
-        <v>484</v>
+      <c r="H6" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I6" s="60"/>
       <c r="J6" s="60"/>
       <c r="K6" s="60"/>
       <c r="L6" s="60"/>
     </row>
-    <row r="7" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="73" t="s">
         <v>109</v>
       </c>
       <c r="B7" s="57" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C7" s="57" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="108" t="s">
+      <c r="D7" s="77" t="s">
         <v>34</v>
       </c>
       <c r="E7" s="62" t="s">
         <v>85</v>
       </c>
       <c r="F7" s="57" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G7" s="57"/>
-      <c r="H7" s="107" t="s">
-        <v>484</v>
+      <c r="H7" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I7" s="57"/>
       <c r="J7" s="57"/>
       <c r="K7" s="57"/>
       <c r="L7" s="57"/>
     </row>
-    <row r="8" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="71" t="s">
         <v>140</v>
       </c>
       <c r="B8" s="60" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C8" s="60" t="s">
         <v>135</v>
@@ -5589,26 +5602,26 @@
         <v>85</v>
       </c>
       <c r="F8" s="60" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G8" s="60"/>
-      <c r="H8" s="107" t="s">
-        <v>484</v>
+      <c r="H8" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I8" s="60"/>
       <c r="J8" s="60"/>
       <c r="K8" s="60"/>
       <c r="L8" s="60"/>
     </row>
-    <row r="9" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="73" t="s">
         <v>164</v>
       </c>
       <c r="B9" s="57" t="s">
+        <v>492</v>
+      </c>
+      <c r="C9" s="57" t="s">
         <v>493</v>
-      </c>
-      <c r="C9" s="57" t="s">
-        <v>494</v>
       </c>
       <c r="D9" s="72" t="s">
         <v>83</v>
@@ -5617,51 +5630,51 @@
         <v>85</v>
       </c>
       <c r="F9" s="57" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G9" s="57"/>
-      <c r="H9" s="107" t="s">
-        <v>484</v>
+      <c r="H9" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I9" s="57"/>
       <c r="J9" s="57"/>
       <c r="K9" s="57"/>
       <c r="L9" s="57"/>
     </row>
-    <row r="10" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="71" t="s">
         <v>151</v>
       </c>
       <c r="B10" s="60" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C10" s="60" t="s">
         <v>153</v>
       </c>
-      <c r="D10" s="108" t="s">
+      <c r="D10" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="106" t="s">
+      <c r="E10" s="75" t="s">
         <v>21</v>
       </c>
       <c r="F10" s="60" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="G10" s="60"/>
-      <c r="H10" s="107" t="s">
-        <v>484</v>
+      <c r="H10" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I10" s="60"/>
       <c r="J10" s="60"/>
       <c r="K10" s="60"/>
       <c r="L10" s="60"/>
     </row>
-    <row r="11" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="73" t="s">
         <v>176</v>
       </c>
       <c r="B11" s="57" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C11" s="57" t="s">
         <v>14</v>
@@ -5673,23 +5686,23 @@
         <v>85</v>
       </c>
       <c r="F11" s="57" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G11" s="57"/>
-      <c r="H11" s="107" t="s">
-        <v>484</v>
+      <c r="H11" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I11" s="57"/>
       <c r="J11" s="57"/>
       <c r="K11" s="57"/>
       <c r="L11" s="57"/>
     </row>
-    <row r="12" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="71" t="s">
         <v>180</v>
       </c>
       <c r="B12" s="60" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C12" s="60" t="s">
         <v>14</v>
@@ -5701,18 +5714,18 @@
         <v>85</v>
       </c>
       <c r="F12" s="60" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G12" s="60"/>
-      <c r="H12" s="107" t="s">
-        <v>484</v>
+      <c r="H12" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I12" s="60"/>
       <c r="J12" s="60"/>
       <c r="K12" s="60"/>
       <c r="L12" s="60"/>
     </row>
-    <row r="13" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="73" t="s">
         <v>190</v>
       </c>
@@ -5729,51 +5742,51 @@
         <v>85</v>
       </c>
       <c r="F13" s="57" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G13" s="57"/>
-      <c r="H13" s="107" t="s">
-        <v>484</v>
+      <c r="H13" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I13" s="57"/>
       <c r="J13" s="57"/>
       <c r="K13" s="57"/>
       <c r="L13" s="57"/>
     </row>
-    <row r="14" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="71" t="s">
         <v>195</v>
       </c>
       <c r="B14" s="60" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C14" s="60" t="s">
         <v>197</v>
       </c>
-      <c r="D14" s="108" t="s">
+      <c r="D14" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="106" t="s">
+      <c r="E14" s="75" t="s">
         <v>21</v>
       </c>
       <c r="F14" s="60" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="G14" s="60"/>
-      <c r="H14" s="107" t="s">
-        <v>484</v>
+      <c r="H14" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I14" s="60"/>
       <c r="J14" s="60"/>
       <c r="K14" s="60"/>
       <c r="L14" s="60"/>
     </row>
-    <row r="15" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="73" t="s">
         <v>208</v>
       </c>
       <c r="B15" s="57" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C15" s="57" t="s">
         <v>79</v>
@@ -5785,23 +5798,23 @@
         <v>85</v>
       </c>
       <c r="F15" s="57" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="G15" s="57"/>
-      <c r="H15" s="107" t="s">
-        <v>484</v>
+      <c r="H15" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I15" s="57"/>
       <c r="J15" s="57"/>
       <c r="K15" s="57"/>
       <c r="L15" s="57"/>
     </row>
-    <row r="16" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="71" t="s">
         <v>378</v>
       </c>
       <c r="B16" s="60" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C16" s="60" t="s">
         <v>135</v>
@@ -5809,27 +5822,27 @@
       <c r="D16" s="72" t="s">
         <v>83</v>
       </c>
-      <c r="E16" s="106" t="s">
+      <c r="E16" s="75" t="s">
         <v>21</v>
       </c>
       <c r="F16" s="60" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="G16" s="60"/>
-      <c r="H16" s="107" t="s">
-        <v>484</v>
+      <c r="H16" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I16" s="60"/>
       <c r="J16" s="60"/>
       <c r="K16" s="60"/>
       <c r="L16" s="60"/>
     </row>
-    <row r="17" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="73" t="s">
         <v>396</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C17" s="57" t="s">
         <v>170</v>
@@ -5837,15 +5850,15 @@
       <c r="D17" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="E17" s="106" t="s">
+      <c r="E17" s="75" t="s">
         <v>21</v>
       </c>
       <c r="F17" s="57" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="G17" s="57"/>
-      <c r="H17" s="107" t="s">
-        <v>484</v>
+      <c r="H17" s="76" t="s">
+        <v>483</v>
       </c>
       <c r="I17" s="57"/>
       <c r="J17" s="57"/>
@@ -5864,12 +5877,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9578EDDF-5D6A-9145-9892-C45CF7563863}">
   <dimension ref="A1:G46"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="8" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5878,522 +5891,538 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="104" t="s">
+    <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="107" t="s">
         <v>291</v>
       </c>
-      <c r="B2" s="76"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="105" t="s">
+      <c r="B2" s="86"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="110" t="s">
         <v>237</v>
       </c>
-      <c r="B4" s="88"/>
-      <c r="C4" s="88"/>
-      <c r="D4" s="88"/>
-      <c r="E4" s="88"/>
-      <c r="F4" s="88"/>
-      <c r="G4" s="88"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B4" s="93"/>
+      <c r="C4" s="93"/>
+      <c r="D4" s="93"/>
+      <c r="E4" s="93"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="93"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="102" t="s">
+      <c r="B5" s="109" t="s">
         <v>238</v>
       </c>
-      <c r="C5" s="88"/>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="88"/>
-      <c r="G5" s="88"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C5" s="93"/>
+      <c r="D5" s="93"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="102" t="s">
+      <c r="B6" s="109" t="s">
         <v>239</v>
       </c>
-      <c r="C6" s="88"/>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C6" s="93"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="B7" s="102" t="s">
+      <c r="B7" s="109" t="s">
         <v>240</v>
       </c>
-      <c r="C7" s="88"/>
-      <c r="D7" s="88"/>
-      <c r="E7" s="88"/>
-      <c r="F7" s="88"/>
-      <c r="G7" s="88"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C7" s="93"/>
+      <c r="D7" s="93"/>
+      <c r="E7" s="93"/>
+      <c r="F7" s="93"/>
+      <c r="G7" s="93"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="49" t="s">
         <v>150</v>
       </c>
-      <c r="B8" s="102" t="s">
+      <c r="B8" s="109" t="s">
         <v>241</v>
       </c>
-      <c r="C8" s="88"/>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C8" s="93"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="50" t="s">
         <v>175</v>
       </c>
-      <c r="B9" s="102" t="s">
+      <c r="B9" s="109" t="s">
         <v>242</v>
       </c>
-      <c r="C9" s="88"/>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C9" s="93"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="51" t="s">
         <v>194</v>
       </c>
-      <c r="B10" s="102" t="s">
+      <c r="B10" s="109" t="s">
         <v>243</v>
       </c>
-      <c r="C10" s="88"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="88"/>
-      <c r="F10" s="88"/>
-      <c r="G10" s="88"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="103" t="s">
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="111" t="s">
         <v>244</v>
       </c>
-      <c r="B12" s="76"/>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="76"/>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B12" s="86"/>
+      <c r="C12" s="86"/>
+      <c r="D12" s="86"/>
+      <c r="E12" s="86"/>
+      <c r="F12" s="86"/>
+      <c r="G12" s="86"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="102" t="s">
+      <c r="B13" s="109" t="s">
         <v>245</v>
       </c>
-      <c r="C13" s="88"/>
-      <c r="D13" s="88"/>
-      <c r="E13" s="88"/>
-      <c r="F13" s="88"/>
-      <c r="G13" s="88"/>
-    </row>
-    <row r="14" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="93"/>
+      <c r="D13" s="93"/>
+      <c r="E13" s="93"/>
+      <c r="F13" s="93"/>
+      <c r="G13" s="93"/>
+    </row>
+    <row r="14" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="102" t="s">
+      <c r="B14" s="109" t="s">
         <v>246</v>
       </c>
-      <c r="C14" s="88"/>
-      <c r="D14" s="88"/>
-      <c r="E14" s="88"/>
-      <c r="F14" s="88"/>
-      <c r="G14" s="88"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C14" s="93"/>
+      <c r="D14" s="93"/>
+      <c r="E14" s="93"/>
+      <c r="F14" s="93"/>
+      <c r="G14" s="93"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="102" t="s">
+      <c r="B15" s="109" t="s">
         <v>247</v>
       </c>
-      <c r="C15" s="88"/>
-      <c r="D15" s="88"/>
-      <c r="E15" s="88"/>
-      <c r="F15" s="88"/>
-      <c r="G15" s="88"/>
-    </row>
-    <row r="16" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="93"/>
+      <c r="D15" s="93"/>
+      <c r="E15" s="93"/>
+      <c r="F15" s="93"/>
+      <c r="G15" s="93"/>
+    </row>
+    <row r="16" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="54" t="s">
         <v>248</v>
       </c>
-      <c r="B16" s="102" t="s">
+      <c r="B16" s="109" t="s">
         <v>249</v>
       </c>
-      <c r="C16" s="88"/>
-      <c r="D16" s="88"/>
-      <c r="E16" s="88"/>
-      <c r="F16" s="88"/>
-      <c r="G16" s="88"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="103" t="s">
+      <c r="C16" s="93"/>
+      <c r="D16" s="93"/>
+      <c r="E16" s="93"/>
+      <c r="F16" s="93"/>
+      <c r="G16" s="93"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="111" t="s">
         <v>250</v>
       </c>
-      <c r="B18" s="76"/>
-      <c r="C18" s="76"/>
-      <c r="D18" s="76"/>
-      <c r="E18" s="76"/>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B18" s="86"/>
+      <c r="C18" s="86"/>
+      <c r="D18" s="86"/>
+      <c r="E18" s="86"/>
+      <c r="F18" s="86"/>
+      <c r="G18" s="86"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="102" t="s">
+      <c r="B19" s="109" t="s">
         <v>292</v>
       </c>
-      <c r="C19" s="88"/>
-      <c r="D19" s="88"/>
-      <c r="E19" s="88"/>
-      <c r="F19" s="88"/>
-      <c r="G19" s="88"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C19" s="93"/>
+      <c r="D19" s="93"/>
+      <c r="E19" s="93"/>
+      <c r="F19" s="93"/>
+      <c r="G19" s="93"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="102" t="s">
+      <c r="B20" s="109" t="s">
         <v>251</v>
       </c>
-      <c r="C20" s="88"/>
-      <c r="D20" s="88"/>
-      <c r="E20" s="88"/>
-      <c r="F20" s="88"/>
-      <c r="G20" s="88"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C20" s="93"/>
+      <c r="D20" s="93"/>
+      <c r="E20" s="93"/>
+      <c r="F20" s="93"/>
+      <c r="G20" s="93"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="54" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="102" t="s">
+      <c r="B21" s="109" t="s">
         <v>252</v>
       </c>
-      <c r="C21" s="88"/>
-      <c r="D21" s="88"/>
-      <c r="E21" s="88"/>
-      <c r="F21" s="88"/>
-      <c r="G21" s="88"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="103" t="s">
+      <c r="C21" s="93"/>
+      <c r="D21" s="93"/>
+      <c r="E21" s="93"/>
+      <c r="F21" s="93"/>
+      <c r="G21" s="93"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="111" t="s">
         <v>253</v>
       </c>
-      <c r="B23" s="76"/>
-      <c r="C23" s="76"/>
-      <c r="D23" s="76"/>
-      <c r="E23" s="76"/>
-      <c r="F23" s="76"/>
-      <c r="G23" s="76"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B23" s="86"/>
+      <c r="C23" s="86"/>
+      <c r="D23" s="86"/>
+      <c r="E23" s="86"/>
+      <c r="F23" s="86"/>
+      <c r="G23" s="86"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="102" t="s">
+      <c r="B24" s="109" t="s">
         <v>293</v>
       </c>
-      <c r="C24" s="88"/>
-      <c r="D24" s="88"/>
-      <c r="E24" s="88"/>
-      <c r="F24" s="88"/>
-      <c r="G24" s="88"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C24" s="93"/>
+      <c r="D24" s="93"/>
+      <c r="E24" s="93"/>
+      <c r="F24" s="93"/>
+      <c r="G24" s="93"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="102" t="s">
+      <c r="B25" s="109" t="s">
         <v>294</v>
       </c>
-      <c r="C25" s="88"/>
-      <c r="D25" s="88"/>
-      <c r="E25" s="88"/>
-      <c r="F25" s="88"/>
-      <c r="G25" s="88"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C25" s="93"/>
+      <c r="D25" s="93"/>
+      <c r="E25" s="93"/>
+      <c r="F25" s="93"/>
+      <c r="G25" s="93"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="52" t="s">
         <v>89</v>
       </c>
-      <c r="B26" s="102" t="s">
+      <c r="B26" s="109" t="s">
         <v>295</v>
       </c>
-      <c r="C26" s="88"/>
-      <c r="D26" s="88"/>
-      <c r="E26" s="88"/>
-      <c r="F26" s="88"/>
-      <c r="G26" s="88"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="103" t="s">
+      <c r="C26" s="93"/>
+      <c r="D26" s="93"/>
+      <c r="E26" s="93"/>
+      <c r="F26" s="93"/>
+      <c r="G26" s="93"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="111" t="s">
         <v>254</v>
       </c>
-      <c r="B28" s="76"/>
-      <c r="C28" s="76"/>
-      <c r="D28" s="76"/>
-      <c r="E28" s="76"/>
-      <c r="F28" s="76"/>
-      <c r="G28" s="76"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B28" s="86"/>
+      <c r="C28" s="86"/>
+      <c r="D28" s="86"/>
+      <c r="E28" s="86"/>
+      <c r="F28" s="86"/>
+      <c r="G28" s="86"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="55" t="s">
         <v>255</v>
       </c>
-      <c r="B29" s="85" t="s">
+      <c r="B29" s="88" t="s">
         <v>256</v>
       </c>
-      <c r="C29" s="88"/>
-      <c r="D29" s="88"/>
-      <c r="E29" s="88"/>
-      <c r="F29" s="88"/>
-      <c r="G29" s="88"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C29" s="93"/>
+      <c r="D29" s="93"/>
+      <c r="E29" s="93"/>
+      <c r="F29" s="93"/>
+      <c r="G29" s="93"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="55" t="s">
         <v>257</v>
       </c>
-      <c r="B30" s="85" t="s">
+      <c r="B30" s="88" t="s">
         <v>258</v>
       </c>
-      <c r="C30" s="88"/>
-      <c r="D30" s="88"/>
-      <c r="E30" s="88"/>
-      <c r="F30" s="88"/>
-      <c r="G30" s="88"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C30" s="93"/>
+      <c r="D30" s="93"/>
+      <c r="E30" s="93"/>
+      <c r="F30" s="93"/>
+      <c r="G30" s="93"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="55" t="s">
         <v>259</v>
       </c>
-      <c r="B31" s="85" t="s">
+      <c r="B31" s="88" t="s">
         <v>260</v>
       </c>
-      <c r="C31" s="88"/>
-      <c r="D31" s="88"/>
-      <c r="E31" s="88"/>
-      <c r="F31" s="88"/>
-      <c r="G31" s="88"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C31" s="93"/>
+      <c r="D31" s="93"/>
+      <c r="E31" s="93"/>
+      <c r="F31" s="93"/>
+      <c r="G31" s="93"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="55" t="s">
         <v>261</v>
       </c>
-      <c r="B32" s="85" t="s">
+      <c r="B32" s="88" t="s">
         <v>262</v>
       </c>
-      <c r="C32" s="88"/>
-      <c r="D32" s="88"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="88"/>
-      <c r="G32" s="88"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C32" s="93"/>
+      <c r="D32" s="93"/>
+      <c r="E32" s="93"/>
+      <c r="F32" s="93"/>
+      <c r="G32" s="93"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="55" t="s">
         <v>263</v>
       </c>
-      <c r="B33" s="85" t="s">
+      <c r="B33" s="88" t="s">
         <v>264</v>
       </c>
-      <c r="C33" s="88"/>
-      <c r="D33" s="88"/>
-      <c r="E33" s="88"/>
-      <c r="F33" s="88"/>
-      <c r="G33" s="88"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C33" s="93"/>
+      <c r="D33" s="93"/>
+      <c r="E33" s="93"/>
+      <c r="F33" s="93"/>
+      <c r="G33" s="93"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="55" t="s">
         <v>265</v>
       </c>
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="88" t="s">
         <v>266</v>
       </c>
-      <c r="C34" s="88"/>
-      <c r="D34" s="88"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="88"/>
-      <c r="G34" s="88"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C34" s="93"/>
+      <c r="D34" s="93"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="93"/>
+      <c r="G34" s="93"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="55" t="s">
         <v>267</v>
       </c>
-      <c r="B35" s="85" t="s">
+      <c r="B35" s="88" t="s">
         <v>268</v>
       </c>
-      <c r="C35" s="88"/>
-      <c r="D35" s="88"/>
-      <c r="E35" s="88"/>
-      <c r="F35" s="88"/>
-      <c r="G35" s="88"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C35" s="93"/>
+      <c r="D35" s="93"/>
+      <c r="E35" s="93"/>
+      <c r="F35" s="93"/>
+      <c r="G35" s="93"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="55" t="s">
         <v>269</v>
       </c>
-      <c r="B36" s="85" t="s">
+      <c r="B36" s="88" t="s">
         <v>270</v>
       </c>
-      <c r="C36" s="88"/>
-      <c r="D36" s="88"/>
-      <c r="E36" s="88"/>
-      <c r="F36" s="88"/>
-      <c r="G36" s="88"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C36" s="93"/>
+      <c r="D36" s="93"/>
+      <c r="E36" s="93"/>
+      <c r="F36" s="93"/>
+      <c r="G36" s="93"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="55" t="s">
         <v>271</v>
       </c>
-      <c r="B37" s="85" t="s">
+      <c r="B37" s="88" t="s">
         <v>272</v>
       </c>
-      <c r="C37" s="88"/>
-      <c r="D37" s="88"/>
-      <c r="E37" s="88"/>
-      <c r="F37" s="88"/>
-      <c r="G37" s="88"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C37" s="93"/>
+      <c r="D37" s="93"/>
+      <c r="E37" s="93"/>
+      <c r="F37" s="93"/>
+      <c r="G37" s="93"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="55" t="s">
         <v>273</v>
       </c>
-      <c r="B38" s="85" t="s">
+      <c r="B38" s="88" t="s">
         <v>274</v>
       </c>
-      <c r="C38" s="88"/>
-      <c r="D38" s="88"/>
-      <c r="E38" s="88"/>
-      <c r="F38" s="88"/>
-      <c r="G38" s="88"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C38" s="93"/>
+      <c r="D38" s="93"/>
+      <c r="E38" s="93"/>
+      <c r="F38" s="93"/>
+      <c r="G38" s="93"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="55" t="s">
         <v>275</v>
       </c>
-      <c r="B39" s="85" t="s">
+      <c r="B39" s="88" t="s">
         <v>276</v>
       </c>
-      <c r="C39" s="88"/>
-      <c r="D39" s="88"/>
-      <c r="E39" s="88"/>
-      <c r="F39" s="88"/>
-      <c r="G39" s="88"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C39" s="93"/>
+      <c r="D39" s="93"/>
+      <c r="E39" s="93"/>
+      <c r="F39" s="93"/>
+      <c r="G39" s="93"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="55" t="s">
         <v>277</v>
       </c>
-      <c r="B40" s="85" t="s">
+      <c r="B40" s="88" t="s">
         <v>278</v>
       </c>
-      <c r="C40" s="88"/>
-      <c r="D40" s="88"/>
-      <c r="E40" s="88"/>
-      <c r="F40" s="88"/>
-      <c r="G40" s="88"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C40" s="93"/>
+      <c r="D40" s="93"/>
+      <c r="E40" s="93"/>
+      <c r="F40" s="93"/>
+      <c r="G40" s="93"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="55" t="s">
         <v>279</v>
       </c>
-      <c r="B41" s="85" t="s">
+      <c r="B41" s="88" t="s">
         <v>280</v>
       </c>
-      <c r="C41" s="88"/>
-      <c r="D41" s="88"/>
-      <c r="E41" s="88"/>
-      <c r="F41" s="88"/>
-      <c r="G41" s="88"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C41" s="93"/>
+      <c r="D41" s="93"/>
+      <c r="E41" s="93"/>
+      <c r="F41" s="93"/>
+      <c r="G41" s="93"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="55" t="s">
         <v>281</v>
       </c>
-      <c r="B42" s="85" t="s">
+      <c r="B42" s="88" t="s">
         <v>282</v>
       </c>
-      <c r="C42" s="88"/>
-      <c r="D42" s="88"/>
-      <c r="E42" s="88"/>
-      <c r="F42" s="88"/>
-      <c r="G42" s="88"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C42" s="93"/>
+      <c r="D42" s="93"/>
+      <c r="E42" s="93"/>
+      <c r="F42" s="93"/>
+      <c r="G42" s="93"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="55" t="s">
         <v>283</v>
       </c>
-      <c r="B43" s="85" t="s">
+      <c r="B43" s="88" t="s">
         <v>284</v>
       </c>
-      <c r="C43" s="88"/>
-      <c r="D43" s="88"/>
-      <c r="E43" s="88"/>
-      <c r="F43" s="88"/>
-      <c r="G43" s="88"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C43" s="93"/>
+      <c r="D43" s="93"/>
+      <c r="E43" s="93"/>
+      <c r="F43" s="93"/>
+      <c r="G43" s="93"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="55" t="s">
         <v>285</v>
       </c>
-      <c r="B44" s="85" t="s">
+      <c r="B44" s="88" t="s">
         <v>286</v>
       </c>
-      <c r="C44" s="88"/>
-      <c r="D44" s="88"/>
-      <c r="E44" s="88"/>
-      <c r="F44" s="88"/>
-      <c r="G44" s="88"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C44" s="93"/>
+      <c r="D44" s="93"/>
+      <c r="E44" s="93"/>
+      <c r="F44" s="93"/>
+      <c r="G44" s="93"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="55" t="s">
         <v>287</v>
       </c>
-      <c r="B45" s="85" t="s">
+      <c r="B45" s="88" t="s">
         <v>288</v>
       </c>
-      <c r="C45" s="88"/>
-      <c r="D45" s="88"/>
-      <c r="E45" s="88"/>
-      <c r="F45" s="88"/>
-      <c r="G45" s="88"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C45" s="93"/>
+      <c r="D45" s="93"/>
+      <c r="E45" s="93"/>
+      <c r="F45" s="93"/>
+      <c r="G45" s="93"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="55" t="s">
         <v>289</v>
       </c>
-      <c r="B46" s="85" t="s">
+      <c r="B46" s="88" t="s">
         <v>290</v>
       </c>
-      <c r="C46" s="88"/>
-      <c r="D46" s="88"/>
-      <c r="E46" s="88"/>
-      <c r="F46" s="88"/>
-      <c r="G46" s="88"/>
+      <c r="C46" s="93"/>
+      <c r="D46" s="93"/>
+      <c r="E46" s="93"/>
+      <c r="F46" s="93"/>
+      <c r="G46" s="93"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B43:G43"/>
+    <mergeCell ref="B44:G44"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B46:G46"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B33:G33"/>
+    <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B35:G35"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="B10:G10"/>
@@ -6406,28 +6435,12 @@
     <mergeCell ref="B19:G19"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B36:G36"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="B30:G30"/>
-    <mergeCell ref="B31:G31"/>
-    <mergeCell ref="B32:G32"/>
-    <mergeCell ref="B33:G33"/>
-    <mergeCell ref="B34:G34"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B43:G43"/>
-    <mergeCell ref="B44:G44"/>
-    <mergeCell ref="B45:G45"/>
-    <mergeCell ref="B46:G46"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="B39:G39"/>
-    <mergeCell ref="B40:G40"/>
-    <mergeCell ref="B41:G41"/>
-    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>